<commit_message>
Fixed error in direction and radius query
</commit_message>
<xml_diff>
--- a/Model_Testing/test_results_gpt-5.4-mini.xlsx
+++ b/Model_Testing/test_results_gpt-5.4-mini.xlsx
@@ -501,33 +501,33 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>The city of Münster is located in the federal state of Nordrhein-Westfalen.</t>
+          <t>The city of Münster refers to two different places. One Münster is a city in the district of Münster, in the administrative district of Münster, in the federal state of Nordrhein-Westfalen, in Germany. The other Münster is a city in the district of Rain, in the district of Donau-Ries, in the administrative district of Schwaben, in the federal state of Bayern, in Germany.</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>9.443</v>
+        <v>22.096</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>The ACTUAL answer correctly states that one Münster is in Nordrhein-Westfalen, but it omits the expected details about the specific district/administrative district for that Münster and the existence/location of the second Münster in Bayern.</t>
+          <t>The actual answer includes both Münster locations with the same administrative hierarchy as the expected answer, adding only the explicit mention of Germany, which is correct.</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>0.866</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>0.8438</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>0.855</v>
       </c>
     </row>
     <row r="3">
@@ -553,14 +553,14 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>The city of Cologne is located in Cologne, which is in Cologne, and in Nordrhein-Westfalen.</t>
+          <t>Nothing was found. No geometry found.</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.218</v>
+        <v>4.793</v>
       </c>
       <c r="G3" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -569,17 +569,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>The ACTUAL answer correctly identifies Nordrhein-Westfalen and indicates the city is in the Cologne/ Köln administrative area, but it is repetitive and does not clearly state 'administrative district Köln' as such.</t>
+          <t>The actual answer contains no information about Cologne’s location in Nordrhein-Westfalen or the administrative district Köln.</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.0223</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>-0.1243</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>-0.0526</v>
       </c>
     </row>
     <row r="4">
@@ -605,11 +605,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>The administrative community of Eisenhüttenstadt is located in the district of Oder-Spree, in the federal state of Brandenburg.</t>
+          <t>Eisenhüttenstadt is an administrative community in the district of Oder-Spree, in the federal state of Brandenburg, in Germany.</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>5.163</v>
+        <v>4.404</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
@@ -621,17 +621,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>The actual answer exactly matches the expected information about the district (Oder-Spree) and federal state (Brandenburg).</t>
+          <t>The actual answer includes the expected district (Oder-Spree) and federal state (Brandenburg); the added detail that it is in Germany does not contradict the expected content.</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.7947</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>0.8041</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.7997</v>
       </c>
     </row>
     <row r="5">
@@ -657,11 +657,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>The AdministrativeCommunity of Esens is located in the District of Wittmund, in the FederalState of Niedersachsen.</t>
+          <t>The administrative community of Esens is located in the district of Wittmund, in the federal state of Niedersachsen, in Germany.</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>4.566</v>
+        <v>4.962</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
@@ -673,17 +673,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>The actual answer states that Esens is in the District of Wittmund and the Federal State of Niedersachsen (Lower Saxony), matching all details in the expected answer.</t>
+          <t>The actual answer states Esens is in the Wittmund district and in the federal state of Niedersachsen (Lower Saxony), matching all details in the expected answer.</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.6778</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>0.8022</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.7388</v>
       </c>
     </row>
     <row r="6">
@@ -709,11 +709,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>The district of Gießen is located in the city of Gießen and in the federal state of Hessen.</t>
+          <t>The district of Gießen is located in Gießen, within the FederalState of Hessen, in Germany.</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>4.167</v>
+        <v>4.23</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
@@ -725,17 +725,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>The ACTUAL answer correctly states that the district of Gießen is located in the federal state of Hessen, matching the EXPECTED answer (with additional correct detail about the city of Gießen).</t>
+          <t>The actual answer states that the district of Gießen is in the Federal State of Hessen, which matches the expected information.</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>0.6244</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>0.7841</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>0.7020999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -761,11 +761,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>The district of Nordsachsen is located in the Federal State of Sachsen.</t>
+          <t>Nordsachsen is a District located in Sachsen, which is a FederalState, in Germany, which is a State.</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>4.509</v>
+        <v>14.058</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
@@ -777,17 +777,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>The actual answer states that Nordsachsen is located in the federal state of Sachsen, matching the expected answer (case differences only).</t>
+          <t>The actual answer states that Nordsachsen is located in Sachsen (the federal state), matching the expected information.</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>0.3251</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>0.5463</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>0.4309</v>
       </c>
     </row>
     <row r="8">
@@ -813,11 +813,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>The AdministrativeDistrict Freiburg is located in the FederalState Baden-Württemberg.</t>
+          <t>Freiburg is in Baden-Württemberg, which is in Germany.</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.345</v>
+        <v>22.579</v>
       </c>
       <c r="G8" t="n">
         <v>1</v>
@@ -829,17 +829,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>The actual answer states that the AdministrativeDistrict Freiburg is located in the FederalState Baden-Württemberg, matching the expected information.</t>
+          <t>The actual answer states that Freiburg is in Baden-Württemberg, which matches the expected location information. It additionally mentions Germany, which is not contradictory.</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>0.5149</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>0.4196</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>0.467</v>
       </c>
     </row>
     <row r="9">
@@ -865,33 +865,33 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>The administrative district of Oberfranken is located in the federal state of Bayern.</t>
+          <t>No geometry found for the administrative district of Oberfranken.</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>5.352</v>
+        <v>3.856</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>The actual answer matches the expected answer: Oberfranken is located in the federal state of Bayern.</t>
+          <t>The actual answer provides no information about the administrative district's location and does not state that Oberfranken is in Bayern.</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>0.4923</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>0.4752</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>0.4845</v>
       </c>
     </row>
     <row r="10">
@@ -917,33 +917,33 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sachsen is a Federal State located at POINT (13.348518008906732 51.05230081187263).</t>
+          <t>Sachsen is a FederalState in Germany.</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>6.392</v>
+        <v>8.632</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>The actual answer includes the correct location level (federal state) and matches the expected centroid coordinates exactly.</t>
+          <t>The actual answer does not provide the centroid location or the coordinates specified in the expected answer.</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>0.2389</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>-0.2359</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>-0.0298</v>
       </c>
     </row>
     <row r="11">
@@ -969,14 +969,14 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>The federal state of Saarland is located at the FederalState level.</t>
+          <t>Saarland is a FederalState located in Germany, which is the State.</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>4.475</v>
+        <v>4.023</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -985,17 +985,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>The actual answer only states the location at the 'FederalState level' but does not include the expected centroid coordinates (6.953360955673903, 49.38438040655551).</t>
+          <t>The actual answer only states that Saarland is a federal state in Germany but does not provide the expected centroid coordinates (6.953360955673903, 49.38438040655551).</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>0.3243</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>-0.1416</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>0.06279999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -1021,11 +1021,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>The district of Coesfeld includes the cities of Olfen, Ascheberg, Coesfeld, Lüdinghausen, Nordkirchen, Dülmen, Nottuln, Havixbeck, Billerbeck, Rosendahl, and Senden.</t>
+          <t>The district of Coesfeld includes the cities Rosendahl, Havixbeck, Senden, Billerbeck, Ascheberg, Dülmen, Nottuln, Coesfeld, Nordkirchen, Lüdinghausen, and Olfen. Coesfeld is a district in the administrative district of Münster, in the federal state of North Rhine-Westphalia, in Germany.</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>4.82</v>
+        <v>18.866</v>
       </c>
       <c r="G12" t="n">
         <v>1</v>
@@ -1037,17 +1037,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>All expected cities (Coesfeld, Olfen, Senden, Nottuln, Havixbeck, Nordkirchen, Billerbeck, Lüdinghausen, Rosendahl, Dülmen, Ascheberg) are included in the actual answer, matching exactly.</t>
+          <t>All expected cities (Coesfeld, Olfen, Senden, Nottuln, Havixbeck, Nordkirchen, Billerbeck, Lüdinghausen, Rosendahl, Dülmen, Ascheberg) are included in the actual answer; extra unrelated administrative details are correct and do not affect inclusion.</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>0.5353</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>0.7692</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>0.647</v>
       </c>
     </row>
     <row r="13">
@@ -1073,11 +1073,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>The administrative district of Oberbayern includes the districts of Neuburg-Schrobenhausen, Mühldorf a.Inn, Pfaffenhofen a.d.Ilm, Erding, Rosenheim, Miesbach, Ebersberg, Traunstein, Landsberg am Lech, München, Freising, Garmisch-Partenkirchen, Starnberg, Eichstätt, Ingolstadt, Fürstenfeldbruck, Dachau, Berchtesgadener Land, Altötting, Weilheim-Schongau, and Bad Tölz-Wolfratshausen. It also includes the districts of Rosenheim and München more than once in the data provided.</t>
+          <t>The administrative district of Oberbayern includes the districts Dachau, Miesbach, Garmisch-Partenkirchen, Landsberg am Lech, Rosenheim, Eichstätt, Ingolstadt, Fürstenfeldbruck, München, Berchtesgadener Land, Bad Tölz-Wolfratshausen, Ebersberg, Pfaffenhofen a.d.Ilm, Traunstein, Neuburg-Schrobenhausen, Mühldorf a.Inn, Starnberg, Altötting, Weilheim-Schongau, Freising, and Erding. Oberbayern is an administrative district in the FederalState of Bayern in Germany.</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>9.728999999999999</v>
+        <v>5.342</v>
       </c>
       <c r="G13" t="n">
         <v>1</v>
@@ -1089,17 +1089,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>All districts listed in the expected answer are present in the actual answer, including the note that Rosenheim and München appear more than once.</t>
+          <t>The ACTUAL answer lists all the districts named in the EXPECTED answer (including Fürstenfeldbruck, Erding, München, Freising, Ingolstadt, Mühldorf a.Inn, Rosenheim, Garmisch-Partenkirchen, Eichstätt, Landsberg am Lech, Weilheim-Schongau, Dachau, Altötting, Neuburg-Schrobenhausen, Pfaffenhofen a.d.Ilm, Ebersberg, Bad Tölz-Wolfratshausen, Traunstein, Miesbach, Starnberg, Berchtesgadener Land). It also contains the same district names; extra information about Bayern is correct and not conflicting.</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>0.5697</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>0.5463</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>0.5586</v>
       </c>
     </row>
     <row r="14">
@@ -1125,11 +1125,11 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>The Federal State Hessen includes the following Districts: Werra-Meißner-Kreis, Kassel, Fulda, Kassel, Schwalm-Eder-Kreis, Hersfeld-Rotenburg, Waldeck-Frankenberg, Limburg-Weilburg, Gießen, Vogelsbergkreis, Lahn-Dill-Kreis, Marburg-Biedenkopf, Main-Kinzig-Kreis, Groß-Gerau, Odenwaldkreis, Offenbach am Main, Rheingau-Taunus-Kreis, Offenbach, Bergstraße, Main-Taunus-Kreis, Frankfurt am Main, Wiesbaden, Hochtaunuskreis, Wetteraukreis, Darmstadt, and Darmstadt-Dieburg.</t>
+          <t>The federal state of Hessen includes the districts Limburg-Weilburg, Vogelsbergkreis, Lahn-Dill-Kreis, Marburg-Biedenkopf, Gießen, Hersfeld-Rotenburg, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis, Kassel, Schwalm-Eder-Kreis, Main-Kinzig-Kreis, Darmstadt, Wiesbaden, Rheingau-Taunus-Kreis, Bergstraße, Darmstadt-Dieburg, Frankfurt am Main, Offenbach, Main-Taunus-Kreis, Odenwaldkreis, Offenbach am Main, Hochtaunuskreis, Groß-Gerau, and Wetteraukreis. Hessen is a federal state in Germany, and Germany is the state.</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>4.81</v>
+        <v>4.685</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
@@ -1141,17 +1141,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>All districts listed in the expected answer appear in the actual answer (and no expected district is missing). Duplicate 'Kassel' in actual is harmless.</t>
+          <t>All districts listed in the expected answer are present in the actual answer (including Offenbach am Main, Groß-Gerau, Main-Taunus-Kreis, Wetteraukreis, Offenbach, Main-Kinzig-Kreis, Hochtaunuskreis, Odenwaldkreis, Darmstadt-Dieburg, Rheingau-Taunus-Kreis, Wiesbaden, Frankfurt am Main, Bergstraße, Darmstadt, Marburg-Biedenkopf, Gießen, Lahn-Dill-Kreis, Limburg-Weilburg, Vogelsbergkreis, Schwalm-Eder-Kreis, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis, and Hersfeld-Rotenburg).</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>0.6945</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>0.7262999999999999</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>0.7107</v>
       </c>
     </row>
     <row r="15">
@@ -1177,11 +1177,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>The district of Steinburg has the following administrative communities: Krempermarsch, Glückstadt, Horst-Herzhorn, Kellinghusen, Schenefeld, Wilster, Breitenburg, Wilstermarsch, Itzehoe-Land, and Itzehoe.</t>
+          <t>The district of Steinburg includes the following administrative communities: Itzehoe-Land, Schenefeld, Wilstermarsch, Itzehoe, Horst-Herzhorn, Krempermarsch, Breitenburg, Glückstadt, Wilster, and Kellinghusen. Steinburg is a district in the federal state of Schleswig-Holstein in Germany.</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>4.895</v>
+        <v>19.867</v>
       </c>
       <c r="G15" t="n">
         <v>1</v>
@@ -1193,17 +1193,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>The ACTUAL answer lists all administrative communities mentioned in the EXPECTED answer (Wilster, Krempermarsch, Itzehoe-Land, Horst-Herzhorn, Breitenburg, Schenefeld, Wilstermarsch, Glückstadt, Kellinghusen, and Itzehoe).</t>
+          <t>The ACTUAL answer lists all 10 administrative communities named in the EXPECTED answer: Wilster, Krempermarsch, Itzehoe-Land, Horst-Herzhorn, Breitenburg, Schenefeld, Wilstermarsch, Glückstadt, Kellinghusen, and Itzehoe. The ACTUAL includes an extra correct sentence about Steinburg being a district in Schleswig-Holstein.</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>0.6375999999999999</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>0.777</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>0.7058</v>
       </c>
     </row>
     <row r="16">
@@ -1229,11 +1229,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>The district of Paderborn includes 10 cities: Salzkotten, Hövelhof, Büren, Bad Wünnenberg, Paderborn, Delbrück, Lichtenau, Borchen, Altenbeken, and Bad Lippspringe.</t>
+          <t>Paderborn is a district in the administrative district of Detmold in the federal state of North Rhine-Westphalia in Germany. It has 10 cities: Altenbeken, Hövelhof, Borchen, Delbrück, Paderborn, Büren, Bad Wünnenberg, Lichtenau, Salzkotten, and Bad Lippspringe.</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4.564</v>
+        <v>6.977</v>
       </c>
       <c r="G16" t="n">
         <v>1</v>
@@ -1245,17 +1245,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>The ACTUAL answer lists the same 10 cities as the EXPECTED answer, matching names and count.</t>
+          <t>The actual answer lists exactly the same 10 cities as the expected answer (Paderborn, Bad Lippspringe, Borchen, Büren, Altenbeken, Hövelhof, Lichtenau, Bad Wünnenberg, Salzkotten, Delbrück), matching both the count and membership.</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>0.5279</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>0.7751</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>0.6456</v>
       </c>
     </row>
     <row r="17">
@@ -1281,11 +1281,11 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>No. Nothing no geometry found for the City of Dülmen within the District of Coesfeld.</t>
+          <t>No. No geometry was found for the city of Dülmen, so there is no provided information showing it within the district of Coesfeld.</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>4.61</v>
+        <v>5.02</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -1297,17 +1297,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>The actual answer states that Dülmen is not within the district of Coesfeld (or provides no supporting geometry), which contradicts the expected 'Yes'.</t>
+          <t>The actual answer states that there is no information/geometry to show Dülmen is within Coesfeld, which contradicts the expected yes.</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>0.3164</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>0.5364</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>0.4216</v>
       </c>
     </row>
     <row r="18">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Yes. Coesfeld is a District, and it is associated with Münster as an Administrative District.</t>
+          <t>Yes. Coesfeld is located in the AdministrativeDistrict of Münster, and the location hierarchy continues up to the FederalState and then to Germany as the State.</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>4.699</v>
+        <v>4.854</v>
       </c>
       <c r="G18" t="n">
         <v>1</v>
@@ -1349,17 +1349,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>The actual answer confirms that Coesfeld is associated with Münster as an administrative district, matching the expected statement.</t>
+          <t>The ACTUAL answer confirms that Coesfeld is located in the AdministrativeDistrict of Münster, which matches the expected statement.</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>0.3008</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>0.6104000000000001</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>0.4454</v>
       </c>
     </row>
     <row r="19">
@@ -1385,11 +1385,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Yes, Oberfranken is an AdministrativeDistrict and it belongs to the FederalState Bayern.</t>
+          <t>Yes. Oberfranken is an AdministrativeDistrict in the FederalState Bayern, and Bayern is in Germany.</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>4.598</v>
+        <v>4.488</v>
       </c>
       <c r="G19" t="n">
         <v>1</v>
@@ -1401,17 +1401,17 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>The actual answer states that Oberfranken (the administrative district) belongs to the federal state of Bayern, matching the expected answer.</t>
+          <t>The actual answer explicitly states that Oberfranken is an administrative district in the federal state of Bayern, matching the expected answer.</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>0.3456</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>0.5054</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>0.4234</v>
       </c>
     </row>
     <row r="20">
@@ -1437,11 +1437,11 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>No, nothing with geometry was found for the district of Steinfurt, so it cannot be confirmed from the provided information that it is located in the FederalState of Nordrhein-Westfalen.</t>
+          <t>No, nothing was found, so there is no geometry available to show that the district of Steinfurt is located in the federal state of Nordrhein-Westfalen.</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>4.267</v>
+        <v>4.195</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -1453,17 +1453,17 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>The actual answer states it cannot be confirmed and says 'No', which contradicts the expected claim that Steinfurt is in Nordrhein-Westfalen.</t>
+          <t>The actual answer explicitly denies/does not confirm that Steinfurt is located in Nordrhein-Westfalen.</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>0.5227000000000001</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>0.8366</v>
       </c>
       <c r="L20" t="n">
-        <v>0</v>
+        <v>0.6699000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -1489,11 +1489,11 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>No. Nothing no geometry found for Bocholt within the District of Cloppenburg.</t>
+          <t>No. No geometry found, so there is no information showing the city of Bocholt within the district of Cloppenburg.</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>4.672</v>
+        <v>4.06</v>
       </c>
       <c r="G21" t="n">
         <v>1</v>
@@ -1505,17 +1505,17 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Both expected and actual state that Bocholt is not located within the district of Cloppenburg.</t>
+          <t>Both the expected and actual answers state that Bocholt is not located within the district of Cloppenburg.</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>0.517</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>0.6833</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>0.5978</v>
       </c>
     </row>
     <row r="22">
@@ -1541,11 +1541,11 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Yes, Coesfeld, a District, touches Borken, a District.</t>
+          <t>Yes. Coesfeld touches Borken. Coesfeld is a district in Germany, and Borken is also a district in Germany.</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>4.807</v>
+        <v>4.509</v>
       </c>
       <c r="G22" t="n">
         <v>1</v>
@@ -1557,17 +1557,17 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>The actual answer states that the districts of Coesfeld and Borken touch each other, matching the expected answer.</t>
+          <t>The ACTUAL answer states that Coesfeld touches Borken, which directly matches the expected answer.</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>0.359</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>0.3544</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>0.3577</v>
       </c>
     </row>
     <row r="23">
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>5.078</v>
+        <v>4.431</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -1609,17 +1609,17 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>The actual answer does not address whether Senden and Münster are geographically disjoint and contains no relevant geographic information.</t>
+          <t>The actual answer does not address whether Senden and Münster are geographically disjoint and provides no relevant comparison.</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>-0.0587</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>0.0346</v>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>-0.0118</v>
       </c>
     </row>
     <row r="24">
@@ -1645,11 +1645,11 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Yes, Niedersachsen, a FederalState, touches Nordrhein-Westfalen, a FederalState.</t>
+          <t>Yes. Niedersachsen touches Nordrhein-Westfalen. Both are FederalStates, and the hierarchy ends with Germany as the State.</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>4.444</v>
+        <v>9.087999999999999</v>
       </c>
       <c r="G24" t="n">
         <v>1</v>
@@ -1661,17 +1661,17 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>The actual answer explicitly states that Niedersachsen touches Nordrhein-Westfalen, matching the expected answer.</t>
+          <t>The ACTUAL answer confirms that Niedersachsen touches Nordrhein-Westfalen, matching the EXPECTED answer. Additional notes about their classification are also correct.</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>0.3587</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>0.5385</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>0.4457</v>
       </c>
     </row>
     <row r="25">
@@ -1697,11 +1697,11 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>No, Berlin is not completely surrounded by Brandenburg. The information only shows Berlin as a City and two target Cities: Neuenhagen bei Berlin and Schöneiche bei Berlin.</t>
+          <t>No. Berlin is not completely surrounded by Brandenburg, because Berlin is associated with Schöneiche bei Berlin and Neuenhagen bei Berlin, both of which are cities in the Federal State of Brandenburg in Germany.</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>5.716</v>
+        <v>6.159</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -1713,17 +1713,17 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>The expected answer says Berlin is completely surrounded by Brandenburg, but the actual answer explicitly says it is not completely surrounded.</t>
+          <t>The expected answer is that Berlin is completely surrounded by Brandenburg, but the actual answer says it is not completely surrounded by Brandenburg.</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>0.1183</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>0.4937</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>0.2897</v>
       </c>
     </row>
     <row r="26">
@@ -1749,11 +1749,11 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Yes. Münster is north of Dortmund. Both are cities.</t>
+          <t>Yes. Münster is north of Dortmund. Both are cities in Germany.</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>6.515</v>
+        <v>5.818</v>
       </c>
       <c r="G26" t="n">
         <v>1</v>
@@ -1765,17 +1765,17 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>The ACTUAL answer confirms that Münster is north of Dortmund, matching the EXPECTED answer. Additional detail about both being cities is correct and does not contradict.</t>
+          <t>The actual answer states that Münster is north of Dortmund, matching the expected answer.</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>0.5278</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>0.7801</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>0.6478</v>
       </c>
     </row>
     <row r="27">
@@ -1801,11 +1801,11 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Greven is located directly north of Münster. It is a City.</t>
+          <t>Greven is located directly north of Münster. Greven is a city in Germany.</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>6.825</v>
+        <v>9.445</v>
       </c>
       <c r="G27" t="n">
         <v>1</v>
@@ -1817,17 +1817,17 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>The actual answer matches the expected answer exactly, stating that Greven is directly north of Münster.</t>
+          <t>The ACTUAL answer includes the same key information as the EXPECTED answer: that Greven is located directly north of Münster. Additional detail about Greven being a city in Germany does not contradict anything.</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>0.6457000000000001</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>0.7264</v>
       </c>
     </row>
     <row r="28">
@@ -1853,11 +1853,11 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Yes. Leipzig is located to the northeast of Erfurt. Both are cities.</t>
+          <t>Yes. Leipzig is located to the northeast of Erfurt.</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>5.972</v>
+        <v>5.839</v>
       </c>
       <c r="G28" t="n">
         <v>1</v>
@@ -1869,17 +1869,17 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>The actual answer states that Leipzig is located to the northeast of Erfurt, matching the expected response.</t>
+          <t>The ACTUAL answer explicitly states that Leipzig is located northeast of Erfurt, matching the EXPECTED answer.</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>0.7761</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>0.8472</v>
       </c>
       <c r="L28" t="n">
-        <v>0</v>
+        <v>0.8114</v>
       </c>
     </row>
     <row r="29">
@@ -1905,11 +1905,11 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>The distance between the City of Köln and the City of Bonn is 6.63 km.</t>
+          <t>Köln and Bonn are 6.63 km apart. Köln is a city in the administrative community, district, administrative district, federal state, and state hierarchy ending in Germany, and Bonn is a city in the administrative community, district, administrative district, federal state, and state hierarchy ending in Germany.</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>24.876</v>
+        <v>14.396</v>
       </c>
       <c r="G29" t="n">
         <v>1</v>
@@ -1921,17 +1921,17 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>The ACTUAL answer matches the EXPECTED distance (6.63 km) exactly, with only minor wording differences.</t>
+          <t>The actual answer states the distance between Köln and Bonn is 6.63 km, matching the expected value. Extra irrelevant location hierarchy details do not affect correctness.</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>0.042</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>0.3787</v>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>0.1969</v>
       </c>
     </row>
     <row r="30">
@@ -1957,33 +1957,33 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
+          <t>Hannover and Braunschweig are 0.0 km apart. Hannover is a city in the administrative community of Hannover, in the district Region Hannover, in the federal state of Niedersachsen, in Germany. Braunschweig is a city in the administrative community of Braunschweig, in the district Braunschweig, in the federal state of Niedersachsen, in Germany.</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>24.75</v>
+        <v>12.337</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
+          <t>Expected distance is 34.92 km, but the actual answer states Hannover and Braunschweig are 0.0 km apart.</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>0.1242</v>
       </c>
       <c r="K30" t="n">
-        <v>0</v>
+        <v>0.2878</v>
       </c>
       <c r="L30" t="n">
-        <v>0</v>
+        <v>0.2037</v>
       </c>
     </row>
     <row r="31">
@@ -2009,33 +2009,33 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
+          <t>Hessen and Thüringen are both FederalStates in Germany, the State. Based on their centroids, Hessen is at POINT (9.03095915220893 50.60325000970925) and Thüringen is at POINT (11.024691697649146 50.90384061550545). No distance between them is provided in the information.</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>24.58</v>
+        <v>10.893</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
+          <t>The expected answer states they are 0.0 km apart, but the actual answer provides centroid coordinates and does not give any distance value. Therefore it does not contain the expected information.</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
+        <v>-0.1934</v>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>0.3061</v>
       </c>
       <c r="L31" t="n">
-        <v>0</v>
+        <v>0.0227</v>
       </c>
     </row>
     <row r="32">
@@ -2061,11 +2061,11 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>The three closest Districts to the District of Miesbach are the District of Bad Tölz-Wolfratshausen, the District of Rosenheim, and the District of München.</t>
+          <t>The district of Miesbach is closest to the districts of München, Bad Tölz-Wolfratshausen, and Rosenheim. Miesbach is a District in the AdministrativeDistrict of Upper Bavaria in the FederalState of Bavaria in Germany. Each of the three closest districts is also a District in the AdministrativeDistrict of Upper Bavaria in the FederalState of Bavaria in Germany.</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>5.181</v>
+        <v>4.838</v>
       </c>
       <c r="G32" t="n">
         <v>1</v>
@@ -2077,17 +2077,17 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>The actual answer lists the same three closest districts as the expected answer (Bad Tölz-Wolfratshausen, Rosenheim, and München). Only wording/capitalization differs.</t>
+          <t>The ACTUAL answer lists the same three closest districts as the EXPECTED: München, Bad Tölz-Wolfratshausen, and Rosenheim (with additional irrelevant but correct details).</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>0.2139</v>
       </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>0.6635</v>
       </c>
       <c r="L32" t="n">
-        <v>0</v>
+        <v>0.4162</v>
       </c>
     </row>
     <row r="33">
@@ -2113,11 +2113,11 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>The district of Warendorf touches the districts of Gütersloh, Hamm, Münster, Steinfurt, Osnabrück, Coesfeld, and Soest. Warendorf is a District. All of the listed places are Districts as well.</t>
+          <t>The district of Warendorf touches the districts of Gütersloh, Steinfurt, Soest, Coesfeld, Osnabrück, Münster, and Hamm. Warendorf is a district in the AdministrativeDistrict of Münster in the FederalState of North Rhine-Westphalia in Germany.</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>4.441</v>
+        <v>4.425</v>
       </c>
       <c r="G33" t="n">
         <v>1</v>
@@ -2129,17 +2129,17 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>The ACTUAL answer lists the same eight neighboring districts as the EXPECTED answer: Gütersloh, Hamm, Münster, Steinfurt, Osnabrück, Coesfeld, and Soest.</t>
+          <t>The ACTUAL answer lists all the districts in the EXPECTED answer (Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld, Soest). The added administrative information is extra but correct.</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>0.4594</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>0.8108</v>
       </c>
       <c r="L33" t="n">
-        <v>0</v>
+        <v>0.6226</v>
       </c>
     </row>
     <row r="34">
@@ -2165,11 +2165,11 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>The administrative community Leezen is adjacent to the administrative communities Auenland Südholstein, Wahlstedt, Itzstedt, Buchholz (Forstgutsbez.), Kisdorf, Bad Oldesloe-Land, Trave-Land, Boostedt-Rickling, and Bad Segeberg. Leezen is an AdministrativeCommunity, and all of these are AdministrativeCommunities.</t>
+          <t>The administrative community Leezen is adjacent to Bad Oldesloe-Land, Trave-Land, Boostedt-Rickling, Auenland Südholstein, Wahlstedt, Kisdorf, Bad Segeberg, Itzstedt, and Buchholz (Forstgutsbez.). Leezen is an administrative community in the district of Segeberg, in the federal state of Schleswig-Holstein, in Germany.</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>4.954</v>
+        <v>4.422</v>
       </c>
       <c r="G34" t="n">
         <v>1</v>
@@ -2181,17 +2181,17 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>All nine adjacent administrative communities listed in the expected answer are present in the actual answer (Auenland Südholstein, Kisdorf, Bad Oldesloe-Land, Trave-Land, Wahlstedt, Itzstedt, Bad Segeberg, Boostedt-Rickling, Buchholz (Forstgutsbez.)).</t>
+          <t>The ACTUAL answer lists all nine adjacent administrative communities named in the EXPECTED answer: Auenland Südholstein, Kisdorf, Bad Oldesloe-Land, Trave-Land, Wahlstedt, Itzstedt, Bad Segeberg, Boostedt-Rickling, and Buchholz (Forstgutsbez.). Additional statement about location is extra but correct.</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>0.579</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>0.754</v>
       </c>
       <c r="L34" t="n">
-        <v>0</v>
+        <v>0.6637999999999999</v>
       </c>
     </row>
     <row r="35">
@@ -2217,33 +2217,33 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Mittelfranken (as an Administrative District/Regierungsbezirk) is surrounded by these Administrative Districts/Regierungsbezirke: Oberpfalz, Oberbayern, Unterfranken, Oberfranken, and Schwaben.</t>
+          <t>Mittelfranken is surrounded by the administrative districts of Oberpfalz, Oberbayern, Schwaben, Oberfranken, Unterfranken, and Stuttgart. Mittelfranken is an AdministrativeDistrict in Germany.</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>4.386</v>
+        <v>8.212</v>
       </c>
       <c r="G35" t="n">
-        <v>0.83</v>
+        <v>1</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>The actual answer includes five of the six expected surrounding districts (Oberpfalz, Oberbayern, Unterfranken, Oberfranken, Schwaben) but omits Stuttgart.</t>
+          <t>The ACTUAL answer lists all expected surrounding administrative districts: Oberpfalz, Unterfranken, Oberfranken, Oberbayern, Schwaben, and Stuttgart (order differs).</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
+        <v>0.6868</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>0.8639</v>
       </c>
       <c r="L35" t="n">
-        <v>0</v>
+        <v>0.7725</v>
       </c>
     </row>
     <row r="36">
@@ -2269,23 +2269,23 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Federal state: Thüringen is located among the states listed, and the federal states located north of Thüringen are Mecklenburg-Vorpommern, Sachsen-Anhalt, Schleswig-Holstein, and Hamburg.</t>
+          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>114.439</v>
+        <v>23.434</v>
       </c>
       <c r="G36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>The actual answer lists exactly the same four federal states north of Thüringen as the expected answer: Hamburg, Schleswig-Holstein, Mecklenburg-Vorpommern, and Sachsen-Anhalt.</t>
+          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="J36" t="n">
@@ -2321,12 +2321,11 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>The districts west of Münster are:
-Kleve (District / Kreis) and Borken (District / Kreis).</t>
+          <t>The districts west of Münster are Kleve and Borken. Münster is a district in the administrative district of Münster, in the federal state of North Rhine-Westphalia, in Germany. Kleve and Borken are districts in the administrative district of Münster, in the federal state of North Rhine-Westphalia, in Germany.</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>123.846</v>
+        <v>35.348</v>
       </c>
       <c r="G37" t="n">
         <v>1</v>
@@ -2338,17 +2337,17 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>The actual answer identifies Kleve and Borken as the districts west of Münster, matching the expected information.</t>
+          <t>The ACTUAL answer states that the districts west of Münster are Kleve and Borken, matching the EXPECTED information. Additional context is not incorrect.</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>0.07140000000000001</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>0.5495</v>
       </c>
       <c r="L37" t="n">
-        <v>0</v>
+        <v>0.2833</v>
       </c>
     </row>
     <row r="38">
@@ -2374,23 +2373,23 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>The administrative communities located north of the administrative community Kiel are Geltinger Bucht, Dänischenhagen, and Altenholz. There is also Kiel itself and Kappeln listed as well.</t>
+          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>82.021</v>
+        <v>24.255</v>
       </c>
       <c r="G38" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>The ACTUAL answer includes Altenholz, Dänischenhagen, and Geltinger Bucht, but it does not match the expected set because Kappeln is incorrectly included (it may not be north of Kiel per the expected answer).</t>
+          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="J38" t="n">
@@ -2426,23 +2425,23 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>The district of Göttingen is within a radius of 10 km from the following districts: Northeim, Kassel, Goslar, Nordhausen, Werra-Meißner-Kreis, Eichsfeld, Kassel, and Harz. All of these are Districts.</t>
+          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>74.773</v>
+        <v>23.819</v>
       </c>
       <c r="G39" t="n">
-        <v>0.95</v>
+        <v>0</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>The ACTUAL answer lists all districts from the EXPECTED set (Harz, Northeim, Goslar, Kassel, Eichsfeld, Werra-Meißner-Kreis, Nordhausen). It repeats Kassel, but duplicates do not omit any expected information.</t>
+          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="J39" t="n">
@@ -2478,23 +2477,23 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>The cities located within a radius of 5 km of Aachen are the City of Würselen, the City of Alsdorf, the City of Roetgen, the City of Herzogenrath, the City of Eschweiler, the City of Hürtgenwald, the City of Stolberg (Rhld.), and the City of Simmerath.</t>
+          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>76.48699999999999</v>
+        <v>23.143</v>
       </c>
       <c r="G40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>All expected cities (Alsdorf, Simmerath, Würselen, Hürtgenwald, Roetgen, Herzogenrath, Eschweiler, Stolberg (Rhld.)) are present in the actual answer. Only minor wording differences (e.g., 'City of' prefix) exist.</t>
+          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="J40" t="n">
@@ -2530,33 +2529,33 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>The cities located less than 2 km around the City of München are Krailling, Hebertshausen, Putzbrunn, Gräfelfing, Pullach i.Isartal, Bergkirchen, Ottobrunn, Haar, Gröbenzell, Vaterstetten, Karlsfeld, Planegg, Puchheim, Grünwalder Forst, Neubiberg, Oberschleißheim, Germering, Perlacher Forst, Dachau, Feldkirchen, Olching, Unterföhring, Unterhaching, Garching b.München, Ismaning, Neuried, Hohenbrunn, Forstenrieder Park, Aschheim, Grünwald, and Grasbrunn.</t>
+          <t>The cities located around Munich are Grasbrunn, Ismaning, Karlsfeld, Gräfelfing, Olching, Hebertshausen, Grünwalder Forst, Neuried, Neubiberg, Putzbrunn, Grünwald, Garching b.München, Perlacher Forst, Vaterstetten, Bergkirchen, Hohenbrunn, Unterföhring, Germering, Oberschleißheim, Krailling, Unterhaching, Gröbenzell, Planegg, Haar, Aschheim, Dachau, Feldkirchen, Pullach i.Isartal, Ottobrunn, Forstenrieder Park, and Puchheim. Munich is a city in the district, administrative district, federal state, and state hierarchy ending with Germany.</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>77.593</v>
+        <v>43.585</v>
       </c>
       <c r="G41" t="n">
-        <v>0.83</v>
+        <v>0.86</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>All expected cities appear in the actual answer except Feldkirchen? (actually included) and none missing except Forstenrieder Park included, Grünwald included, Feldkirchen included, Aschheim included, Haar included, Unterhaching included, Pullach i.Isartal included, Bergkirchen included, Neuried included, Germering included, Olching included, Garching b.München included, Planegg included, Ismaning included, Puchheim included, Unterföhring included, Gröbenzell included, Neubiberg included, Oberschleißheim included, Putzbrunn included, Perlacher Forst included, Gräfelfing included, Karlsfeld included. However expected includes 22 named places and actual includes them all; plus additional cities (Krailling, Hebertshausen, Ottobrunn, Vaterstetten, Grünwalder Forst, Dachau, Hohenbrunn, Grasbrunn).</t>
+          <t>Most expected cities are present in the actual answer, but several expected ones are missing (For example: Unterföhring is present but not missing; however missing include: Unterföhring is present; missing are Feldkirchen? present; actually present: Feldkirchen, Aschheim, Haar, Unterhaching, Pullach i.Isartal, Bergkirchen, Neuried, Germering, Olching, Garching b.München, Planegg, Ismaning, Puchheim, Unterföhring, Gröbenzell, Neubiberg, Oberschleißheim, Putzbrunn, Perlacher Forst, Gräfelfing, Karlsfeld, Forstenrieder Park, Grünwald, Grünwalder Forst. The actual is missing: Feldkirchen? it's present. The ones clearly missing from actual are: Ismaning, Gräfelfing, Karlsfeld are present; Actually Ismaning is present (listed as Ismaning). Gräfelfing present. Karlsfeld present. However the expected includes 'Perlacher Forst' and 'Perlacher Forst' is present. Expected includes 'Bergkirchen' present. Expected includes 'Germering' present. Expected includes 'Unterföhring' present. The main missing expected city is 'Haar' present, 'Neubiberg' present. The only notable expected city not in actual is 'Auberschleißheim' no it's Oberschleißheim present. Expected also includes 'Neubibiberg' spelled correctly. I conclude the missing are: 'Putzbrunn' present. 'Gräfelfing' present. So overall mismatch is smaller but actual includes additional cities; no expected cities seem missing except potentially 'Forstenrieder Park' present. Score slightly below 1 due to uncertainty from matching; actual doesn't include 'Feldkirchen' yes it does. Thus near-complete.</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>0.6126</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>0.7153</v>
       </c>
       <c r="L41" t="n">
-        <v>0</v>
+        <v>0.6634</v>
       </c>
     </row>
     <row r="42">
@@ -2582,11 +2581,13 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Es gibt zwei Orte namens Münster: eine Stadt in Nordrhein-Westfalen mit Verwaltungsgemeinde Münster, Kreis Münster, Regierungsbezirk und Bundesland Nordrhein-Westfalen, sowie eine Stadt in Bayern bei Rain, im Kreis Donau-Ries, im Regierungsbezirk Schwaben und im Bundesland Bayern.</t>
+          <t>Die Stadt Münster ist nicht eindeutig, denn es gibt zwei Orte mit diesem Namen:
+Münster liegt in der Verwaltungsgemeinde Münster, im Kreis Münster, im Regierungsbezirk Münster, im Bundesland Nordrhein-Westfalen, in Deutschland.
+Münster liegt in der Gemeinde Rain, im Kreis Donau-Ries, im Regierungsbezirk Schwaben, im Bundesland Bayern, in Deutschland.</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>7.134</v>
+        <v>5.849</v>
       </c>
       <c r="G42" t="n">
         <v>1</v>
@@ -2598,17 +2599,17 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort enthält beide in der Erwartung genannten Orte mit denselben jeweiligen Bundesländern, Regierungsbezirken und Kreisen/Gebieten; nur Formulierungen unterscheiden sich leicht.</t>
+          <t>Die tatsächliche Antwort enthält alle Informationen aus der erwarteten Antwort (beide Orte mit den jeweiligen Kreis-/Regierungsbezirks- und Bundeslandangaben) und ist inhaltlich korrekt.</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>0.6414</v>
       </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>0.6308</v>
       </c>
       <c r="L42" t="n">
-        <v>0</v>
+        <v>0.6367</v>
       </c>
     </row>
     <row r="43">
@@ -2634,11 +2635,11 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Die Stadt Köln liegt in der Stadt Köln und im Bundesland Nordrhein-Westfalen.</t>
+          <t>Köln liegt in Köln, im Kreis Köln, im Bundesland Nordrhein-Westfalen und im Bundesstaat Deutschland.</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>4.142</v>
+        <v>6.266</v>
       </c>
       <c r="G43" t="n">
         <v>0.5</v>
@@ -2650,17 +2651,17 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Der ACTUAL nennt korrekt das Bundesland Nordrhein-Westfalen, aber er erwähnt nicht den Regierungsbezirk Köln und enthält außerdem eine unzutreffende/unklare Angabe „in der Stadt Köln“.</t>
+          <t>Die Lage im Bundesland Nordrhein-Westfalen stimmt. Die Angabe zum Regierungsbezirk Köln fehlt jedoch; stattdessen nennt die Antwort zusätzliche (und teilweise falsche bzw. unpassende) Details wie „in Köln“ und „im Bundesstaat Deutschland“.</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>0.7084</v>
       </c>
       <c r="K43" t="n">
-        <v>0</v>
+        <v>0.7418</v>
       </c>
       <c r="L43" t="n">
-        <v>0</v>
+        <v>0.7254</v>
       </c>
     </row>
     <row r="44">
@@ -2686,11 +2687,11 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Die Verwaltungsgemeinde Eisenhüttenstadt liegt in der Stadt Eisenhüttenstadt im Kreis Oder-Spree im Bundesland Brandenburg.</t>
+          <t>Die Verwaltungsgemeinschaft Eisenhüttenstadt liegt in der Stadt Eisenhüttenstadt, im Kreis Oder-Spree, im Bundesland Brandenburg, in Deutschland.</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>4.892</v>
+        <v>10.08</v>
       </c>
       <c r="G44" t="n">
         <v>1</v>
@@ -2702,17 +2703,17 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Der tatsächliche Text nennt ebenfalls Landkreis Oder-Spree und Bundesland Brandenburg; die zusätzliche Angabe, dass sie in der Stadt Eisenhüttenstadt liegt, ergänzt nur und deckt sich mit der erwarteten Information.</t>
+          <t>Die tatsächliche Antwort nennt den Landkreis Oder-Spree und das Bundesland Brandenburg; zusätzlich präzisiert sie den Sitz in der Stadt Eisenhüttenstadt und fügt den Staat hinzu, was nicht im Widerspruch steht.</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>0.6378</v>
       </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>0.7674</v>
       </c>
       <c r="L44" t="n">
-        <v>0</v>
+        <v>0.7013</v>
       </c>
     </row>
     <row r="45">
@@ -2738,11 +2739,11 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Die Verwaltungsgemeinde Esens liegt in der Stadt Esens im Kreis Wittmund im Bundesland Niedersachsen.</t>
+          <t>Die Verwaltungsgemeinschaft Esens liegt in der Stadt Esens im Kreis Wittmund im Bundesland Niedersachsen in Deutschland.</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>4.311</v>
+        <v>4.389</v>
       </c>
       <c r="G45" t="n">
         <v>1</v>
@@ -2754,17 +2755,17 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Die Antwort nennt korrekt den Ort, dass Esens im Kreis/Landkreis Wittmund in Niedersachsen liegt. Die Zusatzangabe zur Stadt Esens ist ebenfalls korrekt.</t>
+          <t>Die tatsächliche Antwort nennt den Landkreis/Kreis Wittmund sowie Niedersachsen und damit alle Kernaussagen der erwarteten Antwort; zusätzliche Details (Stadt Esens, Deutschland) sind korrekt.</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>0.7292</v>
       </c>
       <c r="K45" t="n">
-        <v>0</v>
+        <v>0.8506</v>
       </c>
       <c r="L45" t="n">
-        <v>0</v>
+        <v>0.7887999999999999</v>
       </c>
     </row>
     <row r="46">
@@ -2790,14 +2791,14 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Der Kreis Gießen liegt in Gießen, Stadt, im Bundesland Hessen.</t>
+          <t>Der Kreis Gießen liegt in der Stadt Gießen im Bundesland Hessen in Deutschland.</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.603</v>
+        <v>4.049</v>
       </c>
       <c r="G46" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -2806,17 +2807,17 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Die erwartete Information ist enthalten: Der (Kreis/Landkreis) Gießen liegt im Bundesland Hessen. Die Antwort ergänzt nur weitere Details (in Gießen, Stadt).</t>
+          <t>Die Kernaussage stimmt: Der Kreis/Landkreis Gießen liegt im Bundesland Hessen. Die Antwort ergänzt korrekt die Lage in der Stadt Gießen und in Deutschland, ohne Widerspruch.</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>0</v>
+        <v>0.6906</v>
       </c>
       <c r="K46" t="n">
-        <v>0</v>
+        <v>0.8376</v>
       </c>
       <c r="L46" t="n">
-        <v>0</v>
+        <v>0.7623</v>
       </c>
     </row>
     <row r="47">
@@ -2842,11 +2843,11 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Der Kreis Nordsachsen liegt im Bundesland Sachsen.</t>
+          <t>Der Kreis Nordsachsen liegt im Bundesland Sachsen in Deutschland.</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>4.604</v>
+        <v>6.848</v>
       </c>
       <c r="G47" t="n">
         <v>1</v>
@@ -2858,17 +2859,17 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort enthält die erwartete Information: Der Landkreis/Kreis Nordsachsen liegt im Bundesland Sachsen.</t>
+          <t>Die tatsächliche Antwort nennt korrekt, dass der Kreis/Landkreis Nordsachsen im Bundesland Sachsen liegt; die zusätzliche Angabe „in Deutschland“ ist ebenfalls korrekt.</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
+        <v>0.866</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>0.9375</v>
       </c>
       <c r="L47" t="n">
-        <v>0</v>
+        <v>0.9014</v>
       </c>
     </row>
     <row r="48">
@@ -2894,11 +2895,11 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Der Regierungsbezirk Freiburg liegt im Bundesland Baden-Württemberg.</t>
+          <t>Der Regierungsbezirk Freiburg liegt im Bundesland Baden-Württemberg in Deutschland.</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>4.413</v>
+        <v>4.567</v>
       </c>
       <c r="G48" t="n">
         <v>1</v>
@@ -2910,17 +2911,17 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort enthält die gleiche Information wie die erwartete: Der Regierungs-/Verwaltungsbezirk Freiburg liegt im Bundesland Baden-Württemberg.</t>
+          <t>Die tatsächliche Antwort nennt korrekt, dass der Regierungsbezirk Freiburg im Bundesland Baden-Württemberg liegt. Zusätzliche Angabe: Deutschland ist ebenfalls korrekt.</t>
         </is>
       </c>
       <c r="J48" t="n">
-        <v>0</v>
+        <v>0.8056</v>
       </c>
       <c r="K48" t="n">
-        <v>0</v>
+        <v>0.8273</v>
       </c>
       <c r="L48" t="n">
-        <v>0</v>
+        <v>0.8167</v>
       </c>
     </row>
     <row r="49">
@@ -2946,11 +2947,11 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Der Regierungsbezirk Oberfranken liegt im Bundesland Bayern.</t>
+          <t>Der Regierungsbezirk Oberfranken liegt im Bundesland Bayern in Deutschland.</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>4.336</v>
+        <v>4.619</v>
       </c>
       <c r="G49" t="n">
         <v>1</v>
@@ -2962,17 +2963,17 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Der tatsächliche Antworttext nennt korrekt, dass Oberfranken im Bundesland Bayern liegt. Inhalt der erwarteten Aussage wird vollständig abgedeckt.</t>
+          <t>Der tatsächliche Text enthält die erwartete Information: Oberfranken liegt im Bundesland Bayern (zusätzlich wird erwähnt, dass es in Deutschland ist).</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>0</v>
+        <v>0.7915</v>
       </c>
       <c r="K49" t="n">
-        <v>0</v>
+        <v>0.8001</v>
       </c>
       <c r="L49" t="n">
-        <v>0</v>
+        <v>0.7961</v>
       </c>
     </row>
     <row r="50">
@@ -2998,14 +2999,14 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Das Bundesland Sachsen liegt in der Hierarchie auf der Ebene Bundesland. Es ist nicht weiter in Stadt, Verwaltungsgemeinde, Kreis oder Regierungsbezirk angegeben.</t>
+          <t>Sachsen liegt in Deutschland. Sachsen ist ein Bundesland und Deutschland ist ein Bundesstaat.</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>5.713</v>
+        <v>7.09</v>
       </c>
       <c r="G50" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -3014,17 +3015,17 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Der ACTUAL beschreibt die Ebene (Bundesland), nennt aber nicht den erwarteten Punkt mit den Koordinaten (13.348518008906732, 51.05230081187263).</t>
+          <t>Die Antwort enthält keine Lageangabe mit den erwarteten Koordinaten bzw. keine genaue Position auf Bundeslandebene.</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>0</v>
+        <v>0.3462</v>
       </c>
       <c r="K50" t="n">
-        <v>0</v>
+        <v>-0.2781</v>
       </c>
       <c r="L50" t="n">
-        <v>0</v>
+        <v>-0.0201</v>
       </c>
     </row>
     <row r="51">
@@ -3050,33 +3051,33 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Das Bundesland Saarland liegt auf der Ebene Bundesland. Sein Mittelpunkt liegt bei POINT (6.953360955673903 49.38438040655551).</t>
+          <t>Das Bundesland Saarland liegt in Deutschland.</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>4.35</v>
+        <v>5.269</v>
       </c>
       <c r="G51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Die tatsächlichen Koordinaten des Mittelpunkts stimmen mit den erwarteten Koordinaten überein (innerhalb der Toleranz) und die Lage auf Bundeslandebene wird ebenfalls korrekt beschrieben.</t>
+          <t>Die ACTUAL-Antwort enthält keine geografischen Koordinaten bzw. keinen Punkt wie im EXPECTED angegeben. Nur der Ort in Deutschland wird genannt.</t>
         </is>
       </c>
       <c r="J51" t="n">
-        <v>0</v>
+        <v>0.5564</v>
       </c>
       <c r="K51" t="n">
-        <v>0</v>
+        <v>-0.2312</v>
       </c>
       <c r="L51" t="n">
-        <v>0</v>
+        <v>0.0814</v>
       </c>
     </row>
     <row r="52">
@@ -3102,11 +3103,11 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Zum Kreis Coesfeld gehören die Städte Olfen, Ascheberg, Coesfeld, Lüdinghausen, Nordkirchen, Dülmen, Nottuln, Havixbeck, Billerbeck, Rosendahl und Senden. Der Kreis Coesfeld liegt im Regierungsbezirk und im Bundesland, die im Ergebnis jedoch nicht näher benannt sind.</t>
+          <t>Zum Kreis Coesfeld gehören die Städte Rosendahl, Havixbeck, Senden, Billerbeck, Ascheberg, Dülmen, Nottuln, Coesfeld, Nordkirchen, Lüdinghausen und Olfen. Der Kreis Coesfeld liegt im Regierungsbezirk Münster im Bundesland Nordrhein-Westfalen in Deutschland.</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>4.505</v>
+        <v>4.54</v>
       </c>
       <c r="G52" t="n">
         <v>1</v>
@@ -3118,17 +3119,17 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Die Liste der Städte im Kreis Coesfeld stimmt vollständig mit der erwarteten Antwort überein (alle 11 Städte enthalten). Zusätzliche allgemeine Informationen sind ebenfalls korrekt bzw. nicht widersprüchlich.</t>
+          <t>Die ACTUAL-Antwort nennt alle erwarteten Städte (Coesfeld, Olfen, Senden, Nottuln, Havixbeck, Nordkirchen, Billerbeck, Lüdinghausen, Rosendahl, Dülmen, Ascheberg). Zusatzinfo zur Lage ist korrekt und ändert nichts.</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>0</v>
+        <v>0.6214</v>
       </c>
       <c r="K52" t="n">
-        <v>0</v>
+        <v>0.7581</v>
       </c>
       <c r="L52" t="n">
-        <v>0</v>
+        <v>0.6883</v>
       </c>
     </row>
     <row r="53">
@@ -3154,33 +3155,33 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Im Regierungsbezirk Oberbayern liegen die Kreise Neuburg-Schrobenhausen, Mühldorf a.Inn, Pfaffenhofen a.d.Ilm, Erding, Rosenheim, Miesbach, Ebersberg, Traunstein, Landsberg am Lech, München, Freising, Garmisch-Partenkirchen, Starnberg, Eichstätt, Ingolstadt, Fürstenfeldbruck, Dachau, Berchtesgadener Land, Altötting, Weilheim-Schongau und Bad Tölz-Wolfratshausen sowie die Städte Ingolstadt und München.</t>
+          <t>Im Regierungsbezirk Oberbayern liegen die Kreise Dachau, Miesbach, Garmisch-Partenkirchen, Landsberg am Lech, Rosenheim, Eichstätt, Ingolstadt, Fürstenfeldbruck, München, Berchtesgadener Land, Bad Tölz-Wolfratshausen, Ebersberg, Pfaffenhofen a.d.Ilm, Traunstein, Neuburg-Schrobenhausen, Mühldorf a.Inn, Starnberg, Altötting, Weilheim-Schongau, Freising und Erding. Oberbayern liegt im Bundesland Bayern in Deutschland.</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>5.055</v>
+        <v>4.749</v>
       </c>
       <c r="G53" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Die Auflistung der Landkreise im Regierungsbezirk Oberbayern stimmt in den meisten Fällen mit der Erwartung überein; es fehlen jedoch die beiden Kreise "Rosenheim" und "München" als explizite Einträge (stattdessen werden die Städte Ingolstadt und München genannt). Der erwartete Hinweis auf mehr als einen Kreis mit dem Namen Rosenheim und München ist dadurch nicht enthalten. Inhaltlich sind die übrigen genannten Landkreise vorhanden.</t>
+          <t>Die tatsächliche Antwort nennt alle im Erwarteten aufgeführten Landkreise im Regierungsbezirk Oberbayern. Zusätzlich enthält sie eine allgemeine Zusatzinformation (Lage in Bayern/Deutschland).</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>0</v>
+        <v>0.598</v>
       </c>
       <c r="K53" t="n">
-        <v>0</v>
+        <v>0.5343</v>
       </c>
       <c r="L53" t="n">
-        <v>0</v>
+        <v>0.5664</v>
       </c>
     </row>
     <row r="54">
@@ -3206,33 +3207,33 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Zum Bundesland Hessen gehören folgende Kreise: Werra-Meißner-Kreis, Kassel, Fulda, Kassel, Schwalm-Eder-Kreis, Hersfeld-Rotenburg, Waldeck-Frankenberg, Limburg-Weilburg, Gießen, Vogelsbergkreis, Lahn-Dill-Kreis, Marburg-Biedenkopf, Main-Kinzig-Kreis, Groß-Gerau, Odenwaldkreis, Offenbach am Main, Rheingau-Taunus-Kreis, Offenbach, Bergstraße, Main-Taunus-Kreis, Frankfurt am Main, Wiesbaden, Hochtaunuskreis, Wetteraukreis, Darmstadt und Darmstadt-Dieburg. Es handelt sich um Kreise im Bundesland Hessen.</t>
+          <t>Zum Bundesland Hessen gehören die Kreise Limburg-Weilburg, Vogelsbergkreis, Lahn-Dill-Kreis, Marburg-Biedenkopf, Gießen, Hersfeld-Rotenburg, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis, Schwalm-Eder-Kreis, Main-Kinzig-Kreis, Rheingau-Taunus-Kreis, Bergstraße, Darmstadt-Dieburg, Main-Taunus-Kreis, Odenwaldkreis, Hochtaunuskreis, Groß-Gerau und Wetteraukreis sowie die Städte Darmstadt, Wiesbaden, Frankfurt am Main und Offenbach am Main und außerdem Offenbach und Kassel. Hessen liegt in Deutschland.</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>5.078</v>
+        <v>4.169</v>
       </c>
       <c r="G54" t="n">
-        <v>0.87</v>
+        <v>1</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Die ACTUAL-Antwort nennt 22 der 24 erwarteten Kreise (es fehlen: Odenwaldkreis? ist vorhanden; tatsächlich fehlen Offenbach am Main? ist vorhanden; fehlen dagegen: Rheingau-Taunus-Kreis ist vorhanden; die fehlenden sind Frankfurt am Main? ist vorhanden). Es fehlen jedoch im Vergleich die Kreise Waldeck? ist vorhanden. Insgesamt fehlen: Werra-Meißner-Kreis? ist vorhanden. Die fehlenden erwarteten Einträge sind: keiner klar zusätzlich, aber die erwartete Liste enthält 24 und die tatsächliche wirkt wie 23 ohne 'Hochtaunuskreis'? ist vorhanden. Zusätzlich fehlt in ACTUAL: 'Hochtaunuskreis' ist vorhanden, also nicht. Plausibel fehlend: 'Offenbach am Main'? vorhanden. Die einzige eindeutige Unstimmigkeit ist ein fehlender Eintrag: 'Werra-Meißner-Kreis' ist vorhanden. Daher Hauptabzug wegen unvollständiger Abdeckung gegenüber der erwarteten Liste (2 fehlen).</t>
+          <t>Alle im EXPECTED genannten Landkreise sind im ACTUAL enthalten; ACTUAL ergänzt zusätzlich Hinweise (z.B. dass Hessen in Deutschland liegt) und nennt die kreisfreien Städte ebenfalls, ohne etwas Falsches wegzulassen.</t>
         </is>
       </c>
       <c r="J54" t="n">
-        <v>0</v>
+        <v>0.6746</v>
       </c>
       <c r="K54" t="n">
-        <v>0</v>
+        <v>0.71</v>
       </c>
       <c r="L54" t="n">
-        <v>0</v>
+        <v>0.6926</v>
       </c>
     </row>
     <row r="55">
@@ -3258,11 +3259,11 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Zum Kreis Steinburg gehören die Verwaltungsgemeinden Krempermarsch, Glückstadt, Horst-Herzhorn, Kellinghusen, Schenefeld, Wilster, Breitenburg, Wilstermarsch, Itzehoe-Land und Itzehoe. Der Kreis Steinburg liegt im Regierungsbezirk und im Bundesland, diese höheren Ebenen sind im Ergebnis jedoch nicht weiter benannt.</t>
+          <t>Zum Kreis Steinburg gehören die Verwaltungsgemeinden Itzehoe-Land, Schenefeld, Wilstermarsch, Itzehoe, Horst-Herzhorn, Krempermarsch, Breitenburg, Glückstadt, Wilster und Kellinghusen. Der Kreis Steinburg liegt im Bundesland Schleswig-Holstein in Deutschland.</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>4.858</v>
+        <v>4.208</v>
       </c>
       <c r="G55" t="n">
         <v>1</v>
@@ -3274,17 +3275,17 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Alle in der Erwartung genannten Verwaltungsgemeinden (Wilster, Krempermarsch, Itzehoe-Land, Horst-Herzhorn, Breitenburg, Schenefeld, Wilstermarsch, Glückstadt, Kellinghusen, Itzehoe) sind im tatsächlichen Text enthalten; zusätzliche allgemeine Angaben ändern daran nichts.</t>
+          <t>Die ACTUAL-Antwort nennt alle zehn erwarteten Verwaltungsgemeinden des Kreises Steinburg; zusätzlich wird noch der Bundeslandhinweis gegeben, der korrekt ist.</t>
         </is>
       </c>
       <c r="J55" t="n">
-        <v>0</v>
+        <v>0.6793</v>
       </c>
       <c r="K55" t="n">
-        <v>0</v>
+        <v>0.7786</v>
       </c>
       <c r="L55" t="n">
-        <v>0</v>
+        <v>0.7284</v>
       </c>
     </row>
     <row r="56">
@@ -3310,33 +3311,33 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Zum Kreis Paderborn gehören 10 Städte: Salzkotten, Hövelhof, Büren, Bad Wünnenberg, Paderborn, Delbrück, Lichtenau, Borchen, Altenbeken und Bad Lippspringe. Der Kreis Paderborn ist dem Regierungsbezirk und dem Bundesland zugeordnet.</t>
+          <t>Es wurden keine Geometrien gefunden. Daher lässt sich aus den vorliegenden Informationen nicht sagen, wie viele Städte zum Kreis Paderborn gehören.</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>4.598</v>
+        <v>5.009</v>
       </c>
       <c r="G56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Die ACTUAL-Antwort nennt dieselben 10 Städte wie die EXPECTED-Antwort; zusätzliche, sachlich korrekte Zusatzinformation ist enthalten.</t>
+          <t>Die Antwort enthält keine Information darüber, wie viele Städte zum Kreis Paderborn gehören oder welche Städte dies sind.</t>
         </is>
       </c>
       <c r="J56" t="n">
-        <v>0</v>
+        <v>0.0191</v>
       </c>
       <c r="K56" t="n">
-        <v>0</v>
+        <v>-0.1612</v>
       </c>
       <c r="L56" t="n">
-        <v>0</v>
+        <v>-0.07439999999999999</v>
       </c>
     </row>
     <row r="57">
@@ -3362,11 +3363,11 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Nein, zu Dülmen liegen keine Informationen vor; es wurde keine Geometrie gefunden.</t>
+          <t>Nein, es wurde keine Geometrie gefunden.</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>5.384</v>
+        <v>4.163</v>
       </c>
       <c r="G57" t="n">
         <v>0</v>
@@ -3378,17 +3379,17 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Die erwartete Aussage „Ja, Dülmen liegt im Kreis Coesfeld“ wird in der tatsächlichen Antwort nicht bestätigt; stattdessen wird verneint bzw. keine Information gefunden.</t>
+          <t>Die ACTUAL-Antwort bestätigt nicht, dass Dülmen im Kreis Coesfeld liegt; sie sagt stattdessen, dass keine Geometrie gefunden wurde.</t>
         </is>
       </c>
       <c r="J57" t="n">
-        <v>0</v>
+        <v>0.09569999999999999</v>
       </c>
       <c r="K57" t="n">
-        <v>0</v>
+        <v>0.0251</v>
       </c>
       <c r="L57" t="n">
-        <v>0</v>
+        <v>0.0611</v>
       </c>
     </row>
     <row r="58">
@@ -3414,33 +3415,33 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Nein. Für den Kreis Coesfeld wurde keine Geometrie gefunden.</t>
+          <t>Ja, der Kreis Coesfeld liegt im Regierungsbezirk Münster, im Bundesland Nordrhein-Westfalen in Deutschland.</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>4.354</v>
+        <v>4.404</v>
       </c>
       <c r="G58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort sagt, dass keine Geometrie gefunden wurde und verneint implizit die Frage. Die erwartete Aussage „Ja, der Kreis Coesfeld liegt im Regierungsbezirk Münster“ wird nicht bestätigt.</t>
+          <t>Die tatsächliche Antwort bestätigt ebenfalls, dass der Kreis Coesfeld im Regierungsbezirk Münster liegt; Zusatzinformationen sind korrekt und schmälern die Übereinstimmung nicht.</t>
         </is>
       </c>
       <c r="J58" t="n">
-        <v>0</v>
+        <v>0.5699</v>
       </c>
       <c r="K58" t="n">
-        <v>0</v>
+        <v>0.8419</v>
       </c>
       <c r="L58" t="n">
-        <v>0</v>
+        <v>0.6988</v>
       </c>
     </row>
     <row r="59">
@@ -3466,11 +3467,11 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Ja, der Regierungsbezirk Oberfranken gehört zum Bundesland Bayern.</t>
+          <t>Ja, Oberfranken gehört zum Bundesland Bayern in Deutschland.</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>4.368</v>
+        <v>3.604</v>
       </c>
       <c r="G59" t="n">
         <v>1</v>
@@ -3482,17 +3483,17 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort stimmt mit der erwarteten Aussage überein.</t>
+          <t>Die Antwort bestätigt korrekt, dass der Regierungsbezirk Oberfranken zu Bayern gehört.</t>
         </is>
       </c>
       <c r="J59" t="n">
-        <v>0</v>
+        <v>0.6207</v>
       </c>
       <c r="K59" t="n">
-        <v>0</v>
+        <v>0.5692</v>
       </c>
       <c r="L59" t="n">
-        <v>0</v>
+        <v>0.5952</v>
       </c>
     </row>
     <row r="60">
@@ -3522,7 +3523,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>4.534</v>
+        <v>3.74</v>
       </c>
       <c r="G60" t="n">
         <v>0</v>
@@ -3534,17 +3535,17 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort verneint die Frage bzw. enthält keine Information darüber, dass der Kreis Steinfurt in Nordrhein-Westfalen liegt.</t>
+          <t>Die tatsächliche Antwort enthält keine Aussage dazu, ob der Kreis Steinfurt in Nordrhein-Westfalen liegt, sondern behauptet nur, dass keine Geometrie gefunden wurde.</t>
         </is>
       </c>
       <c r="J60" t="n">
-        <v>0</v>
+        <v>0.0958</v>
       </c>
       <c r="K60" t="n">
-        <v>0</v>
+        <v>-0.059</v>
       </c>
       <c r="L60" t="n">
-        <v>0</v>
+        <v>0.0165</v>
       </c>
     </row>
     <row r="61">
@@ -3574,7 +3575,7 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>4.222</v>
+        <v>6.76</v>
       </c>
       <c r="G61" t="n">
         <v>0</v>
@@ -3586,17 +3587,17 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort enthält keine Aussage darüber, ob Bocholt im Kreis Cloppenburg liegt; sie nennt nur, dass keine Geometrie gefunden wurde.</t>
+          <t>Die ACTUAL-Antwort liefert keine Aussage dazu, ob Bocholt im Kreis Cloppenburg liegt, sondern erwähnt nur fehlende Geometrie.</t>
         </is>
       </c>
       <c r="J61" t="n">
-        <v>0</v>
+        <v>0.2787</v>
       </c>
       <c r="K61" t="n">
-        <v>0</v>
+        <v>0.1121</v>
       </c>
       <c r="L61" t="n">
-        <v>0</v>
+        <v>0.193</v>
       </c>
     </row>
     <row r="62">
@@ -3622,11 +3623,11 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Ja, der Kreis Coesfeld grenzt an den Kreis Borken.</t>
+          <t>Ja, der Kreis Coesfeld grenzt an den Kreis Borken. Beide liegen im Bundesland Nordrhein-Westfalen in Deutschland.</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>5.135</v>
+        <v>5.027</v>
       </c>
       <c r="G62" t="n">
         <v>1</v>
@@ -3638,17 +3639,17 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort bestätigt ebenfalls, dass der Kreis Coesfeld an den Kreis Borken grenzt, was der erwarteten Aussage entspricht.</t>
+          <t>Der tatsächliche Antworttext bestätigt, dass der Kreis Coesfeld an den Kreis Borken angrenzt. Zusatzinformationen sind korrekt und beeinträchtigen nicht.</t>
         </is>
       </c>
       <c r="J62" t="n">
-        <v>0</v>
+        <v>0.3801</v>
       </c>
       <c r="K62" t="n">
-        <v>0</v>
+        <v>0.5206</v>
       </c>
       <c r="L62" t="n">
-        <v>0</v>
+        <v>0.4489</v>
       </c>
     </row>
     <row r="63">
@@ -3674,11 +3675,11 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Hallo. Dieser Chatbot beantwortet nur Fragen zu den Geografien Deutschlands. Bitte versuche es mit einer anderen Frage.</t>
+          <t>Die Städte Senden und Münster sind geografisch voneinander getrennt, liegen aber beide in Nordrhein-Westfalen und relativ nah beieinander. Münster ist eine eigenständige Stadt, Senden eine Gemeinde im Kreis Coesfeld südlich davon.</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>4.226</v>
+        <v>10.682</v>
       </c>
       <c r="G63" t="n">
         <v>0</v>
@@ -3690,17 +3691,17 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort enthält keine Aussage dazu, ob Senden und Münster geografisch getrennt sind.</t>
+          <t>Die erwartete Antwort sagt, dass Senden und Münster nebeneinander liegen und nicht getrennt sind. Die tatsächliche Antwort widerspricht und behauptet, die Städte seien geografisch voneinander getrennt.</t>
         </is>
       </c>
       <c r="J63" t="n">
-        <v>0</v>
+        <v>0.028</v>
       </c>
       <c r="K63" t="n">
-        <v>0</v>
+        <v>0.2776</v>
       </c>
       <c r="L63" t="n">
-        <v>0</v>
+        <v>0.1458</v>
       </c>
     </row>
     <row r="64">
@@ -3726,11 +3727,11 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Ja, Niedersachsen als Bundesland grenzt an Nordrhein-Westfalen als Bundesland.</t>
+          <t>Ja, Niedersachsen grenzt an Nordrhein-Westfalen. Beide sind Bundesländer in Deutschland, also im Bundesstaat Deutschland.</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>5.548</v>
+        <v>4.348</v>
       </c>
       <c r="G64" t="n">
         <v>1</v>
@@ -3742,17 +3743,17 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort bestätigt eindeutig, dass Niedersachsen an Nordrhein-Westfalen grenzt; Inhalt entspricht der erwarteten Aussage.</t>
+          <t>Der tatsächliche Antwortsatz bestätigt korrekt, dass Niedersachsen an Nordrhein-Westfalen grenzt. Zusätzliche Informationen (Bundesländer in Deutschland) sind zutreffend und ändern nichts am Kerninhalt.</t>
         </is>
       </c>
       <c r="J64" t="n">
-        <v>0</v>
+        <v>0.4103</v>
       </c>
       <c r="K64" t="n">
-        <v>0</v>
+        <v>0.601</v>
       </c>
       <c r="L64" t="n">
-        <v>0</v>
+        <v>0.5023</v>
       </c>
     </row>
     <row r="65">
@@ -3778,11 +3779,11 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Ja. Berlin ist laut den vorliegenden Angaben mit Neuenhagen bei Berlin und Schöneiche bei Berlin verbunden, beides Städte. Damit ist Berlin in diesem Ergebnis nicht vollständig von Brandenburg umgeben.</t>
+          <t>Nein, Berlin ist nicht vollständig von Brandenburg umgeben. In den vorliegenden Angaben wird Berlin mit Schöneiche bei Berlin und Neuenhagen bei Berlin in Verbindung gebracht. Berlin liegt als Stadt in Deutschland, und Deutschland ist ein Bundesstaat.</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>6.997</v>
+        <v>5.534</v>
       </c>
       <c r="G65" t="n">
         <v>0</v>
@@ -3794,17 +3795,17 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort widerspricht der erwarteten Aussage. Sie behauptet, Berlin sei nicht vollständig von Brandenburg umgeben, weil es mit Neuenhagen bei Berlin und Schöneiche bei Berlin verbunden sei.</t>
+          <t>Die erwartete Antwort lautet „Ja“, die tatsächliche Antwort lautet jedoch „Nein“ und bestätigt damit nicht, dass Berlin vollständig von Brandenburg umgeben ist.</t>
         </is>
       </c>
       <c r="J65" t="n">
-        <v>0</v>
+        <v>0.1192</v>
       </c>
       <c r="K65" t="n">
-        <v>0</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="L65" t="n">
-        <v>0</v>
+        <v>0.3167</v>
       </c>
     </row>
     <row r="66">
@@ -3830,11 +3831,11 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Ja, Münster liegt nördlich von Dortmund. Beide Orte sind Städte.</t>
+          <t>Ja, Münster liegt nördlich von Dortmund. Münster ist eine Stadt im Kreis, im Regierungsbezirk, im Bundesland Nordrhein-Westfalen und im Bundesstaat Deutschland; Dortmund ist ebenfalls eine Stadt im Kreis, im Regierungsbezirk, im Bundesland Nordrhein-Westfalen und im Bundesstaat Deutschland.</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>6.282</v>
+        <v>6.453</v>
       </c>
       <c r="G66" t="n">
         <v>1</v>
@@ -3846,17 +3847,17 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Die Aussage stimmt: Münster liegt nördlich von Dortmund. Die zusätzliche Information, dass beide Orte Städte sind, ist korrekt.</t>
+          <t>Die ACTUAL-Antwort bestätigt ebenfalls, dass Münster nördlich von Dortmund liegt. Zusätzliche korrekte Kontextinformationen werden genannt.</t>
         </is>
       </c>
       <c r="J66" t="n">
-        <v>0</v>
+        <v>0.0861</v>
       </c>
       <c r="K66" t="n">
-        <v>0</v>
+        <v>0.7317</v>
       </c>
       <c r="L66" t="n">
-        <v>0</v>
+        <v>0.3609</v>
       </c>
     </row>
     <row r="67">
@@ -3882,11 +3883,11 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Direkt nördlich von Münster liegt die Stadt Greven.</t>
+          <t>Greven liegt direkt nördlich von Münster. Beide Städte liegen in Deutschland.</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>5.929</v>
+        <v>8.23</v>
       </c>
       <c r="G67" t="n">
         <v>1</v>
@@ -3898,17 +3899,17 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort nennt korrekt Greven als Stadt direkt nördlich von Münster.</t>
+          <t>Die tatsächliche Antwort enthält genau die erwartete Information: Greven liegt direkt nördlich von Münster. Die Zusatzangabe „beide Städte liegen in Deutschland“ ist korrekt und schadet nicht.</t>
         </is>
       </c>
       <c r="J67" t="n">
-        <v>0</v>
+        <v>0.5765</v>
       </c>
       <c r="K67" t="n">
-        <v>0</v>
+        <v>0.8496</v>
       </c>
       <c r="L67" t="n">
-        <v>0</v>
+        <v>0.7058</v>
       </c>
     </row>
     <row r="68">
@@ -3934,11 +3935,11 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Ja, Leipzig liegt nordöstlich von Erfurt. Erfurt ist die Stadt, und Leipzig ist die Stadt.</t>
+          <t>Ja, Leipzig liegt nordöstlich von Erfurt. Beide Städte liegen in Deutschland.</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>6.125</v>
+        <v>8.16</v>
       </c>
       <c r="G68" t="n">
         <v>1</v>
@@ -3950,17 +3951,17 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort bestätigt dass Leipzig nordöstlich von Erfurt liegt. Die zusätzliche Erläuterung ändert nichts am Inhalt.</t>
+          <t>Die tatsächliche Antwort stimmt mit der erwarteten überein: Leipzig liegt nordöstlich von Erfurt (und damit auch östlich). Zusätzliche Information über Deutschland ist korrekt und nicht widersprüchlich.</t>
         </is>
       </c>
       <c r="J68" t="n">
-        <v>0</v>
+        <v>0.5687</v>
       </c>
       <c r="K68" t="n">
-        <v>0</v>
+        <v>0.8310999999999999</v>
       </c>
       <c r="L68" t="n">
-        <v>0</v>
+        <v>0.6932</v>
       </c>
     </row>
     <row r="69">
@@ -3986,11 +3987,11 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Die Entfernung zwischen der Stadt Köln und der Stadt Bonn beträgt 6,63 km.</t>
+          <t>Köln ist eine Stadt in Nordrhein-Westfalen in Deutschland. Bonn ist eine Stadt in Nordrhein-Westfalen in Deutschland. Die Entfernung zwischen Köln und Bonn beträgt 6,63 km.</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>20.672</v>
+        <v>16.558</v>
       </c>
       <c r="G69" t="n">
         <v>1</v>
@@ -4002,17 +4003,17 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort stimmt mit der erwarteten Entfernung (6,63 km) überein.</t>
+          <t>Die tatsächliche Antwort nennt ebenfalls die Entfernung zwischen Köln und Bonn als 6,63 km (übereinstimmend mit der erwarteten Angabe).</t>
         </is>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
+        <v>0.3742</v>
       </c>
       <c r="K69" t="n">
-        <v>0</v>
+        <v>0.6902</v>
       </c>
       <c r="L69" t="n">
-        <v>0</v>
+        <v>0.5218</v>
       </c>
     </row>
     <row r="70">
@@ -4038,33 +4039,33 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
+          <t>Hannover liegt in der Stadt Hannover, in der Verwaltungsgemeinde Hannover, im Kreis Region Hannover, im Bundesland Niedersachsen und im Bundesstaat Deutschland. Braunschweig liegt in der Stadt Braunschweig, in der Kreis Braunschweig, im Bundesland Niedersachsen und im Bundesstaat Deutschland. Die Entfernung zwischen Hannover und Braunschweig beträgt 0,0 km.</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>25.407</v>
+        <v>10.891</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
+          <t>Die erwartete Entfernung beträgt 34,92 km, im tatsächlichen Antworttext wird jedoch 0,0 km angegeben.</t>
         </is>
       </c>
       <c r="J70" t="n">
-        <v>0</v>
+        <v>0.1092</v>
       </c>
       <c r="K70" t="n">
-        <v>0</v>
+        <v>0.5834</v>
       </c>
       <c r="L70" t="n">
-        <v>0</v>
+        <v>0.3201</v>
       </c>
     </row>
     <row r="71">
@@ -4090,14 +4091,14 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Die Entfernung beträgt 171,35 km zwischen Münster in Hessen, einer Stadt im Bundesland Hessen, und Mühlhausen in Thüringen, einer Stadt im Bundesland Thüringen.</t>
+          <t>Hessen und Thüringen sind beide Bundesländer in Deutschland. Hessen liegt in Deutschland und Thüringen liegt ebenfalls in Deutschland. Für Hessen ist eine Entfernung von 0,0 km angegeben. Eine direkte Entfernung zwischen Hessen und Thüringen wird in den bereitgestellten Angaben nicht genannt.</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>22.53</v>
+        <v>11.084</v>
       </c>
       <c r="G71" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -4106,17 +4107,17 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Die erwartete Antwort sagt 0,0 km Abstand, die tatsächliche Antwort nennt 171,35 km. Das widerspricht der erwarteten Angabe.</t>
+          <t>Der ACTUAL-Text nennt keine konkrete Entfernung zwischen Hessen und Thüringen und widerspricht damit der erwarteten Angabe (0,0 km).</t>
         </is>
       </c>
       <c r="J71" t="n">
-        <v>0</v>
+        <v>0.167</v>
       </c>
       <c r="K71" t="n">
-        <v>0</v>
+        <v>0.3646</v>
       </c>
       <c r="L71" t="n">
-        <v>0</v>
+        <v>0.262</v>
       </c>
     </row>
     <row r="72">
@@ -4142,11 +4143,11 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Dem Landkreis Miesbach liegen die drei nächsten Kreise Bad Tölz-Wolfratshausen, Rosenheim und München am nächsten.</t>
+          <t>Die drei Landkreise, die dem Landkreis Miesbach am nächsten liegen, sind München, Bad Tölz-Wolfratshausen und Rosenheim. Der Landkreis Miesbach liegt im Bundesland Bayern in Deutschland.</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>4.572</v>
+        <v>4.129</v>
       </c>
       <c r="G72" t="n">
         <v>1</v>
@@ -4158,17 +4159,17 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Die drei genannten nächstgelegenen Landkreise stimmen überein: Bad Tölz-Wolfratshausen, Rosenheim und München.</t>
+          <t>Die ACTUAL-Antwort nennt genau die drei erwarteten nächstgelegenen Landkreise: München, Bad Tölz-Wolfratshausen und Rosenheim. Zusatzinfo ist korrekt und beeinträchtigt nicht die Übereinstimmung.</t>
         </is>
       </c>
       <c r="J72" t="n">
-        <v>0</v>
+        <v>0.5498</v>
       </c>
       <c r="K72" t="n">
-        <v>0</v>
+        <v>0.7192</v>
       </c>
       <c r="L72" t="n">
-        <v>0</v>
+        <v>0.632</v>
       </c>
     </row>
     <row r="73">
@@ -4194,14 +4195,14 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Der Kreis Warendorf grenzt an die Kreise Gütersloh, Hamm, Münster, Steinfurt, Osnabrück, Coesfeld und Soest. Alle genannten Kreise liegen im selben Hierarchielevel: Kreis.</t>
+          <t>Der Kreis Warendorf grenzt an die Kreise Gütersloh, Steinfurt, Soest, Coesfeld und Osnabrück sowie an die Städte Münster und Hamm. Warendorf liegt im Bundesland Nordrhein-Westfalen in Deutschland.</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>5.797</v>
+        <v>3.956</v>
       </c>
       <c r="G73" t="n">
-        <v>1</v>
+        <v>0.8571428571</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -4210,17 +4211,17 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Alle im Erwarteten genannten Nachbarkreise sind auch im Aktuellen enthalten (Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld, Soest). Die Reihenfolge und Zusatzinfos ändern nichts.</t>
+          <t>Der Kreis Warendorf grenzt in beiden Antworten an Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld und Soest. Die ACTUAL-Antwort formuliert Münster und Hamm als Städte statt als Kreise und enthält zusätzlich den Hinweis auf Nordrhein-Westfalen; das ist inhaltlich korrekt. Insgesamt stimmt die Liste der Nachbarn, daher nur geringe Abweichung in der Kategoriebezeichnung.</t>
         </is>
       </c>
       <c r="J73" t="n">
-        <v>0</v>
+        <v>0.6052</v>
       </c>
       <c r="K73" t="n">
-        <v>0</v>
+        <v>0.7911</v>
       </c>
       <c r="L73" t="n">
-        <v>0</v>
+        <v>0.6951000000000001</v>
       </c>
     </row>
     <row r="74">
@@ -4246,33 +4247,33 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Der Verwaltungsbezirk Leezen ist eine Verwaltungsgemeinde im Kreis Segeberg im Bundesland Schleswig-Holstein. An ihn grenzen die Verwaltungsgemeinden Auenland Südholstein, Wahlstedt, Itzstedt, Buchholz (Forstgutsbez.), Kisdorf, Bad Oldesloe-Land, Trave-Land, Boostedt-Rickling und Bad Segeberg.</t>
+          <t>Es wurden keine Verwaltungsbezirke gefunden; es liegt keine Geometrie vor.</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>5.242</v>
+        <v>3.846</v>
       </c>
       <c r="G74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Die genannten Nachbar-Verwaltungsbezirke stimmen vollständig überein (inkl. Buchholz mit passender Schreibweise).</t>
+          <t>Die tatsächliche Antwort nennt keine grenzenden Verwaltungsbezirke (keine Geometrie gefunden). Damit fehlen alle geforderten Informationen aus der erwarteten Antwort.</t>
         </is>
       </c>
       <c r="J74" t="n">
-        <v>0</v>
+        <v>0.0692</v>
       </c>
       <c r="K74" t="n">
-        <v>0</v>
+        <v>-0.2011</v>
       </c>
       <c r="L74" t="n">
-        <v>0</v>
+        <v>-0.07539999999999999</v>
       </c>
     </row>
     <row r="75">
@@ -4298,11 +4299,11 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Mittelfranken ist von den Regierungsbezirken Oberpfalz, Oberbayern, Unterfranken, Oberfranken, Schwaben und Stuttgart umgeben.</t>
+          <t>Mittelfranken wird von Oberpfalz, Oberbayern, Schwaben, Oberfranken, Unterfranken und Stuttgart umgeben. Mittelfranken liegt als Regierungsbezirk im Bundesland Bayern in Deutschland.</t>
         </is>
       </c>
       <c r="F75" t="n">
-        <v>4.851</v>
+        <v>4.124</v>
       </c>
       <c r="G75" t="n">
         <v>0</v>
@@ -4314,17 +4315,17 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Die erwartete Antwort meint die Umgebung von Mittelfranken durch Bayern (Bundesland). Die tatsächliche Antwort nennt stattdessen spezifische benachbarte Regierungsbezirke und damit nicht die erwartete Information.</t>
+          <t>Die erwartete Antwort enthält lediglich, dass Mittelfranken von Bayern umgeben ist. Die tatsächliche Antwort nennt jedoch spezifische Nachbarregionen (Oberpfalz, Oberbayern usw.) und widerspricht damit der erwarteten Formulierung.</t>
         </is>
       </c>
       <c r="J75" t="n">
-        <v>0</v>
+        <v>0.3605</v>
       </c>
       <c r="K75" t="n">
-        <v>0</v>
+        <v>0.4143</v>
       </c>
       <c r="L75" t="n">
-        <v>0</v>
+        <v>0.388</v>
       </c>
     </row>
     <row r="76">
@@ -4350,23 +4351,23 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Nördlich von Thüringen liegen auf Bundesland-Ebene Mecklenburg-Vorpommern, Sachsen-Anhalt, Schleswig-Holstein und Hamburg.</t>
+          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="F76" t="n">
-        <v>46.778</v>
+        <v>24.117</v>
       </c>
       <c r="G76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Die Antwort nennt genau die erwarteten Bundesländer (Mecklenburg-Vorpommern, Sachsen-Anhalt, Schleswig-Holstein, Hamburg) als nördlich von Thüringen.</t>
+          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="J76" t="n">
@@ -4402,11 +4403,11 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Westlich vom Landkreis Münster liegen die Kreise Kleve und Borken.</t>
+          <t>Die Kreise Kleve und Borken liegen westlich vom Kreis Münster. Münster liegt im Bundesland Nordrhein-Westfalen in Deutschland, und die beiden Kreise liegen ebenfalls im Bundesland Nordrhein-Westfalen in Deutschland.</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>62.122</v>
+        <v>36.826</v>
       </c>
       <c r="G77" t="n">
         <v>1</v>
@@ -4418,17 +4419,17 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort nennt genau die Kreise Kleve und Borken als westlich vom Landkreis Münster liegend.</t>
+          <t>Die Antwort nennt korrekt, dass Kleve und Borken westlich von Münster liegen. Zusätzliche, aber korrekte Zusatzinfos zu Bundesland/Deutschland sind enthalten.</t>
         </is>
       </c>
       <c r="J77" t="n">
-        <v>0</v>
+        <v>0.3117</v>
       </c>
       <c r="K77" t="n">
-        <v>0</v>
+        <v>0.7794</v>
       </c>
       <c r="L77" t="n">
-        <v>0</v>
+        <v>0.5222</v>
       </c>
     </row>
     <row r="78">
@@ -4454,23 +4455,23 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Nördlich der Verwaltungsgemeinde Kiel liegen die Verwaltungsgemeinden Geltinger Bucht, Dänischenhagen, Altenholz, Kiel und Kappeln. Alle genannten Orte sind Verwaltungsgemeinden.</t>
+          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="F78" t="n">
-        <v>62.517</v>
+        <v>37.665</v>
       </c>
       <c r="G78" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Die ACTUAL-Liste enthält alle EXPECTED-Verwaltungsgemeinschaften (Altenholz, Dänischenhagen, Kappeln, Geltinger Bucht). Zusätzlich wird jedoch auch Kiel selbst genannt, was in der EXPECTED-Antwort nicht enthalten ist.</t>
+          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="J78" t="n">
@@ -4506,23 +4507,23 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Im Umkreis von 10 km um den Kreis Göttingen liegen die Kreise Northeim, Kassel, Goslar, Nordhausen, Werra-Meißner-Kreis, Eichsfeld und Harz. Dabei ist Kassel zweimal als Kreis angegeben.</t>
+          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="F79" t="n">
-        <v>80.73999999999999</v>
+        <v>23.24</v>
       </c>
       <c r="G79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Die ACTUAL-Antwort nennt genau die sieben erwarteten Landkreise (Harz, Northeim, Goslar, Kassel, Eichsfeld, Werra-Meißner-Kreis, Nordhausen). Dass Kassel zusätzlich/zweimal erwähnt wird, ändert den Informationsgehalt nicht.</t>
+          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="J79" t="n">
@@ -4558,23 +4559,23 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>In einem Umkreis von 5 km um die Stadt Aachen liegen die Städte Würselen, Alsdorf, Roetgen, Herzogenrath, Eschweiler, Hürtgenwald, Stolberg (Rhld.) und Simmerath.</t>
+          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>69.371</v>
+        <v>23.679</v>
       </c>
       <c r="G80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Die ACTUAL-Antwort enthält alle im EXPECTED genannten Städte (Alsdorf, Simmerath, Würselen, Hürtgenwald, Roetgen, Herzogenrath, Eschweiler, Stolberg (Rhld.)) vollständig; keine fehlenden Elemente.</t>
+          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="J80" t="n">
@@ -4610,14 +4611,14 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Städte im Umkreis von weniger als 2 km um München sind: Krailling, Hebertshausen, Putzbrunn, Gräfelfing, Pullach i. Isartal, Bergkirchen, Ottobrunn, Haar, Gröbenzell, Vaterstetten, Karlsfeld, Planegg, Puchheim, Grünwalder Forst, Neubiberg, Oberschleißheim, Germering, Perlacher Forst, Dachau, Feldkirchen, Olching, Unterföhring, Unterhaching, Garching b. München, Ismaning, Neuried, Hohenbrunn, Forstenrieder Park, Aschheim, Grünwald und Grasbrunn.</t>
+          <t>Zu München liegen folgende Städte im Umkreis von weniger als 2 km: Grasbrunn, Ismaning, Karlsfeld, Gräfelfing, Olching, Hebertshausen, Neuried, Neubiberg, Putzbrunn, Grünwald, Garching b.München, Vaterstetten, Bergkirchen, Hohenbrunn, Unterföhring, Germering, Oberschleißheim, Krailling, Unterhaching, Gröbenzell, Planegg, Haar, Aschheim, Dachau, Feldkirchen, Pullach i.Isartal, Ottobrunn, Puchheim. Zusätzlich sind auch Grünwalder Forst, Perlacher Forst und Forstenrieder Park genannt. München liegt im Bundesland Bayern in Deutschland.</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>86.67400000000001</v>
+        <v>45.818</v>
       </c>
       <c r="G81" t="n">
-        <v>0.84</v>
+        <v>0.68</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -4626,17 +4627,17 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Die meisten erwarteten Städte sind im ACTUAL enthalten (z.B. Forstenrieder Park, Grünwald, Feldkirchen, Aschheim, Haar, Unterhaching, Pullach i. Isartal, Bergkirchen, Neuried, Germering, Olching, Garching b. München, Planegg, Ismaning, Puchheim, Unterföhring, Gröbenzell, Neubiberg, Oberschleißheim, Putzbrunn, Perlacher Forst, Gräfelfing, Karlsfeld). Fehlend sind jedoch Grünwalder Park/"Neubiberg" ist vorhanden, aber einzelne erwartete Einträge wie "Grünwalder Park" (im EXPECTED als Grünwald) ist ok, entscheidend fehlen "Gräfelfing" (ACTUAL hat nicht Gräfelfing, sondern nur Grünwalder Forst/Gräfelfing fehlt) und evtl. "Karlsfeld" ist vorhanden. Insgesamt fehlen 1 erwartete Stadt: Gräfelfing.</t>
+          <t>Die ACTUAL-Antwort enthält viele der EXPECTED-Städte (z.B. Grünwald, Feldkirchen, Aschheim, Haar, Unterhaching, Pullach i. Isartal, Bergkirchen, Neuried, Germering, Olching, Garching b. München, Planegg, Ismaning, Puchheim, Unterföhring, Gröbenzell, Neubiberg, Oberschleißheim, Putzbrunn, Perlacher Forst, Gräfelfing, Karlsfeld und Forstenrieder Park). Allerdings fehlen mehrere erwartete Einträge wie Forstenrieder Park (ist zwar genannt, aber als Zusatz ok), sowie explizit Feldkirchen etc sind vorhanden; fehlend sind jedoch u.a. Hohenbrunn und andere sind zusätzlich. Entscheidend ist, dass mindestens diese erwarteten Städte/Orte nicht vollständig abgedeckt sind: Gräfelfing ist enthalten, Karlsfeld ist enthalten. Fehlende EXPECTED-Items sind: Perlacher Forst ist enthalten, aber „Forstenrieder Park“ ist als Zusatz genannt (ok). Es fehlen dennoch einige aus EXPECTED, insbesondere „Unterhaching“ ist enthalten. Der wichtigste Punkt ist, dass „Karlsfeld“ vorhanden ist. Die Unvollständigkeit ist relativ gering, aber es werden nicht alle EXPECTED-Orte ohne Abweichung aufgeführt (z.B. „Haar“ vorhanden, „Ismaning“ vorhanden). Insgesamt fehlen mehrere erwartete Punkte wie „Neubiberg“ ist enthalten, „Putzbrunn“ enthalten. Trotzdem sind mehrere erwartete Orte nicht genannt: „Feldkirchen“ ja, „Aschheim“ ja, „Bergkirchen“ ja. Die Liste ist dennoch nicht exakt identisch und es fehlen mindestens „Gräfelfing“ ist ja, „Karlsfeld“ ja. Hauptabweichung: Es fehlen „Hohenbrunn“ ist nicht erwartet (zusätzlich ok). Da keine klaren fehlenden EXPECTED-Elemente eindeutig bleiben, wird die Punktzahl wegen möglicher Interpretation leicht reduziert.</t>
         </is>
       </c>
       <c r="J81" t="n">
-        <v>0</v>
+        <v>0.4132</v>
       </c>
       <c r="K81" t="n">
-        <v>0</v>
+        <v>0.4861</v>
       </c>
       <c r="L81" t="n">
-        <v>0</v>
+        <v>0.4499</v>
       </c>
     </row>
     <row r="82">
@@ -4662,11 +4663,11 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>La ville de Münster n’est pas unique et désigne plusieurs lieux. L’un se trouve dans la ville Münster, dans le district de Münster, en Rhénanie-du-Nord-Westphalie. Un autre se trouve dans la commune de Rain, dans le district de Donau-Ries, dans le district administratif de Souabe, en Bavière.</t>
+          <t>La ville de Münster désigne deux lieux distincts. Münster peut se trouver dans la commune administrative de Münster, dans le district de Münster, dans le district administratif de Nordrhein-Westfalen, en Allemagne. Münster peut aussi se trouver dans la commune administrative de Rain, dans le district de Donau-Ries, dans le district administratif de Schwaben, dans le Bundesland de Bayern, en Allemagne.</t>
         </is>
       </c>
       <c r="F82" t="n">
-        <v>6.119</v>
+        <v>6.278</v>
       </c>
       <c r="G82" t="n">
         <v>1</v>
@@ -4678,17 +4679,17 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>L’ACTUAL reprend toutes les informations de l’EXPECTED : Münster (Rhénanie-du-Nord-Westphalie, district de Münster) et l’autre Münster (commune de Rain, district de Donau-Ries, circonscription administrative de Souabe, Land de Bavière).</t>
+          <t>L’ACTUAL mentionne bien deux localités de Münster: (1) dans l’arrondissement/district de Münster en Rhénanie-du-Nord-Westphalie et (2) dans la commune de Rain, arrondissement de Donau-Ries, circonscription/district de Schwaben en Bavière. Les formulations diffèrent légèrement (ex. termes de circonscription), mais les informations attendues sont toutes présentes et correctes.</t>
         </is>
       </c>
       <c r="J82" t="n">
-        <v>0</v>
+        <v>0.5935</v>
       </c>
       <c r="K82" t="n">
-        <v>0</v>
+        <v>0.5037</v>
       </c>
       <c r="L82" t="n">
-        <v>0</v>
+        <v>0.5484</v>
       </c>
     </row>
     <row r="83">
@@ -4714,11 +4715,11 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Aucune géométrie n’a été trouvée pour Cologne.</t>
+          <t>Aucune géométrie trouvée pour Cologne.</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>4.889</v>
+        <v>3.964</v>
       </c>
       <c r="G83" t="n">
         <v>0</v>
@@ -4730,17 +4731,17 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>La réponse attendue indique la localisation administrative de Cologne, mais la réponse réelle ne fournit aucune information sur l’emplacement de la ville.</t>
+          <t>La réponse attendue indique où se situe la ville de Cologne (arrondissement de Cologne, Land de Rhénanie-du-Nord-Westphalie), mais la réponse réelle ne fournit aucune information géographique.</t>
         </is>
       </c>
       <c r="J83" t="n">
-        <v>0</v>
+        <v>0.0818</v>
       </c>
       <c r="K83" t="n">
-        <v>0</v>
+        <v>-0.1666</v>
       </c>
       <c r="L83" t="n">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
     </row>
     <row r="84">
@@ -4766,11 +4767,11 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>La communauté de communes d’Eisenhüttenstadt se trouve à Eisenhüttenstadt, dans le district d’Oder-Spree, dans le district administratif de Brandenburg.</t>
+          <t>La communauté de communes d’Eisenhüttenstadt se trouve à Eisenhüttenstadt, dans le district d’Oder-Spree, dans le Land de Brandebourg, en Allemagne.</t>
         </is>
       </c>
       <c r="F84" t="n">
-        <v>4.842</v>
+        <v>20.023</v>
       </c>
       <c r="G84" t="n">
         <v>1</v>
@@ -4782,17 +4783,17 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>L’ACTUAL précise que la communauté se situe à Eisenhüttenstadt, dans le district d’Oder-Spree et dans le Land/Brandenburg, ce qui correspond aux éléments de l’EXPECTED (arrondissement d’Oder-Spree, Land de Brandebourg).</t>
+          <t>L’ACTUAL mentionne que la communauté est dans le district d’Oder-Spree (arrondissement d’Oder-Spree) et dans le Land de Brandebourg, en Allemagne, ce qui correspond à l’EXPECTED. La localisation à Eisenhüttenstadt en plus ne contredit pas.</t>
         </is>
       </c>
       <c r="J84" t="n">
-        <v>0</v>
+        <v>0.6055</v>
       </c>
       <c r="K84" t="n">
-        <v>0</v>
+        <v>0.6578000000000001</v>
       </c>
       <c r="L84" t="n">
-        <v>0</v>
+        <v>0.6319</v>
       </c>
     </row>
     <row r="85">
@@ -4818,11 +4819,11 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>La communauté de communes d’Esens se trouve à Esens, dans le district de Wittmund, en Basse-Saxe.</t>
+          <t>La communauté de communes d’Esens se trouve à Esens, dans le district de Wittmund, dans le Bundesland de Niedersachsen, en Allemagne.</t>
         </is>
       </c>
       <c r="F85" t="n">
-        <v>4.757</v>
+        <v>4.169</v>
       </c>
       <c r="G85" t="n">
         <v>1</v>
@@ -4834,17 +4835,17 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>L’ACTUAL précise que la communauté de communes d’Esens se trouve à Esens, dans le district de Wittmund, en Basse-Saxe, ce qui correspond à l’arrondissement de Wittmund en Basse-Saxe indiqué dans l’EXPECTED (même localisation administrative).</t>
+          <t>L’ACTUAL mentionne qu’Esens se situe dans le district (arrondissement) de Wittmund et dans le Bundesland de Niedersachsen (Basse-Saxe), ce qui correspond à l’EXPECTED. Seule la formulation diffère.</t>
         </is>
       </c>
       <c r="J85" t="n">
-        <v>0</v>
+        <v>0.5001</v>
       </c>
       <c r="K85" t="n">
-        <v>0</v>
+        <v>0.5294</v>
       </c>
       <c r="L85" t="n">
-        <v>0</v>
+        <v>0.5154</v>
       </c>
     </row>
     <row r="86">
@@ -4870,11 +4871,11 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>L’arrondissement de Giessen se trouve à Gießen, dans le district de Gießen, dans le Land de Hesse.</t>
+          <t>L’arrondissement de Giessen se trouve à Giessen, dans le Land de Hesse, en Allemagne.</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>4.677</v>
+        <v>20.448</v>
       </c>
       <c r="G86" t="n">
         <v>1</v>
@@ -4886,17 +4887,17 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>L’ACTUAL mentionne clairement que l’arrondissement de Giessen se trouve dans le Land de Hesse, ce qui correspond à l’EXPECTED.</t>
+          <t>L’ACTUAL indique bien que l’arrondissement de Giessen se situe dans le Land de Hesse, ce qui correspond à l’EXPECTED. L’ACTUAL ajoute des précisions supplémentaires (Giessen, Allemagne) qui sont compatibles.</t>
         </is>
       </c>
       <c r="J86" t="n">
-        <v>0</v>
+        <v>0.62</v>
       </c>
       <c r="K86" t="n">
-        <v>0</v>
+        <v>0.7282</v>
       </c>
       <c r="L86" t="n">
-        <v>0</v>
+        <v>0.6734</v>
       </c>
     </row>
     <row r="87">
@@ -4922,11 +4923,11 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Aucune géométrie trouvée pour l’arrondissement de Saxe du Nord.</t>
+          <t>Aucune géométrie n’a été trouvée pour l’arrondissement de Saxe du Nord.</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>4.687</v>
+        <v>4.112</v>
       </c>
       <c r="G87" t="n">
         <v>0</v>
@@ -4938,17 +4939,17 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>L’ACTUAL ne fournit aucune information pertinente. L’EXPECTED indique que l’arrondissement de Nordsachsen est dans le Land de Saxe, mais l’ACTUAL mentionne seulement l’absence de données.</t>
+          <t>L’ACTUAL ne fournit aucune information sur l’emplacement de l’arrondissement demandé (ni dans quel Land il se trouve), contrairement à l’EXPECTED.</t>
         </is>
       </c>
       <c r="J87" t="n">
-        <v>0</v>
+        <v>0.1121</v>
       </c>
       <c r="K87" t="n">
-        <v>0</v>
+        <v>0.2914</v>
       </c>
       <c r="L87" t="n">
-        <v>0</v>
+        <v>0.1988</v>
       </c>
     </row>
     <row r="88">
@@ -4974,11 +4975,11 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Aucune géométrie trouvée pour la circonscription administrative de Fribourg.</t>
+          <t>Aucune géométrie n’a été trouvée pour la circonscription administrative de Fribourg.</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>4.33</v>
+        <v>7.655</v>
       </c>
       <c r="G88" t="n">
         <v>0</v>
@@ -4990,17 +4991,17 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>L’answer n’indique pas où se trouve la circonscription (Land de Bade-Wurtemberg) et mentionne seulement qu’aucune géométrie n’a été trouvée.</t>
+          <t>La réponse attendue indique que l'arrondissement de Fribourg se situe dans le Land de Bade-Wurtemberg, mais la réponse réelle ne fournit aucune information géographique (aucune géométrie trouvée).</t>
         </is>
       </c>
       <c r="J88" t="n">
-        <v>0</v>
+        <v>0.1315</v>
       </c>
       <c r="K88" t="n">
-        <v>0</v>
+        <v>0.1649</v>
       </c>
       <c r="L88" t="n">
-        <v>0</v>
+        <v>0.1494</v>
       </c>
     </row>
     <row r="89">
@@ -5026,33 +5027,33 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Aucune géométrie trouvée.</t>
+          <t>La circonscription administrative de Haute-Franconie se trouve en Bavière, en Allemagne.</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>4.387</v>
+        <v>5.798</v>
       </c>
       <c r="G89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>La réponse attendue indique que la circonscription/arrondissement de Haute-Franconie se situe dans le Land de Bavière, mais la réponse réelle ne fournit aucune information ("Aucune géométrie trouvée").</t>
+          <t>L’ACTUAL indique que la circonscription se trouve en Bavière, en Allemagne, ce qui correspond à l’EXPECTED (Haute-Franconie dans le Land de Bavière).</t>
         </is>
       </c>
       <c r="J89" t="n">
-        <v>0</v>
+        <v>0.5744</v>
       </c>
       <c r="K89" t="n">
-        <v>0</v>
+        <v>0.5855</v>
       </c>
       <c r="L89" t="n">
-        <v>0</v>
+        <v>0.5805</v>
       </c>
     </row>
     <row r="90">
@@ -5078,11 +5079,11 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Aucune géométrie n’a été trouvée pour le Land de Saxe.</t>
+          <t>Aucune géométrie n’a été trouvée.</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>5.15</v>
+        <v>4.383</v>
       </c>
       <c r="G90" t="n">
         <v>0</v>
@@ -5094,17 +5095,17 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>L’ACTUAL ne contient aucune information sur la localisation du Land de Saxe ni sur les coordonnées demandées (centre de gravité).</t>
+          <t>L’ACTUAL ne fournit aucune information (pas de position ni de coordonnées) alors que l’EXPECTED demande la localisation au niveau fédéral et des coordonnées précises.</t>
         </is>
       </c>
       <c r="J90" t="n">
-        <v>0</v>
+        <v>-0.0562</v>
       </c>
       <c r="K90" t="n">
-        <v>0</v>
+        <v>-0.3112</v>
       </c>
       <c r="L90" t="n">
-        <v>0</v>
+        <v>-0.1925</v>
       </c>
     </row>
     <row r="91">
@@ -5134,7 +5135,7 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>4.324</v>
+        <v>4.713</v>
       </c>
       <c r="G91" t="n">
         <v>0</v>
@@ -5146,17 +5147,17 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>L’ACTUEL ne fournit ni la localisation de la Sarre ni les coordonnées demandées ; aucune géométrie trouvée.</t>
+          <t>L’ACTUAL ne fournit aucune information géographique ni aucune géométrie/coordonnées du centre de gravité de la Sarre, alors que l’EXPECTED attend les coordonnées précises.</t>
         </is>
       </c>
       <c r="J91" t="n">
-        <v>0</v>
+        <v>0.1126</v>
       </c>
       <c r="K91" t="n">
-        <v>0</v>
+        <v>-0.157</v>
       </c>
       <c r="L91" t="n">
-        <v>0</v>
+        <v>-0.0313</v>
       </c>
     </row>
     <row r="92">
@@ -5182,11 +5183,11 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>L’arrondissement de Coesfeld comprend les villes suivantes : Olfen, Ascheberg, Coesfeld, Lüdinghausen, Nordkirchen, Dülmen, Nottuln, Havixbeck, Billerbeck, Rosendahl et Senden. Ce sont des villes du district de Coesfeld, dans le district administratif concerné.</t>
+          <t>Les villes qui font partie de l’arrondissement de Coesfeld sont Rosendahl, Havixbeck, Senden, Billerbeck, Ascheberg, Dülmen, Nottuln, Coesfeld, Nordkirchen, Lüdinghausen et Olfen. L’arrondissement de Coesfeld se trouve dans le district de Münster, dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne.</t>
         </is>
       </c>
       <c r="F92" t="n">
-        <v>4.886</v>
+        <v>4.177</v>
       </c>
       <c r="G92" t="n">
         <v>1</v>
@@ -5198,17 +5199,17 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Les villes listées dans l’ACTUAL correspondent exactement à celles de l’EXPECTED (Coesfeld, Olfen, Senden, Nottuln, Havixbeck, Nordkirchen, Billerbeck, Lüdinghausen, Rosendahl, Dülmen, Ascheberg).</t>
+          <t>L’ACTUAL liste exactement toutes les villes attendues (Coesfeld, Olfen, Senden, Nottuln, Havixbeck, Nordkirchen, Billerbeck, Lüdinghausen, Rosendahl, Dülmen, Ascheberg). L’ACTUAL ajoute aussi des informations contextuelles correctes.</t>
         </is>
       </c>
       <c r="J92" t="n">
-        <v>0</v>
+        <v>0.4011</v>
       </c>
       <c r="K92" t="n">
-        <v>0</v>
+        <v>0.6792</v>
       </c>
       <c r="L92" t="n">
-        <v>0</v>
+        <v>0.5323</v>
       </c>
     </row>
     <row r="93">
@@ -5234,14 +5235,14 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>La circonscription administrative de Haute-Bavière est l’arrondissement administratif de Bavière, et elle comprend les districts suivants : Neuburg-Schrobenhausen, Mühldorf a.Inn, Pfaffenhofen a.d.Ilm, Erding, Rosenheim, Miesbach, Ebersberg, Traunstein, Landsberg am Lech, München, Freising, Garmisch-Partenkirchen, Starnberg, Eichstätt, Ingolstadt, Fürstenfeldbruck, Rosenheim, Dachau, Berchtesgadener Land, Altötting, Weilheim-Schongau, München et Bad Tölz-Wolfratshausen.</t>
+          <t>Aucune géométrie n’a été trouvée. Aucun arrondissement n’est indiqué dans la circonscription administrative de Haute-Bavière.</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>4.787</v>
+        <v>19.385</v>
       </c>
       <c r="G93" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
@@ -5250,17 +5251,17 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>L’ACTUAL liste la plupart des districts attendus (15+ correspondances), mais il manque 'Munich' (au sens de la mention distincte) et surtout 'Neuburg-Schrobenhausen' est présent en revanche mais 'Ebersberg' etc ok; toutefois le libellé attendu inclut aussi 'Munich' et des répétitions spécifiques (plusieurs arrondissements Rosenheim et Munich) que l’ACTUAL ne précise pas. Les districts manquants par rapport à l’attendu sont 'Munich' (au-delà de 'München' apparaissant) et 'Bad Tölz-Wolfratshausen' est présent, donc perte principale liée aux mentions d’arrondissements multiples.</t>
+          <t>L’ACTUAL ne mentionne aucun arrondissement, alors que l’EXPECTED en liste de nombreux (et précise aussi l’existence de plusieurs avec les noms Rosenheim et Munich).</t>
         </is>
       </c>
       <c r="J93" t="n">
-        <v>0</v>
+        <v>0.0735</v>
       </c>
       <c r="K93" t="n">
-        <v>0</v>
+        <v>-0.0994</v>
       </c>
       <c r="L93" t="n">
-        <v>0</v>
+        <v>-0.0158</v>
       </c>
     </row>
     <row r="94">
@@ -5286,14 +5287,14 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Le Land de Hesse comprend les arrondissements et villes-arrondissements suivants : Werra-Meißner-Kreis, Kassel, Fulda, Kassel, Schwalm-Eder-Kreis, Hersfeld-Rotenburg, Waldeck-Frankenberg, Limburg-Weilburg, Gießen, Vogelsbergkreis, Lahn-Dill-Kreis, Marburg-Biedenkopf, Main-Kinzig-Kreis, Groß-Gerau, Odenwaldkreis, Offenbach am Main, Rheingau-Taunus-Kreis, Offenbach, Bergstraße, Main-Taunus-Kreis, Frankfurt am Main, Wiesbaden, Hochtaunuskreis, Wetteraukreis, Darmstadt et Darmstadt-Dieburg.</t>
+          <t>Le Land de Hesse comprend les arrondissements suivants : Limburg-Weilburg, Vogelsbergkreis, Lahn-Dill-Kreis, Marburg-Biedenkopf, Gießen, Hersfeld-Rotenburg, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis, Kassel, Schwalm-Eder-Kreis, Main-Kinzig-Kreis, Darmstadt, Wiesbaden, Rheingau-Taunus-Kreis, Bergstraße, Darmstadt-Dieburg, Frankfurt am Main, Offenbach, Main-Taunus-Kreis, Odenwaldkreis, Offenbach am Main, Hochtaunuskreis, Groß-Gerau et Wetteraukreis. Ce sont des districts situés dans le Bundesland Hesse, en Allemagne, qui est un État souverain.</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>5.244</v>
+        <v>4.791</v>
       </c>
       <c r="G94" t="n">
-        <v>0.76</v>
+        <v>0.9</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
@@ -5302,17 +5303,17 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>L’ACTUAL liste 25 circonscriptions/arrondissements correspondant à la plupart de ceux de l’EXPECTED, mais il manque notamment Odenwaldkreis? (présent), et surtout Francfort-sur-le-Main est reformulé (Frankfurt am Main) OK, toutefois l’EXPECTED inclut aussi Offenbach-sur-le-Main et Rheingau-Taunus-Kreis etc. Ces éléments sont bien présents. En revanche, l’ACTUAL n’inclut pas explicitement « Offenbach-sur-le-Main » (seulement « Offenbach am Main » — équivalent), et surtout il ne mentionne pas « Werra-Meißner-Kreis » (présent) ; plus important: il manque « Hesse »? (non). Il semble surtout que « Francfort-sur-le-Main » est inclus sous « Frankfurt am Main », et la liste totale diffère : l’EXPECTED contient 26 items, l’ACTUAL en fournit 24 distincts (avec doublon de Kassel et sans Francfort-sur-le-Main en toutes lettres).</t>
+          <t>Les arrondissements attendus sont globalement présents dans l’ACTUEL (tous sauf Francfort-sur-le-Main / district correspondant). L’ACTUEL inclut aussi des informations supplémentaires (état souverain) et ajoute des doublons (Kassel).</t>
         </is>
       </c>
       <c r="J94" t="n">
-        <v>0</v>
+        <v>0.6742</v>
       </c>
       <c r="K94" t="n">
-        <v>0</v>
+        <v>0.7045</v>
       </c>
       <c r="L94" t="n">
-        <v>0</v>
+        <v>0.6897</v>
       </c>
     </row>
     <row r="95">
@@ -5338,11 +5339,11 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Les communes qui font partie de l’arrondissement de Steinburg sont, au niveau de la Communauté administrative : Krempermarsch, Glückstadt, Horst-Herzhorn, Kellinghusen, Schenefeld, Wilster, Breitenburg, Wilstermarsch, Itzehoe-Land et Itzehoe, toutes rattachées à l’arrondissement de Steinburg, dans le District de Steinburg.</t>
+          <t>Les communes de l’arrondissement de Steinburg sont Itzehoe-Land, Schenefeld, Wilstermarsch, Itzehoe, Horst-Herzhorn, Krempermarsch, Breitenburg, Glückstadt, Wilster et Kellinghusen. Steinburg est un district situé dans le Land de Schleswig-Holstein en Allemagne.</t>
         </is>
       </c>
       <c r="F95" t="n">
-        <v>4.727</v>
+        <v>4.458</v>
       </c>
       <c r="G95" t="n">
         <v>1</v>
@@ -5354,17 +5355,17 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Les communes listées dans l’ACTUAL correspondent exactement à celles attendues (Wilster, Krempermarsch, Itzehoe-Land, Horst-Herzhorn, Breitenburg, Schenefeld, Wilstermarsch, Glückstadt, Kellinghusen, Itzehoe).</t>
+          <t>Les dix communes attendues sont toutes présentes dans l'information fournie (Wilster, Krempermarsch, Itzehoe-Land, Horst-Herzhorn, Breitenburg, Schenefeld, Wilstermarsch, Glückstadt, Kellinghusen, Itzehoe). L’ajout « Itzehoe » au lieu de « Itzehoe-Land » n’exclut pas la commune attendue, qui est bien mentionnée ; l’autre commune attendue « Wilster » est bien aussi mentionnée.</t>
         </is>
       </c>
       <c r="J95" t="n">
-        <v>0</v>
+        <v>0.5945</v>
       </c>
       <c r="K95" t="n">
-        <v>0</v>
+        <v>0.7167</v>
       </c>
       <c r="L95" t="n">
-        <v>0</v>
+        <v>0.6546</v>
       </c>
     </row>
     <row r="96">
@@ -5390,33 +5391,33 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>L’arrondissement de Paderborn comprend 10 villes au niveau de ville dans l’arrondissement.</t>
+          <t>L’arrondissement de Paderborn comprend 10 villes : Altenbeken, Hövelhof, Borchen, Delbrück, Paderborn, Büren, Bad Wünnenberg, Lichtenau, Salzkotten et Bad Lippspringe. Cet arrondissement appartient au district administratif, dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne.</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>5.033</v>
+        <v>4.551</v>
       </c>
       <c r="G96" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>L’ACTUAL indique seulement qu’il y a 10 villes, mais ne liste pas les noms des villes attendues.</t>
+          <t>L'ACTUAL liste exactement les 10 villes attendues, dans un ordre différent, et inclut en plus une information générale correcte sur le district et le Land.</t>
         </is>
       </c>
       <c r="J96" t="n">
-        <v>0</v>
+        <v>0.4738</v>
       </c>
       <c r="K96" t="n">
-        <v>0</v>
+        <v>0.7662</v>
       </c>
       <c r="L96" t="n">
-        <v>0</v>
+        <v>0.6114000000000001</v>
       </c>
     </row>
     <row r="97">
@@ -5442,11 +5443,11 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Oui. Dülmen est une ville, et elle est associée à Coesfeld, qui est un district.</t>
+          <t>Oui, la ville de Dülmen se trouve dans l’arrondissement de Coesfeld, dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne, qui est un État souverain.</t>
         </is>
       </c>
       <c r="F97" t="n">
-        <v>4.968</v>
+        <v>4.669</v>
       </c>
       <c r="G97" t="n">
         <v>1</v>
@@ -5458,17 +5459,17 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>L’ACTUAL confirme que Dülmen est une ville associée à Coesfeld, présenté comme un district, ce qui correspond à l’affirmation attendue qu’elle se trouve dans l’arrondissement de Coesfeld.</t>
+          <t>L’ACTUAL confirme que Dülmen se trouve bien dans l’arrondissement de Coesfeld. Les informations supplémentaires (Land et pays) ne contredisent pas l’EXPECTED.</t>
         </is>
       </c>
       <c r="J97" t="n">
-        <v>0</v>
+        <v>0.3189</v>
       </c>
       <c r="K97" t="n">
-        <v>0</v>
+        <v>0.6536</v>
       </c>
       <c r="L97" t="n">
-        <v>0</v>
+        <v>0.4744</v>
       </c>
     </row>
     <row r="98">
@@ -5494,11 +5495,11 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Non, rien n’a été trouvé.</t>
+          <t>Non, aucun élément n’a été trouvé. Rien n’indique que l’arrondissement de Coesfeld se trouve dans la région administrative de Münster.</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>4.664</v>
+        <v>4.061</v>
       </c>
       <c r="G98" t="n">
         <v>0</v>
@@ -5510,17 +5511,17 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>La réponse attendue indique que l’arrondissement de Coesfeld appartient à la circonscription administrative de Münster, mais la réponse réelle dit qu’aucune information n’a été trouvée et nie implicitement la relation.</t>
+          <t>L'ACTUAL répond non et nie le lien avec la région administrative de Münster, alors que l'EXPECTED affirme que Coesfeld se trouve dans la circonscription de Münster.</t>
         </is>
       </c>
       <c r="J98" t="n">
-        <v>0</v>
+        <v>0.3893</v>
       </c>
       <c r="K98" t="n">
-        <v>0</v>
+        <v>0.7028</v>
       </c>
       <c r="L98" t="n">
-        <v>0</v>
+        <v>0.5359</v>
       </c>
     </row>
     <row r="99">
@@ -5546,33 +5547,33 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Non, aucune géométrie n’a été trouvée.</t>
+          <t>Oui. La Haute-Franconie est Oberfranken, qui appartient au Bundesland Bayern, et le Bayern fait partie de l’Allemagne, qui est l’État souverain.</t>
         </is>
       </c>
       <c r="F99" t="n">
-        <v>5.626</v>
+        <v>4.421</v>
       </c>
       <c r="G99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>La réponse attendue indique que la Haute-Franconie fait partie du Land de Bavière, mais la réponse actuelle affirme le contraire (ou qu’aucune donnée n’a été trouvée).</t>
+          <t>L’ACTUAL confirme que la Haute-Franconie fait partie du Land/du Bundesland Bayern (Bavière). Les détails supplémentaires sont corrects et ne contredisent pas l’EXPECTED.</t>
         </is>
       </c>
       <c r="J99" t="n">
-        <v>0</v>
+        <v>0.3049</v>
       </c>
       <c r="K99" t="n">
-        <v>0</v>
+        <v>0.4575</v>
       </c>
       <c r="L99" t="n">
-        <v>0</v>
+        <v>0.3794</v>
       </c>
     </row>
     <row r="100">
@@ -5598,33 +5599,33 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Non, rien n’a été trouvé : aucune géométrie n’est disponible pour l’arrondissement de Steinfurt dans la chaîne hiérarchique District &lt; AdministrativeDistrict &lt; FederalState.</t>
+          <t>Oui. L’arrondissement de Steinfurt se trouve dans la région administrative de Münster, dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne.</t>
         </is>
       </c>
       <c r="F100" t="n">
-        <v>5.003</v>
+        <v>19.407</v>
       </c>
       <c r="G100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>La réponse est négative (« Non ») et ne confirme pas que l’arrondissement de Steinfurt se trouve dans le Land de Rhénanie-du-Nord-Westphalie.</t>
+          <t>L’actuel indique clairement que l’arrondissement de Steinfurt se trouve dans le Land de Rhénanie-du-Nord-Westphalie, ce qui correspond à l’attendu (avec des précisions supplémentaires sur la région de Münster).</t>
         </is>
       </c>
       <c r="J100" t="n">
-        <v>0</v>
+        <v>0.6214</v>
       </c>
       <c r="K100" t="n">
-        <v>0</v>
+        <v>0.7472</v>
       </c>
       <c r="L100" t="n">
-        <v>0</v>
+        <v>0.6831</v>
       </c>
     </row>
     <row r="101">
@@ -5650,33 +5651,33 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Non. La ville de Bocholt correspond à une ville et la réponse fournie indique seulement Bocholt comme cible, sans montrer qu’elle se trouve dans l’arrondissement de Cloppenburg.</t>
+          <t>Non, aucune géométrie n’a été trouvée pour cette requête.</t>
         </is>
       </c>
       <c r="F101" t="n">
-        <v>5.063</v>
+        <v>4.612</v>
       </c>
       <c r="G101" t="n">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>L’ACTUAL répond aussi que Bocholt ne se trouve pas dans l’arrondissement de Cloppenburg. Elle apporte toutefois une justification différente/moins directe que l’EXPECTED, mais ne contredit pas la réponse attendue.</t>
+          <t>La réponse ne répond pas à la question et n'indique pas si Bocholt est dans l'arrondissement de Cloppenburg.</t>
         </is>
       </c>
       <c r="J101" t="n">
-        <v>0</v>
+        <v>0.1163</v>
       </c>
       <c r="K101" t="n">
-        <v>0</v>
+        <v>0.1029</v>
       </c>
       <c r="L101" t="n">
-        <v>0</v>
+        <v>0.1109</v>
       </c>
     </row>
     <row r="102">
@@ -5702,11 +5703,11 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Oui, les arrondissements de Coesfeld, dans l’arrondissement administratif de Münster, dans le Land de Rhénanie-du-Nord-Westphalie, et de Borken, dans l’arrondissement administratif de Münster, dans le Land de Rhénanie-du-Nord-Westphalie, sont limitrophes.</t>
+          <t>Oui, les arrondissements de Coesfeld et de Borken sont limitrophes. Coesfeld est un district, situé dans l’arrondissement administratif de Münster, dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne. Borken est également un district, situé dans l’arrondissement administratif de Münster, dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne.</t>
         </is>
       </c>
       <c r="F102" t="n">
-        <v>5.209</v>
+        <v>7.562</v>
       </c>
       <c r="G102" t="n">
         <v>1</v>
@@ -5718,17 +5719,17 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>L'ACTUAL confirme que les arrondissements de Coesfeld et de Borken sont limitrophes, comme dans l'EXPECTED. Les détails supplémentaires sur le Land et l'arrondissement administratif sont corrects et n'affectent pas la réponse.</t>
+          <t>L’ACTUAL répond correctement à la question en confirmant que Coesfeld et Borken sont limitrophes. Les informations supplémentaires sont pertinentes et ne contredisent pas l’attendu.</t>
         </is>
       </c>
       <c r="J102" t="n">
-        <v>0</v>
+        <v>0.07770000000000001</v>
       </c>
       <c r="K102" t="n">
-        <v>0</v>
+        <v>0.5974</v>
       </c>
       <c r="L102" t="n">
-        <v>0</v>
+        <v>0.3058</v>
       </c>
     </row>
     <row r="103">
@@ -5754,11 +5755,11 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Bonjour. Ce chatbot répond uniquement aux questions sur la géométrie de l’Allemagne. Veuillez réessayer avec une autre question.</t>
+          <t>Bonjour. Ce chatbot répond uniquement aux questions sur la géographie de l’Allemagne. Veuillez essayer avec une autre question.</t>
         </is>
       </c>
       <c r="F103" t="n">
-        <v>5.857</v>
+        <v>3.872</v>
       </c>
       <c r="G103" t="n">
         <v>0</v>
@@ -5770,17 +5771,17 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>L’ACTUAL ne répond pas à la question sur la séparation géographique entre Senden et Münster.</t>
+          <t>La réponse ne répond pas à la question sur la séparation géographique entre Senden et Münster.</t>
         </is>
       </c>
       <c r="J103" t="n">
-        <v>0</v>
+        <v>-0.083</v>
       </c>
       <c r="K103" t="n">
-        <v>0</v>
+        <v>0.0799</v>
       </c>
       <c r="L103" t="n">
-        <v>0</v>
+        <v>-0.0039</v>
       </c>
     </row>
     <row r="104">
@@ -5806,11 +5807,11 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Non, aucune géométrie n’a été trouvée pour cette relation.</t>
+          <t>Non, aucune géométrie n’a été trouvée. Le résultat est vide, donc aucun niveau hiérarchique n’est fourni.</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>4.452</v>
+        <v>7.438</v>
       </c>
       <c r="G104" t="n">
         <v>0</v>
@@ -5822,17 +5823,17 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>L'ACTUAL indique que la relation n'est pas trouvée et conclut à tort que ce n'est pas limitrophe, alors que l'EXPECTED affirme que la Basse-Saxe est limitrophe de la Rhénanie-du-Nord-Westphalie.</t>
+          <t>La réponse attendue dit que la Basse-Saxe est limitrophe de la Rhénanie-du-Nord-Westphalie, mais l’actuelle indique que la géométrie est introuvable et conclut implicitement que c’est non.</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="K104" t="n">
-        <v>0</v>
+        <v>-0.1224</v>
       </c>
       <c r="L104" t="n">
-        <v>0</v>
+        <v>-0.0618</v>
       </c>
     </row>
     <row r="105">
@@ -5858,33 +5859,33 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Non. Berlin n’est pas entièrement entourée par le Brandebourg d’après ce résultat, car Berlin est associée à deux villes de niveau City : Neuenhagen bei Berlin et Schöneiche bei Berlin.</t>
+          <t>Oui. Berlin a des localités correspondantes à Schöneiche bei Berlin et Neuenhagen bei Berlin, et ces lieux se trouvent dans la hiérarchie jusqu’en Allemagne, le Bundesstaat.</t>
         </is>
       </c>
       <c r="F105" t="n">
-        <v>6.076</v>
+        <v>5.5</v>
       </c>
       <c r="G105" t="n">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>L’ACTUEL répond « Non » et indique que Berlin n’est pas entièrement entourée par le Brandebourg, contrairement à « Oui » dans l’EXPECTED.</t>
+          <t>L’ACTUAL confirme bien que Berlin est entourée par le Brandebourg. Elle ajoute toutefois des détails supplémentaires non nécessaires (exemples de localités) mais sans contredire l’EXPECTED.</t>
         </is>
       </c>
       <c r="J105" t="n">
-        <v>0</v>
+        <v>0.1306</v>
       </c>
       <c r="K105" t="n">
-        <v>0</v>
+        <v>0.3052</v>
       </c>
       <c r="L105" t="n">
-        <v>0</v>
+        <v>0.2151</v>
       </c>
     </row>
     <row r="106">
@@ -5910,11 +5911,11 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Oui, Münster se trouve au nord de Dortmund. Dortmund est une ville, et Münster est une ville située dans la direction nord de Dortmund.</t>
+          <t>Oui. Münster se trouve au nord de Dortmund.</t>
         </is>
       </c>
       <c r="F106" t="n">
-        <v>9.815</v>
+        <v>5.252</v>
       </c>
       <c r="G106" t="n">
         <v>1</v>
@@ -5926,17 +5927,17 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>L’ACTUAL confirme clairement que Münster se trouve au nord de Dortmund, ce qui correspond à l’EXPECTED (avec une précision supplémentaire).</t>
+          <t>L’information attendue est présente : Münster se trouve au nord de Dortmund. La réponse est identique à l’attendu.</t>
         </is>
       </c>
       <c r="J106" t="n">
-        <v>0</v>
+        <v>0.8275</v>
       </c>
       <c r="K106" t="n">
-        <v>0</v>
+        <v>0.8275</v>
       </c>
       <c r="L106" t="n">
-        <v>0</v>
+        <v>0.8278</v>
       </c>
     </row>
     <row r="107">
@@ -5962,11 +5963,11 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Greven, une ville, se trouve juste au nord de Münster, une ville.</t>
+          <t>Greven se trouve juste au nord de Münster. Greven est une ville, située dans le district, dans le district administratif, dans le Land, en Allemagne.</t>
         </is>
       </c>
       <c r="F107" t="n">
-        <v>5.734</v>
+        <v>9.558</v>
       </c>
       <c r="G107" t="n">
         <v>1</v>
@@ -5978,17 +5979,17 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>L’ACTUAL indique que Greven se trouve juste au nord de Münster, ce qui correspond exactement à l’EXPECTED.</t>
+          <t>L’ACTUELLE mentionne bien que Greven se trouve juste au nord de Münster, ce qui correspond à l’EXPECTED. Le reste est un ajout de contexte sans contredire l’information demandée.</t>
         </is>
       </c>
       <c r="J107" t="n">
-        <v>0</v>
+        <v>0.2427</v>
       </c>
       <c r="K107" t="n">
-        <v>0</v>
+        <v>0.5677</v>
       </c>
       <c r="L107" t="n">
-        <v>0</v>
+        <v>0.3937</v>
       </c>
     </row>
     <row r="108">
@@ -6014,11 +6015,12 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Oui, Leipzig se trouve au nord-est d’Erfurt, toutes deux étant des villes.</t>
+          <t xml:space="preserve">Oui, Leipzig se trouve au nord-est d’Erfurt, donc pas directement à l’est.
+</t>
         </is>
       </c>
       <c r="F108" t="n">
-        <v>7.686</v>
+        <v>15.863</v>
       </c>
       <c r="G108" t="n">
         <v>1</v>
@@ -6030,17 +6032,17 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>L’ACTUAL répond correctement que Leipzig est située au nord-est d’Erfurt (donc bien à l’est), comme attendu. L’ajout 'toutes deux étant des villes' n’est pas contradictoire.</t>
+          <t>L’ACTUAL indique que Leipzig est au nord-est d’Erfurt, ce qui implique bien qu’elle est à l’est d’Erfurt. La précision supplémentaire (“pas directement à l’est”) reste compatible avec l’EXPECTED.</t>
         </is>
       </c>
       <c r="J108" t="n">
-        <v>0</v>
+        <v>0.6262</v>
       </c>
       <c r="K108" t="n">
-        <v>0</v>
+        <v>0.855</v>
       </c>
       <c r="L108" t="n">
-        <v>0</v>
+        <v>0.7357</v>
       </c>
     </row>
     <row r="109">
@@ -6066,11 +6068,11 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>La distance entre la ville de Cologne et la ville de Bonn est de 6,63 km.</t>
+          <t>Cologne est une ville située dans le district de Cologne, dans le district administratif de Cologne, dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne. Bonn est une ville située dans le district de Bonn, dans le district administratif de Cologne, dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne. La distance entre Cologne et Bonn est de 6,63 km.</t>
         </is>
       </c>
       <c r="F109" t="n">
-        <v>20.112</v>
+        <v>14.27</v>
       </c>
       <c r="G109" t="n">
         <v>1</v>
@@ -6082,17 +6084,17 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>L’ACTUAL reprend exactement la même distance (6,63 km) entre Cologne et Bonn que l’EXPECTED.</t>
+          <t>L’ACTUAL indique clairement que la distance entre Cologne et Bonn est de 6,63 km, ce qui correspond à l’EXPECTED.</t>
         </is>
       </c>
       <c r="J109" t="n">
-        <v>0</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="K109" t="n">
-        <v>0</v>
+        <v>0.6491</v>
       </c>
       <c r="L109" t="n">
-        <v>0</v>
+        <v>0.2797</v>
       </c>
     </row>
     <row r="110">
@@ -6118,11 +6120,11 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Aucune géométrie n’a été trouvée.</t>
+          <t>Aucune géométrie n’a été trouvée pour cette requête.</t>
         </is>
       </c>
       <c r="F110" t="n">
-        <v>4.482</v>
+        <v>4.209</v>
       </c>
       <c r="G110" t="n">
         <v>0</v>
@@ -6134,17 +6136,17 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>La réponse fournie ne donne aucune distance entre Hanovre et Brunswick.</t>
+          <t>L’ACTUAL ne fournit aucune distance (message indiquant qu’aucune géométrie n’a été trouvée), donc l’information attendue (34,92 km) est absente.</t>
         </is>
       </c>
       <c r="J110" t="n">
-        <v>0</v>
+        <v>-0.0461</v>
       </c>
       <c r="K110" t="n">
-        <v>0</v>
+        <v>-0.0803</v>
       </c>
       <c r="L110" t="n">
-        <v>0</v>
+        <v>-0.0618</v>
       </c>
     </row>
     <row r="111">
@@ -6170,33 +6172,33 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Aucune géométrie n’a été trouvée pour la Hesse et la Thuringe.</t>
+          <t>La Hesse et la Thuringe sont toutes deux des Bundesländer en Allemagne. D’après les données fournies, la Hesse est située en Allemagne avec une distance indiquée de 0,0 km, tandis que la Thuringe est également située en Allemagne.</t>
         </is>
       </c>
       <c r="F111" t="n">
-        <v>4.803</v>
+        <v>11.348</v>
       </c>
       <c r="G111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>L’ACTUEL ne fournit aucune distance, alors que l’ATTENDU indique 0,0 km.</t>
+          <t>L’ACTUAL mentionne que la distance entre la Hesse et la Thuringe est de 0,0 km, ce qui correspond à l’EXPECTED (les Länder sont aussi correctement identifiés comme Bundesländer).</t>
         </is>
       </c>
       <c r="J111" t="n">
-        <v>0</v>
+        <v>0.2434</v>
       </c>
       <c r="K111" t="n">
-        <v>0</v>
+        <v>0.3275</v>
       </c>
       <c r="L111" t="n">
-        <v>0</v>
+        <v>0.2857</v>
       </c>
     </row>
     <row r="112">
@@ -6222,11 +6224,11 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Les trois districts les plus proches du district de Miesbach sont, par ordre, le district de Bad Tölz-Wolfratshausen, le district de Rosenheim et le district de München.</t>
+          <t>Les trois districts les plus proches de Miesbach sont München, Bad Tölz-Wolfratshausen et Rosenheim. Miesbach est un district en Bavière, en Allemagne, et ces trois districts sont également des districts en Bavière, en Allemagne.</t>
         </is>
       </c>
       <c r="F112" t="n">
-        <v>4.699</v>
+        <v>4.366</v>
       </c>
       <c r="G112" t="n">
         <v>1</v>
@@ -6238,17 +6240,17 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Les trois districts les plus proches sont identifiés correctement : Bad Tölz-Wolfratshausen, Rosenheim et Munich (München). L’ordre diffère, mais le contenu correspond à l’attendu.</t>
+          <t>Les trois districts listés dans l’ACTUAL (München, Bad Tölz-Wolfratshausen, Rosenheim) correspondent aux trois attendus (Munich, Bad Tölz-Wolfratshausen, Rosenheim). Le reste du texte est additif et correct.</t>
         </is>
       </c>
       <c r="J112" t="n">
-        <v>0</v>
+        <v>0.5098</v>
       </c>
       <c r="K112" t="n">
-        <v>0</v>
+        <v>0.7933</v>
       </c>
       <c r="L112" t="n">
-        <v>0</v>
+        <v>0.6437</v>
       </c>
     </row>
     <row r="113">
@@ -6274,11 +6276,11 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Les districts limitrophes du Kreis de Warendorf sont les Kreise de Gütersloh, Hamm, Münster, Steinfurt, Osnabrück, Coesfeld et Soest.</t>
+          <t>Les districts limitrophes du district de Warendorf sont Gütersloh, Steinfurt, Soest, Coesfeld, Osnabrück, Münster et Hamm. Warendorf est un district dans le Land de Rhénanie-du-Nord-Westphalie en Allemagne.</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>4.757</v>
+        <v>4.467</v>
       </c>
       <c r="G113" t="n">
         <v>1</v>
@@ -6290,17 +6292,17 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Les districts limitrophes mentionnés dans l’ACTUAL sont exactement les mêmes que ceux de l’EXPECTED (Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld, Soest).</t>
+          <t>L’ACTUAL liste exactement les mêmes districts limitrophes que l’EXPECTED (Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld, Soest). L’information supplémentaire sur le Land est correcte et n’affecte pas la correspondance.</t>
         </is>
       </c>
       <c r="J113" t="n">
-        <v>0</v>
+        <v>0.407</v>
       </c>
       <c r="K113" t="n">
-        <v>0</v>
+        <v>0.6821</v>
       </c>
       <c r="L113" t="n">
-        <v>0</v>
+        <v>0.5369</v>
       </c>
     </row>
     <row r="114">
@@ -6326,11 +6328,11 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Les communes administratives limitrophes de la commune administrative de Leezen sont, dans le Kreis concerné, les communes administratives d’Auenland Südholstein, Wahlstedt, Itzstedt, Buchholz (Forstgutsbez.), Kisdorf, Bad Oldesloe-Land, Trave-Land, Boostedt-Rickling et Bad Segeberg.</t>
+          <t>Les communes administratives limitrophes de la commune administrative de Leezen sont Bad Oldesloe-Land, Trave-Land, Boostedt-Rickling, Auenland Südholstein, Wahlstedt, Kisdorf, Bad Segeberg, Itzstedt et Buchholz (Forstgutsbez.). Leezen est une commune administrative située dans le Kreis, dans le Bundesland et dans le Bundesstaat Allemagne.</t>
         </is>
       </c>
       <c r="F114" t="n">
-        <v>4.693</v>
+        <v>4.12</v>
       </c>
       <c r="G114" t="n">
         <v>1</v>
@@ -6342,17 +6344,17 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Les communes listées dans l’ACTUAL correspondent exactement aux communes attendues (Auenland Südholstein, Kisdorf, Bad Oldesloe-Land, Trave-Land, Wahlstedt, Itzstedt, Bad Segeberg, Boostedt-Rickling, Buchholz). L’ACTUAL ajoute simplement une précision de cadre (Kreis concerné), ce qui ne retire aucune information requise.</t>
+          <t>Toutes les communes limitrophes attendues (Auenland Südholstein, Kisdorf, Bad Oldesloe-Land, Trave-Land, Wahlstedt, Itzstedt, Bad Segeberg, Boostedt-Rickling et Buchholz (Forstgutsbez.)) sont présentes dans la réponse. Information supplémentaire ajoutée sans contradiction.</t>
         </is>
       </c>
       <c r="J114" t="n">
-        <v>0</v>
+        <v>0.5562</v>
       </c>
       <c r="K114" t="n">
-        <v>0</v>
+        <v>0.7181999999999999</v>
       </c>
       <c r="L114" t="n">
-        <v>0</v>
+        <v>0.635</v>
       </c>
     </row>
     <row r="115">
@@ -6378,14 +6380,14 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Aucune géométrie n’a été trouvée pour cette question.</t>
+          <t>La Moyenne-Franconie, qui est un district administratif du Bundesland Bavière en Allemagne, est entourée par l’Oberpfalz, l’Oberbayern, la Schwaben, l’Oberfranken, l’Unterfranken et Stuttgart.</t>
         </is>
       </c>
       <c r="F115" t="n">
-        <v>4.174</v>
+        <v>4.991</v>
       </c>
       <c r="G115" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
@@ -6394,17 +6396,17 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>L’ACTUAL ne fournit aucune information permettant d’identifier les districts administratifs entourant la Moyenne-Franconie.</t>
+          <t>L’ACTUAL réponse ne correspond pas à l’EXPECTED : elle décrit que la Moyenne-Franconie est entourée par plusieurs districts (Oberpfalz, Oberbayern, Schwaben, Oberfranken, Unterfranken, Stuttgart), alors que l’EXPECTED indique seulement qu’elle est entourée par la Bavière (Land). La partie concernant l’appartenance à la Bavière est correcte, mais l’information attendue sur le voisinage est incomplète/incorrecte.</t>
         </is>
       </c>
       <c r="J115" t="n">
-        <v>0</v>
+        <v>0.2568</v>
       </c>
       <c r="K115" t="n">
-        <v>0</v>
+        <v>0.6972</v>
       </c>
       <c r="L115" t="n">
-        <v>0</v>
+        <v>0.4557</v>
       </c>
     </row>
     <row r="116">
@@ -6430,11 +6432,11 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Aucune géométrie n’a été trouvée pour cette question ; aucun Land situé au nord de la Thuringe n’est indiqué.</t>
+          <t>Aucun géométrie trouvée.</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>4.645</v>
+        <v>4.478</v>
       </c>
       <c r="G116" t="n">
         <v>0</v>
@@ -6446,17 +6448,17 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>L’ACTUAL ne mentionne aucun des Länder attendus, donc l’information demandée est manquante.</t>
+          <t>La réponse attendue liste des Länder au nord de la Thuringe, mais la réponse fournie indique « Aucun géométrie trouvée » et ne contient aucune information pertinente.</t>
         </is>
       </c>
       <c r="J116" t="n">
-        <v>0</v>
+        <v>-0.0118</v>
       </c>
       <c r="K116" t="n">
-        <v>0</v>
+        <v>-0.2719</v>
       </c>
       <c r="L116" t="n">
-        <v>0</v>
+        <v>-0.1509</v>
       </c>
     </row>
     <row r="117">
@@ -6482,11 +6484,11 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Les districts situés à l’ouest du district de Münster sont les districts de Kleve et de Borken. Münster est un district, et Kleve et Borken sont également des districts.</t>
+          <t>Les districts situés à l’ouest de Münster sont Kleve et Borken. Münster, Kleve et Borken sont des districts, situés dans le district administratif de Münster, dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne.</t>
         </is>
       </c>
       <c r="F117" t="n">
-        <v>65.94</v>
+        <v>37.769</v>
       </c>
       <c r="G117" t="n">
         <v>1</v>
@@ -6498,17 +6500,17 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>L’ACTUAL mentionne clairement que les districts à l’ouest de Münster sont Kleve et Borken, ce qui correspond exactement à l’EXPECTED.</t>
+          <t>L'ACTUAL mentionne correctement que les districts à l'ouest de Münster sont Kleve et Borken, ce qui correspond à l'EXPECTED.</t>
         </is>
       </c>
       <c r="J117" t="n">
-        <v>0</v>
+        <v>0.1426</v>
       </c>
       <c r="K117" t="n">
-        <v>0</v>
+        <v>0.4281</v>
       </c>
       <c r="L117" t="n">
-        <v>0</v>
+        <v>0.2763</v>
       </c>
     </row>
     <row r="118">
@@ -6534,23 +6536,23 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Les communautés administratives situées au nord de la communauté administrative de Kiel sont Geltinger Bucht, Dänischenhagen, Altenholz, Kiel et Kappeln. Toutes sont des communautés administratives.</t>
+          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="F118" t="n">
-        <v>54.295</v>
+        <v>23.164</v>
       </c>
       <c r="G118" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Les communautés attendues (Altenholz, Dänischenhagen, Kappeln, Geltinger Bucht) sont toutes présentes dans l’actual. En revanche, l’actual ajoute aussi 'Kiel', qui ne devrait pas faire partie des communautés situées au nord de Kiel.</t>
+          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="J118" t="n">
@@ -6586,23 +6588,23 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Autour du district de Göttingen, les districts indiqués sont Northeim, Kassel, Goslar, Nordhausen, Werra-Meißner-Kreis, Eichsfeld, Kassel et Harz.</t>
+          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="F119" t="n">
-        <v>3215.127</v>
+        <v>26.84</v>
       </c>
       <c r="G119" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Les districts listés dans l’ACTUAL correspondent exactement à ceux de l’EXPECTED (Harz, Northeim, Goslar, Kassel, Eichsfeld, Werra-Meißner-Kreis, Nordhausen), avec une répétition de Kassel mais sans omission.</t>
+          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="J119" t="n">
@@ -6638,23 +6640,23 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Les villes situées dans un rayon de 5 km autour d’Aachen, qui est une ville, sont Würselen, Alsdorf, Roetgen, Herzogenrath, Eschweiler, Hürtgenwald, Stolberg (Rhld.) et Simmerath, toutes des villes.</t>
+          <t>ERROR: 500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="F120" t="n">
-        <v>39.56</v>
+        <v>23.215</v>
       </c>
       <c r="G120" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>L’ACTUAL liste exactement toutes les villes attendues (Alsdorf, Simmerath, Würselen, Hürtgenwald, Roetgen, Herzogenrath, Eschweiler, Stolberg (Rhld.)), avec en plus la mention du nom de la ville d’origine et un contexte, sans omission.</t>
+          <t>500 Server Error: Internal Server Error for url: http://localhost:8000/api/chat/</t>
         </is>
       </c>
       <c r="J120" t="n">
@@ -6690,14 +6692,15 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Autour de Munich, les villes situées dans un rayon de moins de 2 km sont : Krailling, Hebertshausen, Putzbrunn, Gräfelfing, Pullach i.Isartal, Bergkirchen, Ottobrunn, Haar, Gröbenzell, Vaterstetten, Karlsfeld, Planegg, Puchheim, Grünwalder Forst, Neubiberg, Oberschleißheim, Germering, Perlacher Forst, Dachau, Feldkirchen, Olching, Unterföhring, Unterhaching, Garching b.München, Ismaning, Neuried, Hohenbrunn, Forstenrieder Park, Aschheim, Grünwald et Grasbrunn. Munich est une ville.</t>
+          <t>Autour de München, les villes et lieux suivants sont indiqués comme cibles : Grasbrunn, Ismaning, Karlsfeld, Gräfelfing, Olching, Hebertshausen, Grünwalder Forst, Neuried, Neubiberg, Putzbrunn, Grünwald, Garching b.München, Perlacher Forst, Vaterstetten, Bergkirchen, Hohenbrunn, Unterföhring, Germering, Oberschleißheim, Krailling, Unterhaching, Gröbenzell, Planegg, Haar, Aschheim, Dachau, Feldkirchen, Pullach i.Isartal, Ottobrunn, Forstenrieder Park et Puchheim.
+München est une ville située en Allemagne.</t>
         </is>
       </c>
       <c r="F121" t="n">
-        <v>65.77200000000001</v>
+        <v>42.025</v>
       </c>
       <c r="G121" t="n">
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
@@ -6706,17 +6709,17 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>L’ACTUAL contient la plupart des villes attendues (ex. Forstenrieder Park, Grünwald, Feldkirchen, Aschheim, Haar, Unterhaching, Pullach i.Isartal, Bergkirchen, Neuried, Germering, Olching, Garching b.München, Planegg, Ismaning, Puchheim, Unterföhring, Gröbenzell, Neubiberg, Oberschleißheim, Putzbrunn, Perlacher Forst, Gräfelfing, Karlsfeld). En revanche, il manque plusieurs éléments attendus (Grünwalder Forst est présent mais 'Grünwald' seul ok; mais absence de 'Putzbrunn' est présente, cependant absence de 'Bergkirchen' présent; manquent : 'Haar' présent; principaux manquants : 'Feldkirchen' présent; manque 'Unterföhring' présent; il manque surtout 'Putzbrunn' présent. Il manque toutefois 'Haar' etc. La différence majeure est qu’il manque 'Grünwalder Forst' n’est pas exactement 'Grünwald'—et surtout l’ACTUAL remplace/ajoute des villes supplémentaires (Krailling, Hebertshausen, Ottobrunn, Vaterstetten, Dachau, Hohenbrunn, Grasbrunn) et il manque au moins 'Forstenrieder Park' présent. Globalement le recouvrement est incomplet sur la liste attendue.</t>
+          <t>L’ACTUAL liste la majorité des villes attendues (18/22) : Forstenrieder Park, Grünwald, Feldkirchen, Aschheim, Haar, Unterhaching, Pullach i.Isartal, Bergkirchen, Neuried, Germering, Olching, Garching b.München, Planegg, Ismaning, Puchheim, Unterföhring, Gröbenzell, Neubiberg, Oberschleißheim, Putzbrunn, Perlacher Forst, Gräfelfing. Il manque Karlsfeld et Oberschleißheim est présent, mais l’ACTUAL n’inclut pas clairement 'Karlsfeld' (présent dans ACTUAL) ; en fait, il manque surtout 'Gräfelfing' est présent. Les seules omissions notables par rapport à l’EXPECTED sont 'Karlsfeld' (présent) et 'Unterföhring' (présent). En réalité il manque 'Grünwald' présent, 'Feldkirchen' présent. La différence principale est l’absence de 'Neubiberg' ? présent. Conclusion: l’ACTUAL contient presque tout mais inclut aussi d’autres lieux; le score reste inférieur car la comparaison stricte montre des écarts (ex: 'Karlsfeld' est bien présent mais l’EXPECTED inclut 'Gräfelfing' et 'Karlsfeld' sans mention d’autres comme Dachau).</t>
         </is>
       </c>
       <c r="J121" t="n">
-        <v>0</v>
+        <v>0.5944</v>
       </c>
       <c r="K121" t="n">
-        <v>0</v>
+        <v>0.6891</v>
       </c>
       <c r="L121" t="n">
-        <v>0</v>
+        <v>0.6414</v>
       </c>
     </row>
     <row r="122">
@@ -6730,21 +6733,21 @@
       <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="n">
-        <v>42.133</v>
+        <v>10.546</v>
       </c>
       <c r="G122" t="n">
-        <v>0.7086</v>
+        <v>0.6722</v>
       </c>
       <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr"/>
       <c r="J122" t="n">
-        <v>0</v>
+        <v>0.395</v>
       </c>
       <c r="K122" t="n">
-        <v>0</v>
+        <v>0.5057</v>
       </c>
       <c r="L122" t="n">
-        <v>0</v>
+        <v>0.4429</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update gpt5.4-mini Test results
</commit_message>
<xml_diff>
--- a/Model_Testing/test_results_gpt-5.4-mini.xlsx
+++ b/Model_Testing/test_results_gpt-5.4-mini.xlsx
@@ -501,11 +501,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Münster is a city in the administrative community Münster, in the district Münster, in the administrative district Münster, in the Federal State of Nordrhein-Westfalen, in Germany.</t>
+          <t>Münster is a city in the administrative community of Münster, in the district of Münster, in the administrative district of Münster, in the Federal State of Nordrhein-Westfalen, in Germany.</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>11.951</v>
+        <v>9.044</v>
       </c>
       <c r="G2" t="n">
         <v>0.5</v>
@@ -517,17 +517,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>The actual answer correctly identifies the Münster in Nordrhein-Westfalen, but it omits the additional Münster in Bavaria (Rain, Donau-Ries, Schwaben).</t>
+          <t>The actual answer correctly identifies one Münster (in Nordrhein-Westfalen) but omits the second Münster located in Bayern described in the expected answer.</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.5757</v>
+        <v>0.5955</v>
       </c>
       <c r="K2" t="n">
-        <v>0.3775</v>
+        <v>0.4074</v>
       </c>
       <c r="L2" t="n">
-        <v>0.4729</v>
+        <v>0.4982</v>
       </c>
     </row>
     <row r="3">
@@ -553,33 +553,33 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Cologne is the city of Köln. It is in the administrative community of Köln, in the district of Köln, in the administrative district of Köln, in the federal state of Nordrhein-Westfalen, in Germany.</t>
+          <t>No geometry found for the city of Cologne.</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>5.953</v>
+        <v>4.562</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>The actual answer states that Cologne/Köln is located in Nordrhein-Westfalen and includes the administrative district Köln, matching the expected information (with some extra administrative detail and Germany).</t>
+          <t>The actual answer contains no information about Cologne’s administrative district or federal state, and provides no location details.</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0.6107</v>
+        <v>0.3456</v>
       </c>
       <c r="K3" t="n">
-        <v>0.6967</v>
+        <v>0.2574</v>
       </c>
       <c r="L3" t="n">
-        <v>0.6535</v>
+        <v>0.3016</v>
       </c>
     </row>
     <row r="4">
@@ -605,11 +605,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Eisenhüttenstadt is located in the district of Oder-Spree, in the Federal State of Brandenburg, in Germany.</t>
+          <t>The administrative community of Eisenhüttenstadt is located in the district of Oder-Spree, in the FederalState of Brandenburg, in Germany.</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>7.432</v>
+        <v>4.097</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
@@ -621,17 +621,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>The actual answer includes the expected district (Oder-Spree) and federal state (Brandenburg). It also correctly adds that it is in Germany.</t>
+          <t>The ACTUAL answer includes all information from the EXPECTED answer: district of Oder-Spree and federal state of Brandenburg; it additionally specifies it is in Germany.</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.8300999999999999</v>
+        <v>0.8407</v>
       </c>
       <c r="K4" t="n">
-        <v>0.7837</v>
+        <v>0.9155</v>
       </c>
       <c r="L4" t="n">
-        <v>0.8069</v>
+        <v>0.8777</v>
       </c>
     </row>
     <row r="5">
@@ -657,11 +657,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>The administrative community of Esens is located in the district of Wittmund, in the federal state of Niedersachsen, in Germany.</t>
+          <t>Esens is an administrative community in the district of Wittmund, in the federal state of Niedersachsen, in Germany.</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>6.385</v>
+        <v>4.248</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
@@ -673,17 +673,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>The actual answer states Esens is in the district of Wittmund and in the federal state of Niedersachsen (Lower Saxony), matching the expected information.</t>
+          <t>The actual answer states that Esens is in the district of Wittmund and in the federal state of Niedersachsen (Lower Saxony), matching the expected information.</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.6778</v>
+        <v>0.5322</v>
       </c>
       <c r="K5" t="n">
-        <v>0.8022</v>
+        <v>0.6012</v>
       </c>
       <c r="L5" t="n">
-        <v>0.7388</v>
+        <v>0.5669</v>
       </c>
     </row>
     <row r="6">
@@ -709,11 +709,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>The district of Gießen is located in the administrative district of Gießen, in the FederalState of Hessen, in Germany.</t>
+          <t>The district of Gießen is located in Gießen, in the federal state of Hessen, in Germany.</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>5.471</v>
+        <v>4.203</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
@@ -725,17 +725,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>The actual answer states that the district of Gießen is in the Federal State of Hessen, matching the expected answer. Additional correct details are provided (administrative district of Gießen, Germany).</t>
+          <t>The actual answer states that the district of Gießen is in the federal state of Hessen, matching the expected answer. Additional details (location in Gießen and Germany) are correct and not contradictory.</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0.603</v>
+        <v>0.7274</v>
       </c>
       <c r="K6" t="n">
-        <v>0.7653</v>
+        <v>0.869</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6819</v>
+        <v>0.7965</v>
       </c>
     </row>
     <row r="7">
@@ -761,11 +761,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>The district of Nordsachsen is located in Sachsen, Germany.</t>
+          <t>Nordsachsen is a district in the federal state of Sachsen in Germany.</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>5.782</v>
+        <v>3.978</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
@@ -777,17 +777,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>The actual answer states that Nordsachsen is located in Sachsen, Germany, which matches the expected information that it is in the federal state of Sachsen.</t>
+          <t>The actual answer states that Nordsachsen is a district in the federal state of Sachsen in Germany, which includes all information from the expected answer (located in Sachsen).</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0.847</v>
+        <v>0.7227</v>
       </c>
       <c r="K7" t="n">
-        <v>0.78</v>
+        <v>0.7343</v>
       </c>
       <c r="L7" t="n">
-        <v>0.8133</v>
+        <v>0.7289</v>
       </c>
     </row>
     <row r="8">
@@ -813,11 +813,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Freiburg is located in Baden-Württemberg, which is a FederalState in Germany, a State.</t>
+          <t>Freiburg is an administrative district located in Baden-Württemberg, Germany.</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.987</v>
+        <v>4.585</v>
       </c>
       <c r="G8" t="n">
         <v>1</v>
@@ -829,17 +829,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>The actual answer states that Freiburg is located in Baden-Württemberg, matching the expected federal state location information.</t>
+          <t>The ACTUAL answer states that Freiburg is an administrative district located in Baden-Württemberg, Germany, which includes the expected information that it is in the federal state Baden-Württemberg.</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0.3455</v>
+        <v>0.6313</v>
       </c>
       <c r="K8" t="n">
-        <v>0.4992</v>
+        <v>0.6105</v>
       </c>
       <c r="L8" t="n">
-        <v>0.4205</v>
+        <v>0.6214</v>
       </c>
     </row>
     <row r="9">
@@ -865,11 +865,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Oberfranken is an AdministrativeDistrict in Bayern, which is a FederalState, in Germany, which is a State.</t>
+          <t>Oberfranken is an AdministrativeDistrict in the FederalState of Bayern in Germany.</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>5.431</v>
+        <v>3.931</v>
       </c>
       <c r="G9" t="n">
         <v>1</v>
@@ -881,17 +881,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>The actual answer states that Oberfranken is in Bayern, matching the expected that it is located in the federal state of Bayern (with correct additional context).</t>
+          <t>The actual answer states that Oberfranken (the administrative district) is in the FederalState of Bayern, matching the expected information.</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.2045</v>
+        <v>0.4005</v>
       </c>
       <c r="K9" t="n">
-        <v>0.4188</v>
+        <v>0.5638</v>
       </c>
       <c r="L9" t="n">
-        <v>0.307</v>
+        <v>0.4799</v>
       </c>
     </row>
     <row r="10">
@@ -921,10 +921,10 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>8.478</v>
+        <v>5.249</v>
       </c>
       <c r="G10" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -933,7 +933,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>The actual answer only states that Sachsen is a FederalState in Germany, but it does not provide the required centroid location/coordinates from the expected answer.</t>
+          <t>The actual answer does not provide the expected centroid coordinates (POINT (13.348518008906732 51.05230081187263)) or the specific location information requested.</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -969,14 +969,14 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Saarland is a Federal State in Germany.</t>
+          <t>Saarland is a Federal State located in Germany.</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>5.817</v>
+        <v>4.582</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -985,17 +985,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>The actual answer states that Saarland is a federal state in Germany but does not provide the required centroid coordinates or the specific location details from the expected answer.</t>
+          <t>The actual answer only states that Saarland is a federal state in Germany, but it does not include the required centroid coordinates (POINT (6.953360955673903 49.38438040655551)).</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0.3194</v>
+        <v>0.3773</v>
       </c>
       <c r="K11" t="n">
-        <v>-0.2154</v>
+        <v>-0.1747</v>
       </c>
       <c r="L11" t="n">
-        <v>0.013</v>
+        <v>0.0608</v>
       </c>
     </row>
     <row r="12">
@@ -1021,11 +1021,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>The district of Coesfeld includes the cities of Rosendahl, Havixbeck, Senden, Billerbeck, Ascheberg, Dülmen, Nottuln, Coesfeld, Nordkirchen, Lüdinghausen, and Olfen. The district of Coesfeld is in the administrative district of Münster, in the federal state of North Rhine-Westphalia, in Germany.</t>
+          <t>The district of Coesfeld includes the cities of Rosendahl, Havixbeck, Senden, Billerbeck, Ascheberg, Dülmen, Nottuln, Coesfeld, Nordkirchen, Lüdinghausen, and Olfen. Coesfeld is a district in the administrative district of Münster, in the federal state of North Rhine-Westphalia, in Germany.</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>6.318</v>
+        <v>4.268</v>
       </c>
       <c r="G12" t="n">
         <v>1</v>
@@ -1037,17 +1037,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>All expected cities (Coesfeld, Olfen, Senden, Nottuln, Havixbeck, Nordkirchen, Billerbeck, Lüdinghausen, Rosendahl, Dülmen, Ascheberg) are included in the actual answer. Additional correct information about Münster and North Rhine-Westphalia is also provided.</t>
+          <t>All expected cities (Coesfeld, Olfen, Senden, Nottuln, Havixbeck, Nordkirchen, Billerbeck, Lüdinghausen, Rosendahl, Dülmen, Ascheberg) are included in the actual answer, with correct listing and no missing items.</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0.5621</v>
+        <v>0.5462</v>
       </c>
       <c r="K12" t="n">
-        <v>0.7886</v>
+        <v>0.7863</v>
       </c>
       <c r="L12" t="n">
-        <v>0.6705</v>
+        <v>0.6607</v>
       </c>
     </row>
     <row r="13">
@@ -1073,11 +1073,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>The administrative district of Oberbayern includes the districts of Dachau, Miesbach, Garmisch-Partenkirchen, Landsberg am Lech, Rosenheim, Eichstätt, Ingolstadt, Fürstenfeldbruck, München, Berchtesgadener Land, Bad Tölz-Wolfratshausen, Ebersberg, Pfaffenhofen a.d.Ilm, Traunstein, Neuburg-Schrobenhausen, Mühldorf a.Inn, Starnberg, Altötting, Weilheim-Schongau, Freising, and Erding. München and Rosenheim appear twice in the provided matches, and there are 23 matches in total. Oberbayern is an AdministrativeDistrict in the FederalState of Bayern in Germany.</t>
+          <t>The administrative district of Oberbayern includes the districts Dachau, Miesbach, Garmisch-Partenkirchen, Landsberg am Lech, Rosenheim, Eichstätt, Ingolstadt, Fürstenfeldbruck, München, Berchtesgadener Land, Bad Tölz-Wolfratshausen, Ebersberg, Pfaffenhofen a.d.Ilm, Traunstein, Neuburg-Schrobenhausen, Mühldorf a.Inn, Starnberg, Altötting, Weilheim-Schongau, Freising, and Erding, as well as two districts named München and two districts named Rosenheim. Oberbayern is an administrative district in the federal state of Bayern in Germany.</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>5.721</v>
+        <v>4.539</v>
       </c>
       <c r="G13" t="n">
         <v>1</v>
@@ -1089,17 +1089,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>All 20 districts listed in the expected answer are included in the actual answer (including Fürstenfeldbruck, Erding, München, Freising, Ingolstadt, Mühldorf a.Inn, Rosenheim, Garmisch-Partenkirchen, Eichstätt, Landsberg am Lech, Weilheim-Schongau, Dachau, Altötting, Neuburg-Schrobenhausen, Pfaffenhofen a.d.Ilm, Ebersberg, Bad Tölz-Wolfratshausen, Traunstein, Miesbach, Starnberg, Berchtesgadener Land). The additional note about München and Rosenheim appearing twice is also present.</t>
+          <t>All districts listed in the expected answer are present in the actual answer, including the note about multiple districts named München and Rosenheim. The actual answer also includes an additional correct contextual statement.</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>0.6115</v>
+        <v>0.7186</v>
       </c>
       <c r="K13" t="n">
-        <v>0.6984</v>
+        <v>0.7405</v>
       </c>
       <c r="L13" t="n">
-        <v>0.6546999999999999</v>
+        <v>0.7299</v>
       </c>
     </row>
     <row r="14">
@@ -1125,33 +1125,33 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>The federal state of Hessen includes the following districts: Limburg-Weilburg, Vogelsbergkreis, Lahn-Dill-Kreis, Marburg-Biedenkopf, Gießen, Hersfeld-Rotenburg, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis, Kassel, Schwalm-Eder-Kreis, Main-Kinzig-Kreis, Darmstadt, Wiesbaden, Rheingau-Taunus-Kreis, Bergstraße, Darmstadt-Dieburg, Frankfurt am Main, Offenbach, Main-Taunus-Kreis, Odenwaldkreis, Offenbach am Main, Hochtaunuskreis, Groß-Gerau, and Wetteraukreis. Hessen is a federal state in Germany, and Germany is a state.</t>
+          <t>Hessen is a Federal State in Germany, and the districts belonging to it are Limburg-Weilburg, Vogelsbergkreis, Lahn-Dill-Kreis, Marburg-Biedenkopf, Gießen, Hersfeld-Rotenburg, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis, Kassel, Schwalm-Eder-Kreis, Main-Kinzig-Kreis, Darmstadt, Wiesbaden, Rheingau-Taunus-Kreis, Bergstraße, Darmstadt-Dieburg, Frankfurt am Main, Offenbach, Main-Taunus-Kreis, Odenwaldkreis, Offenbach am Main, Hochtaunuskreis, Groß-Gerau, and Wetteraukreis.</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>6.585</v>
+        <v>4.388</v>
       </c>
       <c r="G14" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>The actual answer includes 25 of the 26 expected districts (missing only Rheingau-Taunus-Kreis? actually present; missing only one: it does not include Hochtaunuskreis? but Hochtaunuskreis is present; it misses one district: Offenbach? present. It misses 'Hochtaunuskreis' not; expected 'Hochtaunuskreis' is present. The missing district is 'Offenbach am Main'? present. The only difference is a duplicate 'Kassel' and the absence of 'Rheingau-Taunus-Kreis' is not—it's included. Therefore mismatch is likely none, but actual has exactly the same set except duplicates and one district missing: 'Limburg-Weilburg' included; all others included except 'Schwalm-Eder-Kreis' included. Actual list matches expected except it lacks 'Vogelsbergkreis'? included. So score slightly below 1 due to uncertainty from ordering/duplication.</t>
+          <t>The ACTUAL answer lists all districts from the EXPECTED answer (including all 24 named districts), with no missing entries. A duplicate 'Kassel' is present but does not affect correctness.</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>0.7037</v>
+        <v>0.7209</v>
       </c>
       <c r="K14" t="n">
-        <v>0.7419</v>
+        <v>0.7375</v>
       </c>
       <c r="L14" t="n">
-        <v>0.7231</v>
+        <v>0.7296</v>
       </c>
     </row>
     <row r="15">
@@ -1177,11 +1177,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>The district of Steinburg has the following administrative communities: Itzehoe-Land, Schenefeld, Wilstermarsch, Itzehoe, Horst-Herzhorn, Krempermarsch, Breitenburg, Glückstadt, Wilster, and Kellinghusen. These administrative communities are in the district of Steinburg, within the administrative district of Germany.</t>
+          <t>The district of Steinburg includes the administrative communities of Itzehoe-Land, Schenefeld, Wilstermarsch, Itzehoe, Horst-Herzhorn, Krempermarsch, Breitenburg, Glückstadt, Wilster, and Kellinghusen. Steinburg is a district in the federal state of Schleswig-Holstein in Germany.</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>6.849</v>
+        <v>4.182</v>
       </c>
       <c r="G15" t="n">
         <v>1</v>
@@ -1193,17 +1193,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>The actual answer lists all 10 administrative communities named in the expected answer: Wilster, Krempermarsch, Itzehoe-Land, Horst-Herzhorn, Breitenburg, Schenefeld, Wilstermarsch, Glückstadt, Kellinghusen, and Itzehoe.</t>
+          <t>The ACTUAL answer lists all 10 administrative communities from the EXPECTED answer (Wilster, Krempermarsch, Itzehoe-Land, Horst-Herzhorn, Breitenburg, Schenefeld, Wilstermarsch, Glückstadt, Kellinghusen, Itzehoe). Additional correct context about Steinburg is included.</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>0.6492</v>
+        <v>0.6703</v>
       </c>
       <c r="K15" t="n">
-        <v>0.768</v>
+        <v>0.8101</v>
       </c>
       <c r="L15" t="n">
-        <v>0.7076</v>
+        <v>0.7386</v>
       </c>
     </row>
     <row r="16">
@@ -1229,11 +1229,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>The district of Paderborn has 10 cities: Altenbeken, Hövelhof, Borchen, Delbrück, Paderborn, Büren, Bad Wünnenberg, Lichtenau, Salzkotten, and Bad Lippspringe. The district is in the administrative district of Detmold, in the Federal State of North Rhine-Westphalia, in Germany.</t>
+          <t>The district of Paderborn includes 10 cities: Altenbeken, Hövelhof, Borchen, Delbrück, Paderborn, Büren, Bad Wünnenberg, Lichtenau, Salzkotten, and Bad Lippspringe. Paderborn is a district in the administrative district of Detmold, in the federal state of North Rhine-Westphalia, in Germany.</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>5.811</v>
+        <v>4.1</v>
       </c>
       <c r="G16" t="n">
         <v>1</v>
@@ -1245,17 +1245,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>The actual answer lists the same 10 cities as the expected answer; additional administrative details are correct and do not affect completeness.</t>
+          <t>The ACTUAL answer lists the same 10 cities as the EXPECTED answer, and the extra sentence is additional correct information.</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>0.5075</v>
+        <v>0.502</v>
       </c>
       <c r="K16" t="n">
-        <v>0.7724</v>
+        <v>0.7693</v>
       </c>
       <c r="L16" t="n">
-        <v>0.6331</v>
+        <v>0.6286</v>
       </c>
     </row>
     <row r="17">
@@ -1281,11 +1281,11 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>No. Nothing no geometry found for the city of Dülmen, so no location hierarchy can be described from the provided information.</t>
+          <t>No, nothing no geometry found for the city of Dülmen in the district of Coesfeld.</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>9.564</v>
+        <v>4.748</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -1297,17 +1297,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>The actual answer states that it cannot determine or describe the location hierarchy and does not confirm that Dülmen lies within the district of Coesfeld.</t>
+          <t>The actual answer states that Dülmen does not lie within Coesfeld (or provides no supporting geometry), contradicting the expected confirmation that it does.</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>0.1651</v>
+        <v>0.394</v>
       </c>
       <c r="K17" t="n">
-        <v>0.3404</v>
+        <v>0.5127</v>
       </c>
       <c r="L17" t="n">
-        <v>0.25</v>
+        <v>0.4525</v>
       </c>
     </row>
     <row r="18">
@@ -1333,33 +1333,33 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Yes. Coesfeld is located in the administrative district of Münster. In the hierarchy, Coesfeld is a district in the administrative district of Münster, which is in the federal state of North Rhine-Westphalia, in Germany.</t>
+          <t>No, nothing was found. There is no geometry available to confirm that the district of Coesfeld is located in the administrative district of Münster.</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>5.451</v>
+        <v>4.04</v>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>The actual answer confirms that Coesfeld is located in the administrative district of Münster, matching the expected answer (with additional correct hierarchical context).</t>
+          <t>The actual answer states it could not find any information/geometry to confirm whether Coesfeld is in the administrative district of Münster, and it does not provide the expected confirmation.</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>0.4088</v>
+        <v>0.4683</v>
       </c>
       <c r="K18" t="n">
-        <v>0.6721</v>
+        <v>0.8161</v>
       </c>
       <c r="L18" t="n">
-        <v>0.5335</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="19">
@@ -1385,11 +1385,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Yes. Oberfranken is an AdministrativeDistrict and it is located in the FederalState Bayern, which is in Germany.</t>
+          <t>Yes. Oberfranken is an AdministrativeDistrict that belongs to the FederalState Bayern, and Bayern is in Germany, the State.</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>5.484</v>
+        <v>4.243</v>
       </c>
       <c r="G19" t="n">
         <v>1</v>
@@ -1401,17 +1401,17 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>The ACTUAL answer explicitly states that Oberfranken is located in the Federal State Bayern (Germany), which matches the EXPECTED answer.</t>
+          <t>The actual answer clearly states that Oberfranken belongs to the FederalState Bayern, matching the expected statement.</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>0.3467</v>
+        <v>0.3587</v>
       </c>
       <c r="K19" t="n">
-        <v>0.5291</v>
+        <v>0.5608</v>
       </c>
       <c r="L19" t="n">
-        <v>0.4349</v>
+        <v>0.4559</v>
       </c>
     </row>
     <row r="20">
@@ -1437,33 +1437,33 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Yes. The district of Steinfurt is located in the Federal State of Nordrhein-Westfalen, and Nordrhein-Westfalen is in Germany.</t>
+          <t>No. Nothing was found for the district of Steinfurt, so there is no information showing that it is located in the federal state of Nordrhein-Westfalen or any higher hierarchy level up to Germany.</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>6.126</v>
+        <v>4.66</v>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>The actual answer confirms that the district of Steinfurt is located in Nordrhein-Westfalen, matching the expected answer.</t>
+          <t>The expected answer states Steinfurt is in Nordrhein-Westfalen, but the actual answer denies finding any information and does not confirm the federal state.</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>0.6948</v>
+        <v>0.3679</v>
       </c>
       <c r="K20" t="n">
-        <v>0.7893</v>
+        <v>0.7198</v>
       </c>
       <c r="L20" t="n">
-        <v>0.7415</v>
+        <v>0.5309</v>
       </c>
     </row>
     <row r="21">
@@ -1489,11 +1489,11 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>No. The provided information only shows Bocholt matching Bocholt itself, so there is no indication that Bocholt is located within the district of Cloppenburg. The hierarchy shown here ends at Bocholt, and no district, administrative district, federal state, or Germany-related location is provided.</t>
+          <t>No. Nothing was found, so Bocholt is not shown as being located within the district of Cloppenburg.</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>6.264</v>
+        <v>4.116</v>
       </c>
       <c r="G21" t="n">
         <v>1</v>
@@ -1505,17 +1505,17 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Both expected and actual state that Bocholt is not located within the district of Cloppenburg. The actual response adds justification but does not contradict the expected claim.</t>
+          <t>Both expected and actual indicate that Bocholt is not located within the district of Cloppenburg; the actual answer adds a note about search results.</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>0.2232</v>
+        <v>0.6027</v>
       </c>
       <c r="K21" t="n">
-        <v>0.6372</v>
+        <v>0.8018</v>
       </c>
       <c r="L21" t="n">
-        <v>0.4111</v>
+        <v>0.6986</v>
       </c>
     </row>
     <row r="22">
@@ -1541,11 +1541,11 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Yes. Coesfeld touches Borken. Coesfeld is a district in the administrative district of Münster in the federal state of North Rhine-Westphalia in Germany, and Borken is a district in the administrative district of Münster in the federal state of North Rhine-Westphalia in Germany.</t>
+          <t>Yes. Coesfeld touches Borken. Coesfeld is a district in the administrative district of Münster in the federal state of North Rhine-Westphalia in Germany, and Borken is also a district in the administrative district of Münster in the federal state of North Rhine-Westphalia in Germany.</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5.924</v>
+        <v>4.718</v>
       </c>
       <c r="G22" t="n">
         <v>1</v>
@@ -1557,17 +1557,17 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>The actual answer states that Coesfeld touches Borken, matching the expected response. Additional details are correct and do not conflict.</t>
+          <t>The ACTUAL answer directly states that Coesfeld touches Borken, which matches the EXPECTED answer.</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>0.1366</v>
+        <v>0.1405</v>
       </c>
       <c r="K22" t="n">
-        <v>0.3919</v>
+        <v>0.4034</v>
       </c>
       <c r="L22" t="n">
-        <v>0.2572</v>
+        <v>0.2644</v>
       </c>
     </row>
     <row r="23">
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>5.68</v>
+        <v>4.849</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>The actual answer does not address whether Senden and Münster are geographically disjoint and provides no relevant geographic information.</t>
+          <t>The actual answer does not address whether Senden and Münster are geographically disjoint and provides no relevant comparison.</t>
         </is>
       </c>
       <c r="J23" t="n">
@@ -1645,11 +1645,11 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Yes. Niedersachsen touches Nordrhein-Westfalen. Both are FederalStates, and the hierarchy ends with Germany as the State.</t>
+          <t>Yes. Niedersachsen touches Nordrhein-Westfalen, and both are FederalStates in Germany.</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>4.869</v>
+        <v>4.545</v>
       </c>
       <c r="G24" t="n">
         <v>1</v>
@@ -1661,17 +1661,17 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>The actual answer confirms that Niedersachsen touches Nordrhein-Westfalen, matching the expected response.</t>
+          <t>The ACTUAL answer states that Niedersachsen touches Nordrhein-Westfalen, matching the EXPECTED answer.</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>0.3587</v>
+        <v>0.4336</v>
       </c>
       <c r="K24" t="n">
-        <v>0.5385</v>
+        <v>0.5523</v>
       </c>
       <c r="L24" t="n">
-        <v>0.4457</v>
+        <v>0.4921</v>
       </c>
     </row>
     <row r="25">
@@ -1697,33 +1697,33 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>No. Berlin is not completely surrounded by Brandenburg based on the provided information. The result only shows that Berlin has two matching neighboring places: Schöneiche bei Berlin and Neuenhagen bei Berlin, both of which are Cities in Germany.</t>
+          <t>Yes. Berlin has two matching places associated with it: Schöneiche bei Berlin and Neuenhagen bei Berlin. Both are cities in Brandenburg, and Brandenburg is a Federal State in Germany.</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>7.194</v>
+        <v>6.052</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>The expected answer says Berlin is completely surrounded by Brandenburg, but the actual answer explicitly says it is not completely surrounded.</t>
+          <t>The ACTUAL answer confirms Berlin is surrounded by Brandenburg and is consistent with the EXPECTED answer. It adds extra details about specific towns, which are not incorrect.</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>0.0849</v>
+        <v>0.1301</v>
       </c>
       <c r="K25" t="n">
-        <v>0.5225</v>
+        <v>0.4314</v>
       </c>
       <c r="L25" t="n">
-        <v>0.2811</v>
+        <v>0.2705</v>
       </c>
     </row>
     <row r="26">
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>6.858</v>
+        <v>4.969</v>
       </c>
       <c r="G26" t="n">
         <v>1</v>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>The actual answer states that Münster is north of Dortmund, matching the expected answer.</t>
+          <t>The actual answer explicitly states that Münster is north of Dortmund, matching the expected answer.</t>
         </is>
       </c>
       <c r="J26" t="n">
@@ -1801,11 +1801,11 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Greven is located directly north of Münster. Both cities are in Germany.</t>
+          <t>Greven is located directly north of Münster. Greven is a city in the district, administrative district, Federal State, and State hierarchy level, ending with Germany as the State.</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>8.593</v>
+        <v>5.902</v>
       </c>
       <c r="G27" t="n">
         <v>1</v>
@@ -1817,17 +1817,17 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>The actual answer states that Greven is directly north of Münster, matching the expected answer. The additional note that both cities are in Germany is correct and does not conflict.</t>
+          <t>The ACTUAL answer states that Greven is located directly north of Münster, matching the EXPECTED answer. Extra administrative hierarchy details are additional and do not contradict the expected content.</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>0.6034</v>
+        <v>0.2425</v>
       </c>
       <c r="K27" t="n">
-        <v>0.859</v>
+        <v>0.7647</v>
       </c>
       <c r="L27" t="n">
-        <v>0.725</v>
+        <v>0.4737</v>
       </c>
     </row>
     <row r="28">
@@ -1853,11 +1853,11 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Yes. Leipzig is located northeast of Erfurt. Both are cities, and their location is in Germany, the State.</t>
+          <t>Yes. Leipzig is located in the northeastern direction from Erfurt. The location hierarchy is: Leipzig is a city in a district, in an administrative district, in a federal state, in Germany. Erfurt is a city in a district, in an administrative district, in a federal state, in Germany.</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>6.347</v>
+        <v>5.034</v>
       </c>
       <c r="G28" t="n">
         <v>1</v>
@@ -1869,17 +1869,17 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>The actual answer explicitly confirms that Leipzig is located northeast of Erfurt, matching the expected content. Additional non-conflicting details are also provided.</t>
+          <t>The actual answer explicitly states that Leipzig is in the northeastern direction from Erfurt, matching the expected response. Additional correct hierarchical location details are included.</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>0.3685</v>
+        <v>-0.0095</v>
       </c>
       <c r="K28" t="n">
-        <v>0.7513</v>
+        <v>0.5593</v>
       </c>
       <c r="L28" t="n">
-        <v>0.5445</v>
+        <v>0.2355</v>
       </c>
     </row>
     <row r="29">
@@ -1905,11 +1905,11 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Köln and Bonn are 6.63 km apart. Köln is a city in the administrative community, district, administrative district, federal state, and state hierarchy ending in Germany. Bonn is a city in the administrative community, district, administrative district, federal state, and state hierarchy ending in Germany.</t>
+          <t>Köln and Bonn are cities in Germany. The distance between Köln and Bonn is 6.63 km.</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>17.222</v>
+        <v>10.517</v>
       </c>
       <c r="G29" t="n">
         <v>1</v>
@@ -1921,17 +1921,17 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>The actual answer states the distance between Köln and Bonn is 6.63 km, matching the expected value.</t>
+          <t>The actual answer states the distance between Köln and Bonn as 6.63 km, matching the expected value.</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>0.0392</v>
+        <v>0.6608000000000001</v>
       </c>
       <c r="K29" t="n">
-        <v>0.3571</v>
+        <v>0.6449</v>
       </c>
       <c r="L29" t="n">
-        <v>0.1862</v>
+        <v>0.6533</v>
       </c>
     </row>
     <row r="30">
@@ -1957,11 +1957,11 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Hannover and Braunschweig are 34.92 km apart. Hannover is a city in Germany, and Braunschweig is a city in Germany.</t>
+          <t>Hannover is a city in the AdministrativeDistrict of Hannover, in the FederalState of Lower Saxony, in Germany. Braunschweig is a city in the AdministrativeDistrict of Braunschweig, in the FederalState of Lower Saxony, in Germany. The distance between Hannover and Braunschweig is 34.92 km.</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>12.308</v>
+        <v>9.452999999999999</v>
       </c>
       <c r="G30" t="n">
         <v>1</v>
@@ -1973,17 +1973,17 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>The actual answer states the distance is 34.92 km, matching the expected value.</t>
+          <t>The actual answer states that the distance between Hannover and Braunschweig is 34.92 km, matching the expected information.</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>0.3009</v>
+        <v>0.0992</v>
       </c>
       <c r="K30" t="n">
-        <v>0.3494</v>
+        <v>0.5893</v>
       </c>
       <c r="L30" t="n">
-        <v>0.3259</v>
+        <v>0.3162</v>
       </c>
     </row>
     <row r="31">
@@ -2009,11 +2009,11 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Hessen is a FederalState in Germany, and Thüringen is also a FederalState in Germany. The distance between them is 0.0 km.</t>
+          <t>Hessen and Thüringen are 0.0 km apart. Both are FederalStates in Germany, the State.</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>15.187</v>
+        <v>11.617</v>
       </c>
       <c r="G31" t="n">
         <v>1</v>
@@ -2025,17 +2025,17 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>The actual answer states that the distance between Hessen and Thüringen is 0.0 km, matching the expected answer.</t>
+          <t>The actual answer matches the expected distance (0.0 km). Additional correct context about them being German federal states is included.</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>0.3552</v>
+        <v>0.5306999999999999</v>
       </c>
       <c r="K31" t="n">
-        <v>0.4911</v>
+        <v>0.647</v>
       </c>
       <c r="L31" t="n">
-        <v>0.4219</v>
+        <v>0.588</v>
       </c>
     </row>
     <row r="32">
@@ -2061,11 +2061,11 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>The district of Miesbach has three closest districts: München, Bad Tölz-Wolfratshausen, and Rosenheim. Miesbach is a district in the Federal State of Bayern, in Germany.</t>
+          <t>The three closest districts to Miesbach are München, Bad Tölz-Wolfratshausen, and Rosenheim. Miesbach is a district in the AdministrativeDistrict of Upper Bavaria in the FederalState of Bavaria, in Germany.</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>5.366</v>
+        <v>3.837</v>
       </c>
       <c r="G32" t="n">
         <v>1</v>
@@ -2077,17 +2077,17 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>The ACTUAL answer lists the same three closest districts—München, Bad Tölz-Wolfratshausen, and Rosenheim—as in the EXPECTED answer.</t>
+          <t>The actual answer lists the same three closest districts as the expected (München, Bad Tölz-Wolfratshausen, Rosenheim). Additional context about Miesbach is correct and does not affect the match.</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>0.5613</v>
+        <v>0.4309</v>
       </c>
       <c r="K32" t="n">
-        <v>0.7284</v>
+        <v>0.7469</v>
       </c>
       <c r="L32" t="n">
-        <v>0.6425</v>
+        <v>0.5787</v>
       </c>
     </row>
     <row r="33">
@@ -2113,11 +2113,11 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>The district of Warendorf touches the districts of Gütersloh, Steinfurt, Soest, Coesfeld, Osnabrück, Münster, and Hamm. Warendorf is a district in an administrative district in a federal state in Germany.</t>
+          <t>Warendorf is a district in the administrative district of Münster in the federal state of North Rhine-Westphalia in Germany. The districts that touch Warendorf are Gütersloh, Steinfurt, Soest, Coesfeld, Osnabrück, Münster, and Hamm.</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>5.659</v>
+        <v>3.934</v>
       </c>
       <c r="G33" t="n">
         <v>1</v>
@@ -2129,17 +2129,17 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>The actual answer lists all the expected neighboring districts: Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld, and Soest (order differs). The extra statement about Warendorf being a district is correct and does not omit anything.</t>
+          <t>The ACTUAL answer lists all expected neighboring districts: Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld, and Soest.</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>0.6095</v>
+        <v>0.4444</v>
       </c>
       <c r="K33" t="n">
-        <v>0.83</v>
+        <v>0.699</v>
       </c>
       <c r="L33" t="n">
-        <v>0.7151999999999999</v>
+        <v>0.5653</v>
       </c>
     </row>
     <row r="34">
@@ -2165,11 +2165,11 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>The administrative community Leezen is adjacent to Bad Oldesloe-Land, Trave-Land, Boostedt-Rickling, Auenland Südholstein, Wahlstedt, Kisdorf, Bad Segeberg, Itzstedt, and Buchholz (Forstgutsbez.). Leezen is an administrative community in the district of Segeberg, in the administrative district of Schleswig-Holstein, in the Federal State of Schleswig-Holstein, in Germany.</t>
+          <t>The administrative community Leezen is adjacent to Bad Oldesloe-Land, Trave-Land, Boostedt-Rickling, Auenland Südholstein, Wahlstedt, Kisdorf, Bad Segeberg, Itzstedt, and Buchholz (Forstgutsbez.). Leezen is an administrative community in the district of Segeberg, in the federal state of Schleswig-Holstein, in Germany.</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>5.708</v>
+        <v>4.329</v>
       </c>
       <c r="G34" t="n">
         <v>1</v>
@@ -2181,17 +2181,17 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>The actual answer lists all the expected adjacent administrative communities: Auenland Südholstein, Kisdorf, Bad Oldesloe-Land, Trave-Land, Wahlstedt, Itzstedt, Bad Segeberg, Boostedt-Rickling, and Buchholz (Forstgutsbez.). Additional district/location information is also correct and does not affect adjacency completeness.</t>
+          <t>The actual answer lists all nine adjacent administrative communities named in the expected answer, including Auenland Südholstein, Kisdorf, Bad Oldesloe-Land, Trave-Land, Wahlstedt, Itzstedt, Bad Segeberg, Boostedt-Rickling, and Buchholz (Forstgutsbez.). Additional information about Leezen is also provided but does not affect correctness.</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>0.5047</v>
+        <v>0.579</v>
       </c>
       <c r="K34" t="n">
-        <v>0.746</v>
+        <v>0.754</v>
       </c>
       <c r="L34" t="n">
-        <v>0.6197</v>
+        <v>0.6637999999999999</v>
       </c>
     </row>
     <row r="35">
@@ -2217,11 +2217,11 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Mittelfranken is surrounded by the administrative districts of Oberpfalz, Oberbayern, Schwaben, Oberfranken, Unterfranken, and Stuttgart. Mittelfranken is an AdministrativeDistrict in the FederalState of Bayern in Germany.</t>
+          <t>Mittelfranken is surrounded by the administrative districts of Oberpfalz, Oberbayern, Schwaben, Oberfranken, Unterfranken, and Stuttgart. Mittelfranken is an AdministrativeDistrict in Germany.</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>5.582</v>
+        <v>3.949</v>
       </c>
       <c r="G35" t="n">
         <v>1</v>
@@ -2233,17 +2233,17 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>The ACTUAL answer lists the same surrounding administrative districts as the EXPECTED: Oberpfalz, Unterfranken, Oberfranken, Oberbayern, Schwaben, and Stuttgart.</t>
+          <t>The ACTUAL answer lists the same six surrounding administrative districts as the EXPECTED answer: Oberpfalz, Unterfranken, Oberfranken, Oberbayern, Schwaben, and Stuttgart. Extra statement about Mittelfranken being an AdministrativeDistrict is correct and does not omit anything.</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>0.6056</v>
+        <v>0.6868</v>
       </c>
       <c r="K35" t="n">
-        <v>0.8517</v>
+        <v>0.8639</v>
       </c>
       <c r="L35" t="n">
-        <v>0.7229</v>
+        <v>0.7725</v>
       </c>
     </row>
     <row r="36">
@@ -2269,11 +2269,11 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>The federal states located north of Thüringen are Mecklenburg-Vorpommern, Sachsen-Anhalt, Schleswig-Holstein, and Hamburg. Thüringen is a federal state in Germany, and these federal states are also in Germany.</t>
+          <t>Thüringen is a FederalState in Germany. The FederalStates shown north of Thüringen are Schleswig-Holstein, Sachsen-Anhalt, Mecklenburg-Vorpommern, and Hamburg, and all of them are in Germany.</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>47.049</v>
+        <v>30.983</v>
       </c>
       <c r="G36" t="n">
         <v>1</v>
@@ -2285,17 +2285,17 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>The actual answer lists exactly the same four federal states north of Thüringen as the expected answer: Hamburg, Schleswig-Holstein, Mecklenburg-Vorpommern, and Sachsen-Anhalt (order differs, but content matches).</t>
+          <t>The actual answer lists the same federal states north of Thüringen as the expected answer: Hamburg, Schleswig-Holstein, Mecklenburg-Vorpommern, and Sachsen-Anhalt.</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>0.5883</v>
+        <v>0.4871</v>
       </c>
       <c r="K36" t="n">
-        <v>0.798</v>
+        <v>0.7452</v>
       </c>
       <c r="L36" t="n">
-        <v>0.6891</v>
+        <v>0.6096</v>
       </c>
     </row>
     <row r="37">
@@ -2321,11 +2321,11 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>The districts west of Münster are Kleve and Borken. Münster is a district in the administrative district of Münster, in the federal state of North Rhine-Westphalia, in Germany. Kleve and Borken are districts in the administrative district of Düsseldorf, in the federal state of North Rhine-Westphalia, in Germany.</t>
+          <t>The districts west of Münster are Kleve and Borken. Both are districts in the AdministrativeDistrict of Münster in the FederalState of North Rhine-Westphalia in Germany.</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>53.2</v>
+        <v>31.492</v>
       </c>
       <c r="G37" t="n">
         <v>1</v>
@@ -2337,17 +2337,17 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>The actual answer states that the districts west of Münster are Kleve and Borken, matching the expected content.</t>
+          <t>The ACTUAL answer states that the districts west of Münster are Kleve and Borken, matching the EXPECTED answer. Additional correct context is provided.</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>0.08119999999999999</v>
+        <v>0.1798</v>
       </c>
       <c r="K37" t="n">
-        <v>0.5554</v>
+        <v>0.6905</v>
       </c>
       <c r="L37" t="n">
-        <v>0.2918</v>
+        <v>0.4058</v>
       </c>
     </row>
     <row r="38">
@@ -2373,11 +2373,11 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>The administrative community Kiel is located in the administrative district Schleswig-Holstein in Germany. The administrative communities located north of Kiel are Geltinger Bucht, Dänischenhagen, Altenholz, and Kappeln, all in the same administrative district Schleswig-Holstein in Germany.</t>
+          <t>The administrative community Kiel is located in the district of Rendsburg-Eckernförde, in the administrative district of Schleswig-Holstein, in the federal state of Schleswig-Holstein, in Germany. The administrative communities located north of Kiel are Geltinger Bucht, Altenholz, Dänischenhagen, and Kappeln.</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>54.887</v>
+        <v>30.793</v>
       </c>
       <c r="G38" t="n">
         <v>1</v>
@@ -2389,17 +2389,17 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>The actual answer lists all expected communities north of Kiel: Altenholz, Dänischenhagen, Kappeln, and Geltinger Bucht. No conflicting information is provided.</t>
+          <t>The actual answer lists exactly the expected northern administrative communities (Altenholz, Dänischenhagen, Kappeln, Geltinger Bucht). Additional context about Kiel’s location is correct and does not affect completeness.</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>0.4421</v>
+        <v>0.3094</v>
       </c>
       <c r="K38" t="n">
-        <v>0.7419</v>
+        <v>0.7366</v>
       </c>
       <c r="L38" t="n">
-        <v>0.5829</v>
+        <v>0.5034</v>
       </c>
     </row>
     <row r="39">
@@ -2425,11 +2425,11 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>The districts within a radius of 10 km from Göttingen are Northeim, Kassel, Goslar, Nordhausen, Werra-Meißner-Kreis, Eichsfeld, another district named Kassel, and Harz. Göttingen is a district in Germany, and all of these districts are also in Germany.</t>
+          <t>The district of Göttingen has eight districts within a radius of 10 km: Harz, Eichsfeld, Kassel, Werra-Meißner-Kreis, Kassel, Northeim, Nordhausen, and Goslar. All of them are districts in Germany.</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>70.682</v>
+        <v>48.075</v>
       </c>
       <c r="G39" t="n">
         <v>1</v>
@@ -2441,17 +2441,17 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>The ACTUAL answer lists all expected districts (Harz, Northeim, Goslar, Kassel, Eichsfeld, Werra-Meißner-Kreis, Nordhausen). The only difference is that Kassel is mentioned twice and there is extra nonessential text, which does not affect correctness.</t>
+          <t>The ACTUAL answer lists all the expected districts within 10 km of Göttingen (Harz, Northeim, Goslar, Kassel, Eichsfeld, Werra-Meißner-Kreis, Nordhausen). The only difference is an extra duplicate mention of Kassel and additional generic wording, which does not omit any expected information.</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>0.5449000000000001</v>
+        <v>0.7195</v>
       </c>
       <c r="K39" t="n">
-        <v>0.7071</v>
+        <v>0.8269</v>
       </c>
       <c r="L39" t="n">
-        <v>0.6238</v>
+        <v>0.7724</v>
       </c>
     </row>
     <row r="40">
@@ -2477,11 +2477,11 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>The cities located within a radius of 5 km of Aachen are Würselen, Alsdorf, Roetgen, Herzogenrath, Eschweiler, Hürtgenwald, Stolberg (Rhld.), and Simmerath. Aachen is a city in the District of Aachen, in the Administrative District of Cologne, in the Federal State of North Rhine-Westphalia, in Germany.</t>
+          <t>The cities located within a radius of 5 km of Aachen are Stolberg (Rhld.), Würselen, Alsdorf, Simmerath, Hürtgenwald, Eschweiler, Roetgen, and Herzogenrath. Aachen is a city in the district of Städteregion Aachen, in the administrative district of Köln, in the federal state of Nordrhein-Westfalen, in Germany.</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>64.473</v>
+        <v>37.623</v>
       </c>
       <c r="G40" t="n">
         <v>1</v>
@@ -2493,17 +2493,17 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>All expected cities (Alsdorf, Simmerath, Würselen, Hürtgenwald, Roetgen, Herzogenrath, Eschweiler, Stolberg (Rhld.)) are present in the actual answer. Additional information about Aachen is correct and does not omit any expected content.</t>
+          <t>All expected cities are present in the actual answer: Alsdorf, Simmerath, Würselen, Hürtgenwald, Roetgen, Herzogenrath, Eschweiler, and Stolberg (Rhld.).</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>0.4458</v>
+        <v>0.4754</v>
       </c>
       <c r="K40" t="n">
-        <v>0.7069</v>
+        <v>0.7222</v>
       </c>
       <c r="L40" t="n">
-        <v>0.5696</v>
+        <v>0.5929</v>
       </c>
     </row>
     <row r="41">
@@ -2529,34 +2529,34 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>The cities located less than 2 km around Munich are Krailling, Hebertshausen, Putzbrunn, Gräfelfing, Pullach i. Isartal, Bergkirchen, Ottobrunn, Haar, Gröbenzell, Vaterstetten, Karlsfeld, Planegg, Puchheim, Grünwalder Forst, Neubiberg, Oberschleißheim, Germering, Perlacher Forst, Dachau, Feldkirchen, Olching, Unterföhring, Unterhaching, Garching b. München, Ismaning, Neuried, Hohenbrunn, Forstenrieder Park, Aschheim, Grünwald, and Grasbrunn.
-Munich is a City in the District of Upper Bavaria, in the FederalState of Bavaria, in Germany.</t>
+          <t>The cities located less than 2 km around Munich are Vaterstetten, Ottobrunn, Gräfelfing, Pullach i.Isartal, Hohenbrunn, Neuried, Hebertshausen, Gröbenzell, Haar, Neubiberg, Unterföhring, Ismaning, Olching, Forstenrieder Park, Karlsfeld, Aschheim, Dachau, Grünwald, Germering, Grünwalder Forst, Grasbrunn, Perlacher Forst, Oberschleißheim, Garching b.München, Feldkirchen, Bergkirchen, Putzbrunn, Krailling, Planegg, Puchheim, and Unterhaching.
+Munich is a city in the AdministrativeCommunity of München, within the District of München, in the AdministrativeDistrict of Oberbayern, in the FederalState of Bayern, in Germany.</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>60.681</v>
+        <v>42.34</v>
       </c>
       <c r="G41" t="n">
-        <v>0.9</v>
+        <v>0.72</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Most expected cities are present in the actual list; however, Feldkirchen is included but some expected entries are missing (e.g., Forstenrieder Park is present, but Grünwald is present; missing cities include Aschheim? (present), yet missing are specifically: Perlacher Forst is present, but Gröbenzell present; the main omissions are Bergkirchen? present; the remaining missing ones appear to be Planegg? present, Ismaning present, but Unterföhring present, Oberschleißheim present, Putzbrunn present, Neuried present, and Germering present. The missing expected city is 'Haar' is present. The only clearly missing expected city is 'Haar'?? (actually present). After comparing, all expected cities except 'Bergkirchen'? present. Overall discrepancy is small but not perfect: expected includes 'Bergkirchen' and 'Neuried' and 'Putzbrunn' all present; expected includes 'Gröbenzell' present. The actual list includes additional cities not in expected (e.g., Krailling, Hebertshausen, Ottobrunn, Vaterstetten, Hohenbrunn, Grasbrunn, Dachau, Hohenbrunn). Because the expected list appears to be fully covered, score is high; but strict check shows 'Aschheim' present, 'Feldkirchen' present. The only mismatch is 'Grünwalder Forst' vs expected 'Forstenrieder Park' etc; these are additional not replacements. So likely passed; however, expected includes 'Neubiberg' which is present as 'Neubiberg'. Hence it should be PASSED—giving slight uncertainty due to formatting/spacing. </t>
+          <t>All expected cities are not present in the actual answer: missing Feldkirchen (present), but missing Erlanger? none. Specifically missing Aschheim? (present), Unterhaching (present), Germering (present), Olching (present), Grünwald (present), etc. However the actual answer includes additional cities like Vaterstetten, Ottobrunn, Hohenbrunn, Hebertshausen, Hebertshausen, etc., and appears to omit Karlsfeld? (present), Neuried (present), Unterföhring (present). The main gap is that 'Neubiberg' and 'Unterhaching' are present; 'Neuried' present; 'Neubiberg' present; 'Gräfelfing' present. The only clear omission from expected is 'Haar'? present. 'Bergkirchen' present. Missing 'Garching b.München'? present. Missing 'Planegg'? present. Missing 'Perlacher Forst'? present. Missing 'Puchheim'? present. Missing 'Gröbenzell'? present. Missing 'Gräfelfing'? present. Missing 'Feldkirchen'? present. Missing 'Aschheim'? present. Missing 'Haar'? present. Missing 'Karlsfeld'? present. Missing 'Garching b.München'? present. 'Oberschleißheim' present. 'Putzbrunn' present. 'Garching b.München' present. The expected list includes 'Bergkirchen' yes present; 'Neubiberg' yes present. But expected includes 'Germering' yes present. Expected includes 'Pullach i.Isartal' yes present. Overall most are present; likely the missing item is 'Haar' present. Another missing is 'Gräfelfing' present. Therefore only a small subset seems missing, but exact count suggests 2-3 missing items (e.g., Feldkirchen present, but 'Unterhaching' present, leaving 'Neuried' present). Due to inability to perfectly verify within the provided text, the score is set to reflect partial coverage.</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>0.6026</v>
+        <v>0.5187</v>
       </c>
       <c r="K41" t="n">
-        <v>0.742</v>
+        <v>0.7402</v>
       </c>
       <c r="L41" t="n">
-        <v>0.6708</v>
+        <v>0.6248</v>
       </c>
     </row>
     <row r="42">
@@ -2582,16 +2582,14 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Es gibt zwei Orte mit dem Namen Münster:
-Münster mit den Hierarchiestufen Stadt, Kreis, Verwaltungsgebiet, Bundesland Nordrhein-Westfalen und Bundesstaat Deutschland liegt in Nordrhein-Westfalen in Deutschland.
-Münster mit den Hierarchiestufen Stadt, Kreis, Verwaltungsgebiet, Bundesland Bayern und Bundesstaat Deutschland liegt in Bayern in Deutschland.</t>
+          <t>Münster liegt in der Verwaltungsgemeinde Münster, im Kreis Münster, im Regierungsbezirk Münster, im Bundesland Nordrhein-Westfalen, in Deutschland.</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>6.868</v>
+        <v>5.01</v>
       </c>
       <c r="G42" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -2600,17 +2598,17 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Die Antwort nennt korrekt, dass es zwei Orte namens Münster gibt und ordnet einen nach Nordrhein-Westfalen und einen nach Bayern ein. Allerdings fehlen die im Erwarteten geforderten Angaben zu Regierungsbezirk (Münster vs. Schwaben) und zu den Landkreisen/Kreis sowie die Zuordnung zum 'Kreis Münster' bzw. 'Landkreis Donau-Ries' sowie der Hinweis zur Gemeinde Rain.</t>
+          <t>Der ACTUAL-Text nennt den Münster-Bezug zu Kreis Münster, Regierungsbezirk Münster und NRW (NRW Deutschland) korrekt. Es fehlt jedoch die im EXPECTED erwähnte zweite Stadt Münster in Rain (Bayern, Schwaben, Landkreis Donau-Ries).</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>0.143</v>
+        <v>0.4701</v>
       </c>
       <c r="K42" t="n">
-        <v>0.1611</v>
+        <v>0.234</v>
       </c>
       <c r="L42" t="n">
-        <v>0.1533</v>
+        <v>0.3463</v>
       </c>
     </row>
     <row r="43">
@@ -2636,11 +2634,11 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Köln liegt in der Stadt Köln, in der Stadt Köln, im Kreis Köln, im Regierungsbezirk Köln, im Bundesland Nordrhein-Westfalen und im Bundesstaat Deutschland.</t>
+          <t>Die Stadt Köln liegt in der Verwaltungsgemeinde Köln, im Kreis Köln, im Bundesland Nordrhein-Westfalen und im Bundesstaat Deutschland.</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>4.977</v>
+        <v>3.944</v>
       </c>
       <c r="G43" t="n">
         <v>1</v>
@@ -2652,17 +2650,17 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Die ACTUAL-Antwort enthält die geforderten Informationen: Köln liegt im Regierungsbezirk Köln und im Bundesland Nordrhein-Westfalen. Zusätzliche Angaben sind ebenfalls korrekt.</t>
+          <t>Die ACTUAL-Antwort enthält das erwartete Bundesland Nordrhein-Westfalen. Sie nennt außerdem weitere, zusätzliche korrekte administrativen Einordnungen. Der spezifische Hinweis „im Regierungsbezirk Köln“ fehlt jedoch, aber die Kerninformation des EXPECTED ist enthalten.</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>0.645</v>
+        <v>0.6515</v>
       </c>
       <c r="K43" t="n">
-        <v>0.7623</v>
+        <v>0.838</v>
       </c>
       <c r="L43" t="n">
-        <v>0.7027</v>
+        <v>0.7416</v>
       </c>
     </row>
     <row r="44">
@@ -2692,7 +2690,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>4.625</v>
+        <v>4.756</v>
       </c>
       <c r="G44" t="n">
         <v>1</v>
@@ -2704,7 +2702,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort nennt Landkreis bzw. Kreis Oder-Spree und Bundesland Brandenburg; das passt vollständig zum Erwarteten. Zusatzangaben zur Stadt Eisenhüttenstadt sind nicht widersprüchlich.</t>
+          <t>Der tatsächliche Antworttext enthält alle Kernaussagen der Erwartung: Ort in der Stadt Eisenhüttenstadt, Kreis/Landkreis Oder-Spree und Bundesland Brandenburg. Zusatzdetails sind korrekt.</t>
         </is>
       </c>
       <c r="J44" t="n">
@@ -2740,11 +2738,11 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Die Verwaltungsgemeinschaft Esens liegt in der Stadt Esens im Kreis Wittmund im Bundesland Niedersachsen in Deutschland.</t>
+          <t>Die Verwaltungsgemeinschaft Esens liegt im Kreis Wittmund im Bundesland Niedersachsen in Deutschland.</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>4.895</v>
+        <v>5.027</v>
       </c>
       <c r="G45" t="n">
         <v>1</v>
@@ -2756,17 +2754,17 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort enthält alle Kernaussagen der erwarteten Antwort: Esens liegt im Kreis/Landkreis Wittmund (Kreis Wittmund) in Niedersachsen. Zusatzinfos (Stadt Esens, Deutschland) sind ebenfalls korrekt.</t>
+          <t>Die tatsächliche Antwort enthält alle Kernaussagen der erwarteten Antwort: Esens liegt im Landkreis/Kreis Wittmund in Niedersachsen (Deutschland).</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>0.7292</v>
+        <v>0.8451</v>
       </c>
       <c r="K45" t="n">
-        <v>0.8506</v>
+        <v>0.9229000000000001</v>
       </c>
       <c r="L45" t="n">
-        <v>0.7887999999999999</v>
+        <v>0.8836000000000001</v>
       </c>
     </row>
     <row r="46">
@@ -2792,11 +2790,11 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Der Kreis Gießen liegt in Gießen, im Bundesland Hessen, in Deutschland.</t>
+          <t>Der Kreis Gießen liegt in der Verwaltungsgemeinde Gießen, im Kreis Gießen, im Bundesland Hessen und im Bundesstaat Deutschland.</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>5.094</v>
+        <v>4.561</v>
       </c>
       <c r="G46" t="n">
         <v>1</v>
@@ -2808,17 +2806,17 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Der tatsächliche Text nennt korrekt, dass der Kreis/Landkreis Gießen im Bundesland Hessen liegt. Die erwartete Angabe wird vollständig abgedeckt; zusätzliche Details (Ort und Deutschland) sind korrekt.</t>
+          <t>Der tatsächliche Text bestätigt, dass der Kreis/Landkreis Gießen im Bundesland Hessen liegt; zusätzliche korrekte Informationen werden genannt.</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>0.6394</v>
+        <v>0.4355</v>
       </c>
       <c r="K46" t="n">
-        <v>0.8264</v>
+        <v>0.753</v>
       </c>
       <c r="L46" t="n">
-        <v>0.7297</v>
+        <v>0.584</v>
       </c>
     </row>
     <row r="47">
@@ -2848,7 +2846,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>7.053</v>
+        <v>4.342</v>
       </c>
       <c r="G47" t="n">
         <v>1</v>
@@ -2860,7 +2858,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort nennt korrekt, dass der Landkreis/Kreis Nordsachsen im Bundesland Sachsen liegt. Die zusätzliche Angabe „in Deutschland“ ist korrekt und schadet nicht.</t>
+          <t>Der tatsächliche Text nennt korrekt, dass der Landkreis/Kreis Nordsachsen im Bundesland Sachsen liegt; die zusätzliche Angabe „in Deutschland“ ist korrekt.</t>
         </is>
       </c>
       <c r="J47" t="n">
@@ -2900,7 +2898,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>5.182</v>
+        <v>3.975</v>
       </c>
       <c r="G48" t="n">
         <v>1</v>
@@ -2912,7 +2910,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Die Antwort nennt korrekt, dass der Regierungsbezirk Freiburg im Bundesland Baden-Württemberg liegt; zusätzliche Angabe „in Deutschland“ ist ebenfalls korrekt.</t>
+          <t>Der tatsächliche Text nennt denselben Regierungs-/Verwaltungsbezug und bestätigt korrekt, dass Freiburg im Bundesland Baden-Württemberg liegt; die zusätzliche Angabe „in Deutschland“ ist nicht widersprüchlich.</t>
         </is>
       </c>
       <c r="J48" t="n">
@@ -2952,7 +2950,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>5.202</v>
+        <v>3.978</v>
       </c>
       <c r="G49" t="n">
         <v>1</v>
@@ -2964,7 +2962,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Der tatsächliche Antwortsatz nennt korrekt, dass Oberfranken im Bundesland Bayern liegt; das entspricht der erwarteten Angabe. Die zusätzliche Information, dass es in Deutschland liegt, schadet nicht.</t>
+          <t>Der tatsächliche Text nennt korrekt, dass Oberfranken im Bundesland Bayern liegt; die erwartete Information ist vollständig enthalten (zusätzlich wird Deutschland erwähnt).</t>
         </is>
       </c>
       <c r="J49" t="n">
@@ -3000,11 +2998,11 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Sachsen ist ein Bundesland in Deutschland.</t>
+          <t>Sachsen liegt im Bundesland Sachsen in Deutschland. Es ist als Bundesland dem Bundesstaat Deutschland zugeordnet.</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>7.316</v>
+        <v>4.978</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
@@ -3016,17 +3014,17 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Die Antwort enthält keine der erwarteten Koordinaten/keine Lagebeschreibung mit dem angegebenen Punkt (13.3485, 51.0523).</t>
+          <t>Die erwartete Ortsangabe bzw. Koordinaten (13.3485..., 51.0523...) fehlen komplett; die tatsächliche Antwort beschreibt nur allgemein, dass Sachsen ein Bundesland in Deutschland ist.</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>0.3879</v>
+        <v>0.3072</v>
       </c>
       <c r="K50" t="n">
-        <v>-0.3221</v>
+        <v>-0.2595</v>
       </c>
       <c r="L50" t="n">
-        <v>-0.0376</v>
+        <v>-0.0207</v>
       </c>
     </row>
     <row r="51">
@@ -3052,11 +3050,11 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Das Saarland liegt in Deutschland.</t>
+          <t>Das Bundesland Saarland liegt in Deutschland, also im Bundesstaat Deutschland.</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>4.712</v>
+        <v>3.87</v>
       </c>
       <c r="G51" t="n">
         <v>0</v>
@@ -3068,17 +3066,17 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort nennt nur allgemein, dass das Saarland in Deutschland liegt, enthält aber keine geografische Koordinate bzw. den verlangten Punkt (6,953360955673903 49,38438040655551).</t>
+          <t>Die ACTUAL-Antwort nennt nur, dass Saarland in Deutschland liegt, aber keine Lage bzw. keinen Punkt mit den geforderten Koordinaten (6,95336, 49,38438).</t>
         </is>
       </c>
       <c r="J51" t="n">
-        <v>0.5946</v>
+        <v>0.4326</v>
       </c>
       <c r="K51" t="n">
-        <v>-0.2394</v>
+        <v>-0.1786</v>
       </c>
       <c r="L51" t="n">
-        <v>0.0872</v>
+        <v>0.07770000000000001</v>
       </c>
     </row>
     <row r="52">
@@ -3104,33 +3102,33 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Zum Kreis Coesfeld gehören die Städte Rosendahl, Havixbeck, Senden, Billerbeck, Ascheberg, Dülmen, Nottuln, Coesfeld, Nordkirchen, Lüdinghausen und Olfen. Der Kreis Coesfeld liegt im Regierungsbezirk Münster, im Bundesland Nordrhein-Westfalen, in Deutschland.</t>
+          <t>Es wurden keine Geodaten gefunden.</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>5.512</v>
+        <v>4.356</v>
       </c>
       <c r="G52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort nennt genau die in der erwarteten Antwort aufgeführten Städte (Coesfeld, Olfen, Senden, Nottuln, Havixbeck, Nordkirchen, Billerbeck, Lüdinghausen, Rosendahl, Dülmen, Ascheberg). Zusatzinfo ist korrekt und beeinträchtigt nicht.</t>
+          <t>Die tatsächliche Antwort enthält keine der Städte aus der erwarteten Liste (keine Geodaten bzw. keine Angaben).</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>0.5961</v>
+        <v>0.0349</v>
       </c>
       <c r="K52" t="n">
-        <v>0.7522</v>
+        <v>-0.3518</v>
       </c>
       <c r="L52" t="n">
-        <v>0.6721</v>
+        <v>-0.1806</v>
       </c>
     </row>
     <row r="53">
@@ -3156,11 +3154,11 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Im Regierungsbezirk Oberbayern liegen die Kreise Dachau, Miesbach, Garmisch-Partenkirchen, Landsberg am Lech, Rosenheim, Eichstätt, Ingolstadt, Fürstenfeldbruck, München, Berchtesgadener Land, Bad Tölz-Wolfratshausen, Ebersberg, München, Pfaffenhofen a.d.Ilm, Traunstein, Neuburg-Schrobenhausen, Mühldorf a.Inn, Starnberg, Rosenheim, Altötting, Weilheim-Schongau, Freising und Erding. Oberbayern liegt im Bundesland Bayern in Deutschland.</t>
+          <t>Im Regierungsbezirk Oberbayern liegen die Kreise Dachau, Miesbach, Garmisch-Partenkirchen, Landsberg am Lech, Rosenheim, Eichstätt, Ingolstadt, Fürstenfeldbruck, München, Berchtesgadener Land, Bad Tölz-Wolfratshausen, Ebersberg, Pfaffenhofen a.d.Ilm, Traunstein, Neuburg-Schrobenhausen, Mühldorf a.Inn, Starnberg, Altötting, Weilheim-Schongau, Freising und Erding. Oberbayern liegt im Bundesland Bayern in Deutschland.</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>5.07</v>
+        <v>4.53</v>
       </c>
       <c r="G53" t="n">
         <v>1</v>
@@ -3172,17 +3170,17 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Alle im Erwarteten genannten Landkreise sind im tatsächlichen Antworttext enthalten. Zusätzlich werden korrekte Zusatzinfos („Oberbayern liegt in Bayern“) genannt.</t>
+          <t>Die Antwort nennt alle im Erwarteten aufgeführten Landkreise im Regierungsbezirk Oberbayern und enthält zusätzlich eine allgemeine Zusatzinfo (Bundesland/Deutschland), die korrekt ist.</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>0.5566</v>
+        <v>0.598</v>
       </c>
       <c r="K53" t="n">
-        <v>0.4941</v>
+        <v>0.5343</v>
       </c>
       <c r="L53" t="n">
-        <v>0.5256</v>
+        <v>0.5664</v>
       </c>
     </row>
     <row r="54">
@@ -3208,11 +3206,11 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Zum Bundesland Hessen gehören die Kreise Limburg-Weilburg, Vogelsbergkreis, Lahn-Dill-Kreis, Marburg-Biedenkopf, Gießen, Hersfeld-Rotenburg, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis, Kassel, Schwalm-Eder-Kreis, Main-Kinzig-Kreis, Darmstadt, Wiesbaden, Rheingau-Taunus-Kreis, Bergstraße, Darmstadt-Dieburg, Frankfurt am Main, Offenbach, Main-Taunus-Kreis, Odenwaldkreis, Offenbach am Main, Hochtaunuskreis, Groß-Gerau und Wetteraukreis. Hessen ist ein Bundesland in Deutschland.</t>
+          <t>Zu Hessen gehören die Kreise Limburg-Weilburg, Vogelsbergkreis, Lahn-Dill-Kreis, Marburg-Biedenkopf, Gießen, Hersfeld-Rotenburg, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis, Kassel, Schwalm-Eder-Kreis, Main-Kinzig-Kreis, Darmstadt, Wiesbaden, Rheingau-Taunus-Kreis, Bergstraße, Darmstadt-Dieburg, Frankfurt am Main, Offenbach, Main-Taunus-Kreis, Odenwaldkreis, Offenbach am Main, Hochtaunuskreis, Groß-Gerau und Wetteraukreis. Hessen ist ein Bundesland in Deutschland.</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>4.994</v>
+        <v>4.458</v>
       </c>
       <c r="G54" t="n">
         <v>1</v>
@@ -3224,17 +3222,17 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Der tatsächliche Text nennt alle in der erwarteten Antwort aufgeführten Landkreise/Kreisfreie Städte: Offenbach am Main, Groß-Gerau, Main-Taunus-Kreis, Wetteraukreis, Offenbach, Main-Kinzig-Kreis, Hochtaunuskreis, Odenwaldkreis, Darmstadt-Dieburg, Rheingau-Taunus-Kreis, Wiesbaden, Frankfurt am Main, Bergstraße, Darmstadt, Marburg-Biedenkopf, Gießen, Lahn-Dill-Kreis, Limburg-Weilburg, Vogelsbergkreis, Schwalm-Eder-Kreis, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis und Hersfeld-Rotenburg. Zusätzliche Informationen sind korrekt und schaden nicht.</t>
+          <t>Alle im Erwartungswert genannten Landkreise/Städte (Offenbach am Main, Groß-Gerau, Main-Taunus-Kreis, Wetteraukreis, Offenbach, Main-Kinzig-Kreis, Hochtaunuskreis, Odenwaldkreis, Darmstadt-Dieburg, Rheingau-Taunus-Kreis, Wiesbaden, Frankfurt am Main, Bergstraße, Darmstadt, Marburg-Biedenkopf, Gießen, Lahn-Dill-Kreis, Limburg-Weilburg, Vogelsbergkreis, Schwalm-Eder-Kreis, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis, Hersfeld-Rotenburg) sind im Antworttext enthalten; zusätzliche Info ist nur korrekt.</t>
         </is>
       </c>
       <c r="J54" t="n">
-        <v>0.7082000000000001</v>
+        <v>0.705</v>
       </c>
       <c r="K54" t="n">
-        <v>0.7208</v>
+        <v>0.7151</v>
       </c>
       <c r="L54" t="n">
-        <v>0.7149</v>
+        <v>0.7105</v>
       </c>
     </row>
     <row r="55">
@@ -3264,7 +3262,7 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>9.224</v>
+        <v>5.838</v>
       </c>
       <c r="G55" t="n">
         <v>1</v>
@@ -3276,7 +3274,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Die ACTUAL-Antwort nennt exakt alle in der EXPECTED-Antwort genannten Gemeinden: Wilster, Krempermarsch, Itzehoe-Land, Horst-Herzhorn, Breitenburg, Schenefeld, Wilstermarsch, Glückstadt, Kellinghusen und Itzehoe; zusätzlich werden noch Kontextinformationen zum Bundesland gegeben.</t>
+          <t>Alle im EXPECTED genannten Verwaltungsgemeinden sind auch im ACTUAL enthalten (Wilster, Krempermarsch, Itzehoe-Land, Horst-Herzhorn, Breitenburg, Schenefeld, Wilstermarsch, Glückstadt, Kellinghusen, Itzehoe) sowie zusätzliche korrekte Zusatzinformation.</t>
         </is>
       </c>
       <c r="J55" t="n">
@@ -3312,11 +3310,11 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Zum Kreis Paderborn gehören 10 Städte: Altenbeken, Hövelhof, Borchen, Delbrück, Paderborn, Büren, Bad Wünnenberg, Lichtenau, Salzkotten und Bad Lippspringe. Der Kreis Paderborn liegt im Regierungsbezirk und im Bundesland Nordrhein-Westfalen in Deutschland.</t>
+          <t>Zum Kreis Paderborn gehören 10 Städte: Altenbeken, Hövelhof, Borchen, Delbrück, Paderborn, Büren, Bad Wünnenberg, Lichtenau, Salzkotten und Bad Lippspringe. Der Kreis Paderborn liegt im Regierungsbezirk Detmold im Bundesland Nordrhein-Westfalen in Deutschland.</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>4.984</v>
+        <v>4.1</v>
       </c>
       <c r="G56" t="n">
         <v>1</v>
@@ -3328,17 +3326,17 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Die ACTUAL-Antwort nennt alle 10 Städte des Kreises Paderborn genau wie in der EXPECTED-Antwort (inkl. Paderborn, Bad Lippspringe, Borchen, Büren, Altenbeken, Hövelhof, Lichtenau, Bad Wünnenberg, Salzkotten, Delbrück). Zusatzinfo ist korrekt und ändert nichts am geforderten Inhalt.</t>
+          <t>Die tatsächliche Antwort nennt alle 10 erwarteten Städte im Kreis Paderborn; zusätzlich enthält sie korrektes Zusatzwissen zum Regierungsbezirk und Bundesland.</t>
         </is>
       </c>
       <c r="J56" t="n">
-        <v>0.6377</v>
+        <v>0.6049</v>
       </c>
       <c r="K56" t="n">
-        <v>0.7635</v>
+        <v>0.7534</v>
       </c>
       <c r="L56" t="n">
-        <v>0.6994</v>
+        <v>0.6773</v>
       </c>
     </row>
     <row r="57">
@@ -3364,33 +3362,33 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Ja, Dülmen liegt im Kreis Coesfeld. Dülmen ist eine Stadt im Kreis Coesfeld, im Bundesland Nordrhein-Westfalen, in Deutschland als Bundesstaat.</t>
+          <t>Nein, es wurde keine Geometrie gefunden.</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>7.639</v>
+        <v>4.115</v>
       </c>
       <c r="G57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Die Antwort bestätigt korrekt, dass Dülmen im Kreis Coesfeld liegt; die zusätzliche Information ist ebenfalls korrekt.</t>
+          <t>Die erwartete Aussage (Dülmen liegt im Kreis Coesfeld) wird in der tatsächlichen Antwort verneint bzw. nicht bestätigt; zudem wird keine Geometrie gefunden.</t>
         </is>
       </c>
       <c r="J57" t="n">
-        <v>0.4172</v>
+        <v>0.09569999999999999</v>
       </c>
       <c r="K57" t="n">
-        <v>0.5954</v>
+        <v>0.0251</v>
       </c>
       <c r="L57" t="n">
-        <v>0.5034999999999999</v>
+        <v>0.0611</v>
       </c>
     </row>
     <row r="58">
@@ -3416,11 +3414,11 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Ja, der Kreis Coesfeld befindet sich im Regierungsbezirk Münster, im Bundesland Nordrhein-Westfalen in Deutschland.</t>
+          <t>Ja, der Kreis Coesfeld liegt im Regierungsbezirk Münster in Nordrhein-Westfalen in Deutschland.</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>5.413</v>
+        <v>4.125</v>
       </c>
       <c r="G58" t="n">
         <v>1</v>
@@ -3432,17 +3430,17 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort bestätigt korrekt, dass der Kreis Coesfeld im Regierungsbezirk Münster liegt; zusätzliche genaue Orts-/Landangaben sind ebenfalls korrekt.</t>
+          <t>Die tatsächliche Antwort bestätigt ebenfalls, dass der Kreis Coesfeld im Regierungsbezirk Münster liegt; die zusätzlichen Ortsangaben sind korrekt und beeinträchtigen die Übereinstimmung nicht.</t>
         </is>
       </c>
       <c r="J58" t="n">
-        <v>0.5599</v>
+        <v>0.5603</v>
       </c>
       <c r="K58" t="n">
-        <v>0.8139</v>
+        <v>0.8003</v>
       </c>
       <c r="L58" t="n">
-        <v>0.6807</v>
+        <v>0.6748</v>
       </c>
     </row>
     <row r="59">
@@ -3468,11 +3466,11 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Ja. Der Regierungsbezirk Oberfranken liegt im Bundesland Bayern, und Bayern liegt in Deutschland als Bundesstaat.</t>
+          <t>Ja. Oberfranken ist ein Regierungsbezirk im Bundesland Bayern in Deutschland.</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>5.835</v>
+        <v>3.767</v>
       </c>
       <c r="G59" t="n">
         <v>1</v>
@@ -3484,17 +3482,17 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort bestätigt korrekt, dass der Regierungsbezirk Oberfranken zum Bundesland Bayern gehört.</t>
+          <t>Die Antwort bestätigt korrekt, dass Oberfranken ein Regierungsbezirk im Bundesland Bayern ist.</t>
         </is>
       </c>
       <c r="J59" t="n">
-        <v>0.371</v>
+        <v>0.5018</v>
       </c>
       <c r="K59" t="n">
-        <v>0.5078</v>
+        <v>0.5219</v>
       </c>
       <c r="L59" t="n">
-        <v>0.4381</v>
+        <v>0.5125</v>
       </c>
     </row>
     <row r="60">
@@ -3524,7 +3522,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>4.788</v>
+        <v>4.35</v>
       </c>
       <c r="G60" t="n">
         <v>0</v>
@@ -3536,7 +3534,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort verneint die Frage und enthält keine Information, dass der Kreis Steinfurt in Nordrhein-Westfalen liegt.</t>
+          <t>Die Antwort verneint die Frage und enthält nicht die erwartete Information, dass der Kreis Steinfurt in Nordrhein-Westfalen liegt.</t>
         </is>
       </c>
       <c r="J60" t="n">
@@ -3572,11 +3570,11 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Nein, Bocholt liegt nicht im Kreis Cloppenburg. Bocholt ist eine Stadt und liegt im Bundesland Nordrhein-Westfalen in Deutschland, also im Bundesstaat Deutschland.</t>
+          <t>Nein, Bocholt liegt nicht im Kreis Cloppenburg. Bocholt ist eine Stadt und liegt in Deutschland.</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>6.385</v>
+        <v>4.226</v>
       </c>
       <c r="G61" t="n">
         <v>1</v>
@@ -3588,17 +3586,17 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort enthält die erwartete Information: Bocholt liegt nicht im Kreis Cloppenburg. Zusatzinfos sind korrekt und stören nicht.</t>
+          <t>Die tatsächliche Antwort stimmt mit der erwarteten überein: Bocholt liegt nicht im Kreis Cloppenburg. Zusätzliche Information ist korrekt.</t>
         </is>
       </c>
       <c r="J61" t="n">
-        <v>0.4532</v>
+        <v>0.617</v>
       </c>
       <c r="K61" t="n">
-        <v>0.7467</v>
+        <v>0.7914</v>
       </c>
       <c r="L61" t="n">
-        <v>0.5913</v>
+        <v>0.7015</v>
       </c>
     </row>
     <row r="62">
@@ -3624,11 +3622,11 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Ja. Der Kreis Coesfeld grenzt an den Kreis Borken. Beide liegen im Bundesland Nordrhein-Westfalen in Deutschland.</t>
+          <t>Ja, die Kreise Coesfeld und Borken grenzen aneinander. Coesfeld liegt in einem Kreis in Deutschland, und Borken liegt ebenfalls in einem Kreis in Deutschland.</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>5.511</v>
+        <v>4.34</v>
       </c>
       <c r="G62" t="n">
         <v>1</v>
@@ -3640,17 +3638,17 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort bestätigt korrekt, dass die Kreise Coesfeld und Borken aneinander grenzen. Zusätzliche Informationen zu Bundesland und Land sind ebenfalls korrekt.</t>
+          <t>Die tatsächliche Antwort bestätigt korrekt, dass der Kreis Coesfeld und der Kreis Borken aneinandergrenzen. Zusatzinformationen sind korrekt und beeinträchtigen nicht die Antwort.</t>
         </is>
       </c>
       <c r="J62" t="n">
-        <v>0.2942</v>
+        <v>0.3705</v>
       </c>
       <c r="K62" t="n">
-        <v>0.4198</v>
+        <v>0.6338</v>
       </c>
       <c r="L62" t="n">
-        <v>0.3561</v>
+        <v>0.4951</v>
       </c>
     </row>
     <row r="63">
@@ -3676,11 +3674,11 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Hallo. Dieser Chatbot beantwortet nur Fragen zu den Geometrien Deutschlands. Bitte versuche es mit einer anderen Frage.</t>
+          <t>Hallo. Dieser Chatbot beantwortet nur Fragen zu den Geometrien Deutschlands. Bitte versuchen Sie es mit einer anderen Frage.</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>4.776</v>
+        <v>4.008</v>
       </c>
       <c r="G63" t="n">
         <v>0</v>
@@ -3692,17 +3690,17 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort beantwortet die Frage nicht und liefert keine Informationen zu Senden und Münster.</t>
+          <t>Die tatsächliche Antwort enthält keine Aussage darüber, ob Senden und Münster geografisch getrennt sind oder nebeneinander liegen.</t>
         </is>
       </c>
       <c r="J63" t="n">
-        <v>-0.0327</v>
+        <v>-0.0277</v>
       </c>
       <c r="K63" t="n">
-        <v>0.1522</v>
+        <v>0.1512</v>
       </c>
       <c r="L63" t="n">
-        <v>0.0564</v>
+        <v>0.0587</v>
       </c>
     </row>
     <row r="64">
@@ -3728,11 +3726,11 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Ja. Niedersachsen grenzt an Nordrhein-Westfalen. Beide sind Bundesländer in Deutschland, einem Bundesstaat.</t>
+          <t>Ja, Niedersachsen grenzt an Nordrhein-Westfalen. Beide sind Bundesländer in Deutschland.</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>5.344</v>
+        <v>4.966</v>
       </c>
       <c r="G64" t="n">
         <v>1</v>
@@ -3744,17 +3742,17 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Die ACTUAL-Antwort bestätigt korrekt, dass Niedersachsen an Nordrhein-Westfalen grenzt. Die Zusatzinformation ist ebenfalls korrekt.</t>
+          <t>Die tatsächliche Antwort bestätigt korrekt, dass Niedersachsen an Nordrhein-Westfalen grenzt. Die Zusatzinformation ist ebenfalls korrekt.</t>
         </is>
       </c>
       <c r="J64" t="n">
-        <v>0.3631</v>
+        <v>0.4794</v>
       </c>
       <c r="K64" t="n">
-        <v>0.5198</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="L64" t="n">
-        <v>0.4395</v>
+        <v>0.5182</v>
       </c>
     </row>
     <row r="65">
@@ -3780,11 +3778,11 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Nein. Berlin ist hier mit Schöneiche bei Berlin und Neuenhagen bei Berlin verbunden; beide sind Städte und liegen im Bundesland Brandenburg in Deutschland.</t>
+          <t>Nein. Berlin ist hier als Stadt genannt und hat Schöneiche bei Berlin sowie Neuenhagen bei Berlin als zugehörige Orte. Diese beiden Orte liegen im Kreis, im Bundesland Brandenburg und im Bundesstaat Deutschland.</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>6.827</v>
+        <v>4.854</v>
       </c>
       <c r="G65" t="n">
         <v>0</v>
@@ -3796,17 +3794,17 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Die erwartete Aussage ist „Ja“, die tatsächliche Antwort sagt jedoch „Nein“ und nennt Bezüge zu Schöneiche und Neuenhagen. Damit fehlt die Information „Berlin ist vollständig von Brandenburg umgeben“.</t>
+          <t>Die erwartete Antwort ist „Ja“, die tatsächliche Antwort lautet jedoch „Nein“ und fügt zudem weitere Details hinzu, die die Erwartung nicht erfüllen.</t>
         </is>
       </c>
       <c r="J65" t="n">
-        <v>0.0495</v>
+        <v>-0.0186</v>
       </c>
       <c r="K65" t="n">
-        <v>0.3722</v>
+        <v>0.2917</v>
       </c>
       <c r="L65" t="n">
-        <v>0.1986</v>
+        <v>0.1249</v>
       </c>
     </row>
     <row r="66">
@@ -3832,11 +3830,11 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Ja, Münster liegt nördlich von Dortmund. Beide Städte liegen in Nordrhein-Westfalen, einem Bundesland Deutschlands, und damit in Deutschland, einem Bundesstaat.</t>
+          <t>Ja, Münster liegt nördlich von Dortmund. Beide Städte liegen in Deutschland; die hier angegebenen Informationen enthalten jedoch keine weiteren Hierarchieebenen wie Kreis, Regierungsbezirk, Bundesland oder Bundesstaat.</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>10.639</v>
+        <v>5.076</v>
       </c>
       <c r="G66" t="n">
         <v>1</v>
@@ -3848,17 +3846,17 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort bestätigt korrekt, dass Münster nördlich von Dortmund liegt. Zusätzliche, aber korrekte Zusatzinformationen zu Nordrhein-Westfalen und Deutschland sind enthalten.</t>
+          <t>Die ACTUAL-Antwort bestätigt die erwartete Aussage, dass Münster nördlich von Dortmund liegt; die zusätzlichen Informationen sind korrekt und beeinträchtigen die Kernaussage nicht.</t>
         </is>
       </c>
       <c r="J66" t="n">
-        <v>0.2627</v>
+        <v>0.0091</v>
       </c>
       <c r="K66" t="n">
-        <v>0.7693</v>
+        <v>0.6775</v>
       </c>
       <c r="L66" t="n">
-        <v>0.4881</v>
+        <v>0.2902</v>
       </c>
     </row>
     <row r="67">
@@ -3884,11 +3882,11 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Greven liegt direkt nördlich von Münster. Greven liegt im Bundesland Nordrhein-Westfalen in Deutschland. Münster liegt im Bundesland Nordrhein-Westfalen in Deutschland.</t>
+          <t>Greven liegt direkt nördlich von Münster. Greven liegt im Kreis Steinfurt, im Regierungsbezirk Münster, im Bundesland Nordrhein-Westfalen in Deutschland. Münster liegt ebenfalls im Kreis Steinfurt, im Regierungsbezirk Münster, im Bundesland Nordrhein-Westfalen in Deutschland.</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>7.706</v>
+        <v>5.765</v>
       </c>
       <c r="G67" t="n">
         <v>1</v>
@@ -3900,17 +3898,17 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort nennt korrekt, dass Greven direkt nördlich von Münster liegt. Zusätzliche, sachlich richtige Zusatzinformationen werden ebenfalls angegeben.</t>
+          <t>Die ACTUAL-Antwort stimmt mit der EXPECTED-Antwort überein: Greven liegt direkt nördlich von Münster. Zusätzliche korrekte Kontextinformationen sind enthalten.</t>
         </is>
       </c>
       <c r="J67" t="n">
-        <v>0.2166</v>
+        <v>0.1011</v>
       </c>
       <c r="K67" t="n">
-        <v>0.6991000000000001</v>
+        <v>0.7094</v>
       </c>
       <c r="L67" t="n">
-        <v>0.432</v>
+        <v>0.3627</v>
       </c>
     </row>
     <row r="68">
@@ -3936,11 +3934,11 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Ja, Leipzig liegt nordöstlich von Erfurt.</t>
+          <t>Ja, Leipzig liegt nordöstlich von Erfurt. Beide Orte liegen in Deutschland.</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>6.731</v>
+        <v>5.74</v>
       </c>
       <c r="G68" t="n">
         <v>1</v>
@@ -3952,17 +3950,17 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort entspricht der erwarteten Aussage (Leipzig liegt nordöstlich von Erfurt).</t>
+          <t>Die tatsächliche Antwort bestätigt wie erwartet, dass Leipzig nordöstlich (östlich) von Erfurt liegt. Zusätzliche, korrekte Information über den Standort in Deutschland ist enthalten.</t>
         </is>
       </c>
       <c r="J68" t="n">
-        <v>1</v>
+        <v>0.5986</v>
       </c>
       <c r="K68" t="n">
-        <v>1</v>
+        <v>0.8682</v>
       </c>
       <c r="L68" t="n">
-        <v>1</v>
+        <v>0.7264</v>
       </c>
     </row>
     <row r="69">
@@ -3988,11 +3986,11 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Köln liegt in Deutschland. Bonn liegt in Deutschland. Die Entfernung zwischen Köln und Bonn beträgt 6,63 km.</t>
+          <t>Köln und Bonn liegen beide in Deutschland. Köln liegt im Bundesland Nordrhein-Westfalen in Deutschland, und Bonn liegt ebenfalls im Bundesland Nordrhein-Westfalen in Deutschland. Die Entfernung zwischen Köln und Bonn beträgt 6,63 km.</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>16.098</v>
+        <v>15.154</v>
       </c>
       <c r="G69" t="n">
         <v>1</v>
@@ -4004,17 +4002,17 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort nennt die Entfernung zwischen Köln und Bonn mit 6,63 km wie in der erwarteten Antwort. Zusatzinformationen sind ebenfalls korrekt.</t>
+          <t>Die tatsächliche Antwort nennt die Entfernung zwischen Köln und Bonn korrekt mit 6,63 km; Zusatzinformationen sind ebenfalls korrekt.</t>
         </is>
       </c>
       <c r="J69" t="n">
-        <v>0.5318000000000001</v>
+        <v>0.2695</v>
       </c>
       <c r="K69" t="n">
-        <v>0.6706</v>
+        <v>0.6516</v>
       </c>
       <c r="L69" t="n">
-        <v>0.5997</v>
+        <v>0.4447</v>
       </c>
     </row>
     <row r="70">
@@ -4044,7 +4042,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>13.187</v>
+        <v>11.546</v>
       </c>
       <c r="G70" t="n">
         <v>1</v>
@@ -4056,7 +4054,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Der ACTUAL-Text nennt die Entfernung Hannover–Braunschweig mit 34,92 km, was exakt dem EXPECTED entspricht.</t>
+          <t>Die tatsächliche Antwort enthält die erwartete Entfernung von 34,92 km zwischen Hannover und Braunschweig.</t>
         </is>
       </c>
       <c r="J70" t="n">
@@ -4092,11 +4090,11 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Hessen liegt als Bundesland in Deutschland, und Thüringen liegt ebenfalls als Bundesland in Deutschland. Die Entfernung zwischen Hessen und Thüringen beträgt 0,0 km.</t>
+          <t>Hessen liegt im Bundesland Hessen in Deutschland, und Thüringen liegt im Bundesland Thüringen in Deutschland. Die Entfernung zwischen Hessen und Thüringen beträgt 0,0 km.</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>22.258</v>
+        <v>11.726</v>
       </c>
       <c r="G71" t="n">
         <v>1</v>
@@ -4108,17 +4106,17 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort nennt dieselbe Entfernung von 0,0 km wie erwartet und stimmt inhaltlich überein.</t>
+          <t>Die tatsächliche Antwort nennt die Entfernung zwischen Hessen und Thüringen ebenfalls als 0,0 km, wie erwartet (Zusatzinformationen sind korrekt).</t>
         </is>
       </c>
       <c r="J71" t="n">
-        <v>0.3331</v>
+        <v>0.3138</v>
       </c>
       <c r="K71" t="n">
-        <v>0.3596</v>
+        <v>0.309</v>
       </c>
       <c r="L71" t="n">
-        <v>0.3473</v>
+        <v>0.3125</v>
       </c>
     </row>
     <row r="72">
@@ -4144,11 +4142,11 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Die drei nächstgelegenen Landkreise zu Miesbach sind München, Bad Tölz-Wolfratshausen und Rosenheim. Miesbach liegt im Bundesland Bayern in Deutschland. München, Bad Tölz-Wolfratshausen und Rosenheim liegen ebenfalls im Bundesland Bayern in Deutschland.</t>
+          <t>Die Gemeinde Miesbach liegt im Kreis Miesbach. Die drei nächstgelegenen Kreise sind München, Bad Tölz-Wolfratshausen und Rosenheim. Diese Kreise liegen im Bundesland Bayern in Deutschland.</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>4.91</v>
+        <v>4.821</v>
       </c>
       <c r="G72" t="n">
         <v>1</v>
@@ -4160,17 +4158,17 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Die ACTUAL-Antwort nennt genau dieselben drei Landkreise wie erwartet: Bad Tölz-Wolfratshausen, München und Rosenheim.</t>
+          <t>Der tatsächliche Antworttext nennt genau dieselben drei nächstgelegenen Landkreise wie erwartet: München, Bad Tölz-Wolfratshausen und Rosenheim. Zusätzliche Infos zur Lage in Bayern sind korrekt und beeinträchtigen die Vergleichsprüfung nicht.</t>
         </is>
       </c>
       <c r="J72" t="n">
-        <v>0.3825</v>
+        <v>0.4737</v>
       </c>
       <c r="K72" t="n">
-        <v>0.5397999999999999</v>
+        <v>0.6375999999999999</v>
       </c>
       <c r="L72" t="n">
-        <v>0.4591</v>
+        <v>0.5534</v>
       </c>
     </row>
     <row r="73">
@@ -4196,14 +4194,14 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Der Kreis Warendorf grenzt an die Kreise Gütersloh, Steinfurt, Soest, Coesfeld und Osnabrück sowie an die Städte Münster und Hamm. Warendorf liegt in Deutschland.</t>
+          <t>Der Landkreis Warendorf grenzt an die Kreise Gütersloh, Steinfurt, Soest, Coesfeld, Osnabrück, Münster und Hamm. Der Landkreis Warendorf liegt im Bundesland Nordrhein-Westfalen in Deutschland. Die genannten Kreise liegen ebenfalls in Deutschland.</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>4.976</v>
+        <v>4.061</v>
       </c>
       <c r="G73" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
@@ -4212,17 +4210,17 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Die genannten Nachbarkreise stimmen weitgehend überein (Gütersloh, Steinfurt, Soest, Coesfeld, Osnabrück sowie zusätzlich Münster und Hamm). In der erwarteten Antwort fehlt nur der Hinweis, dass Münster auch als Landkreis genannt ist; die tatsächliche Antwort nennt Münster als Stadt.</t>
+          <t>Die Liste der angrenzenden Kreise stimmt vollständig überein (Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld, Soest). Zusätzliche allgemeine Angaben sind korrekt und nicht widersprüchlich.</t>
         </is>
       </c>
       <c r="J73" t="n">
-        <v>0.6743</v>
+        <v>0.5521</v>
       </c>
       <c r="K73" t="n">
-        <v>0.7824</v>
+        <v>0.7944</v>
       </c>
       <c r="L73" t="n">
-        <v>0.7276</v>
+        <v>0.6676</v>
       </c>
     </row>
     <row r="74">
@@ -4248,33 +4246,33 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Es wurden keine benachbarten Verwaltungsbezirke gefunden.</t>
+          <t>An den Verwaltungsbezirk Leezen grenzen die Verwaltungsgemeinden Bad Oldesloe-Land, Trave-Land, Boostedt-Rickling, Auenland Südholstein, Wahlstedt, Kisdorf, Bad Segeberg, Itzstedt und Buchholz (Forstgutsbez.). Leezen liegt in Deutschland.</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>9.965999999999999</v>
+        <v>5.418</v>
       </c>
       <c r="G74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort nennt keine benachbarten Verwaltungsbezirke, während im Erwarteten mehrere konkrete Verwaltungsbezirke aufgelistet sind.</t>
+          <t>Die Auflistung der angrenzenden Verwaltungsbezirke/Gemeinden stimmt mit der erwarteten Liste überein (inkl. Buchholz Forstgutsbezirk) und enthält keine abweichenden Punkte; zusätzliche allgemeine Information („Leezen liegt in Deutschland“) ist korrekt.</t>
         </is>
       </c>
       <c r="J74" t="n">
-        <v>0.2451</v>
+        <v>0.6208</v>
       </c>
       <c r="K74" t="n">
-        <v>-0.1763</v>
+        <v>0.7161</v>
       </c>
       <c r="L74" t="n">
-        <v>0.0105</v>
+        <v>0.668</v>
       </c>
     </row>
     <row r="75">
@@ -4300,11 +4298,11 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Mittelfranken ist von den Verwaltungsbezirken Oberpfalz, Oberbayern, Schwaben, Oberfranken, Unterfranken und Stuttgart umgeben. Mittelfranken liegt im Bundesland Bayern in Deutschland.</t>
+          <t>Mittelfranken ist von den Regierungsbezirken Oberpfalz, Oberbayern, Schwaben, Oberfranken, Unterfranken und Stuttgart umgeben. Alle gehören auf der Ebene der Regierungsbezirke zum Bundesland Bayern beziehungsweise zu einem weiteren Regierungsbezirk; die höchste genannte Ebene ist Deutschland als Bundesstaat.</t>
         </is>
       </c>
       <c r="F75" t="n">
-        <v>15.931</v>
+        <v>4.397</v>
       </c>
       <c r="G75" t="n">
         <v>0</v>
@@ -4316,17 +4314,17 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Die erwartete Antwort beschreibt nur die Umgebenden als Bundesland Bayern, während die tatsächliche Antwort die umgebenden Verwaltungsbezirke konkret aufzählt (u.a. Oberpfalz, Oberbayern, Schwaben usw.). Damit enthält die tatsächliche Antwort nicht die geforderte Information zur Umfassung durch Bayern.</t>
+          <t>Die erwartete Antwort erwähnt nur „Bayern“ als Umgebung, während die tatsächliche Antwort stattdessen einzelne Regierungsbezirke aufzählt. Damit enthält die tatsächliche Antwort nicht die erwartete Aussage, dass Mittelfranken von Bayern (bzw. einem Bundesland) umgeben ist.</t>
         </is>
       </c>
       <c r="J75" t="n">
-        <v>0.3477</v>
+        <v>0.1961</v>
       </c>
       <c r="K75" t="n">
-        <v>0.4534</v>
+        <v>0.4122</v>
       </c>
       <c r="L75" t="n">
-        <v>0.4001</v>
+        <v>0.2995</v>
       </c>
     </row>
     <row r="76">
@@ -4352,11 +4350,11 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Nördlich von Thüringen liegen Mecklenburg-Vorpommern, Sachsen-Anhalt, Schleswig-Holstein und Hamburg. Thüringen liegt im Bundesland Thüringen in Deutschland. Die genannten Bundesländer liegen in Deutschland.</t>
+          <t>Nördlich von Thüringen liegen Schleswig-Holstein, Sachsen-Anhalt, Mecklenburg-Vorpommern und Hamburg. Alle genannten Bundesländer liegen in Deutschland.</t>
         </is>
       </c>
       <c r="F76" t="n">
-        <v>52.766</v>
+        <v>32.25</v>
       </c>
       <c r="G76" t="n">
         <v>1</v>
@@ -4368,17 +4366,17 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Die ACTUAL-Antwort nennt genau die vier Bundesländer, die nördlich von Thüringen liegen: Mecklenburg-Vorpommern, Sachsen-Anhalt, Schleswig-Holstein und Hamburg.</t>
+          <t>Alle im Erwarteten genannten Bundesländer (Hamburg, Schleswig-Holstein, Mecklenburg-Vorpommern, Sachsen-Anhalt) werden im tatsächlichen Text vollständig genannt; lediglich die Reihenfolge und eine zusätzliche allgemeine Aussage („liegen in Deutschland“) sind anders.</t>
         </is>
       </c>
       <c r="J76" t="n">
-        <v>0.4955</v>
+        <v>0.6244</v>
       </c>
       <c r="K76" t="n">
-        <v>0.6556999999999999</v>
+        <v>0.7352</v>
       </c>
       <c r="L76" t="n">
-        <v>0.5735</v>
+        <v>0.679</v>
       </c>
     </row>
     <row r="77">
@@ -4404,11 +4402,11 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Westlich vom Landkreis Münster liegen der Kreis Kleve und der Kreis Borken. Beide liegen im Bundesland Nordrhein-Westfalen in Deutschland.</t>
+          <t>Westlich vom Kreis Münster liegen der Kreis Kleve und der Kreis Borken. Beide liegen im Bundesland Nordrhein-Westfalen in Deutschland.</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>67.419</v>
+        <v>33.134</v>
       </c>
       <c r="G77" t="n">
         <v>1</v>
@@ -4420,17 +4418,17 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Der tatsächliche Text nennt genau die Kreise Kleve und Borken als westlich von Münster liegend; die zusätzliche Information zu Bundesland und Deutschland ist korrekt und ändert den Inhalt nicht.</t>
+          <t>Der tatsächliche Antworttext nennt genau die Kreise Kleve und Borken als westlich von Münster liegend; die Zusatzinfo zu Bundesland/Deutschland ist korrekt und deckt die Erwartung vollständig ab.</t>
         </is>
       </c>
       <c r="J77" t="n">
-        <v>0.3644</v>
+        <v>0.3656</v>
       </c>
       <c r="K77" t="n">
-        <v>0.5992</v>
+        <v>0.591</v>
       </c>
       <c r="L77" t="n">
-        <v>0.4763</v>
+        <v>0.4733</v>
       </c>
     </row>
     <row r="78">
@@ -4456,11 +4454,11 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Nördlich der Verwaltungsgemeinschaft Kiel liegen die Verwaltungsgemeinden Geltinger Bucht, Dänischenhagen, Altenholz und Kappeln. Kiel ist ebenfalls als Verwaltungsgemeinde aufgeführt. Alle diese Verwaltungsgemeinden liegen in Deutschland.</t>
+          <t>Nördlich der Verwaltungsgemeinschaft Kiel liegen die Verwaltungsgemeinschaften Geltinger Bucht, Altenholz, Dänischenhagen und Kappeln. Kiel ist ebenfalls in der Liste enthalten. Alle genannten Verwaltungsgemeinschaften liegen in einem Kreis, einem Bundesland und in Deutschland als Bundesstaat.</t>
         </is>
       </c>
       <c r="F78" t="n">
-        <v>67.57299999999999</v>
+        <v>31.133</v>
       </c>
       <c r="G78" t="n">
         <v>1</v>
@@ -4472,17 +4470,17 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Die Antwort nennt alle erwarteten Verwaltungsgemeinschaften (Altenholz, Dänischenhagen, Kappeln, Geltinger Bucht) korrekt; die Zusatzinfo „Kiel ist ebenfalls aufgeführt“ ist nicht relevant für die geforderten nördlichen Gemeinden.</t>
+          <t>Die ACTUAL-Antwort nennt alle in der EXPECTED-Antwort genannten Verwaltungsgemeinschaften (Altenholz, Dänischenhagen, Kappeln, Geltinger Bucht) und zusätzlich die Information, dass Kiel selbst in der Liste enthalten ist sowie weitere korrekte Zusatzangaben.</t>
         </is>
       </c>
       <c r="J78" t="n">
-        <v>0.5148</v>
+        <v>0.3409</v>
       </c>
       <c r="K78" t="n">
-        <v>0.6476</v>
+        <v>0.5755</v>
       </c>
       <c r="L78" t="n">
-        <v>0.5799</v>
+        <v>0.4527</v>
       </c>
     </row>
     <row r="79">
@@ -4508,11 +4506,11 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Um den Kreis Göttingen liegen die Kreise Northeim, Kassel, Goslar, Nordhausen, Werra-Meißner-Kreis, Eichsfeld und Harz. Außerdem ist Kassel zweimal genannt. Der Kreis Göttingen liegt im Regierungsbezirk, in einem Bundesland und in Deutschland als Bundesstaat.</t>
+          <t>Zum Kreis Göttingen gehören im Umkreis von 10 km folgende Kreise: Harz, Eichsfeld, Kassel, Werra-Meißner-Kreis, Kassel, Northeim, Nordhausen und Goslar. Göttingen liegt im Bundesland Niedersachsen in Deutschland.</t>
         </is>
       </c>
       <c r="F79" t="n">
-        <v>58.418</v>
+        <v>39.477</v>
       </c>
       <c r="G79" t="n">
         <v>1</v>
@@ -4524,17 +4522,17 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Die tatsächliche Antwort nennt alle im erwarteten Text genannten Landkreise (Harz, Northeim, Goslar, Kassel, Eichsfeld, Werra-Meißner-Kreis, Nordhausen). Zusätzliche Angaben sind irrelevant, aber nicht falsch.</t>
+          <t>Die im Umkreis von 10 km genannten Landkreise stimmen mit der Erwartung überein: Harz, Northeim, Goslar, Kassel, Eichsfeld, Werra-Meißner-Kreis und Nordhausen; zusätzliche Erläuterungen sind korrekt und betreffen nicht die geforderte Liste.</t>
         </is>
       </c>
       <c r="J79" t="n">
-        <v>0.4894</v>
+        <v>0.6957</v>
       </c>
       <c r="K79" t="n">
-        <v>0.6087</v>
+        <v>0.781</v>
       </c>
       <c r="L79" t="n">
-        <v>0.5482</v>
+        <v>0.738</v>
       </c>
     </row>
     <row r="80">
@@ -4560,11 +4558,11 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Um Aachen liegen im Umkreis von 5 km die Städte Würselen, Alsdorf, Roetgen, Herzogenrath, Eschweiler, Hürtgenwald, Stolberg (Rhld.) und Simmerath. Aachen liegt in keinem weiteren hier angegebenen übergeordneten Gebiet.</t>
+          <t>Um Aachen liegen Stolberg (Rhld.), Würselen, Alsdorf, Simmerath, Hürtgenwald, Eschweiler, Roetgen und Herzogenrath. Aachen und diese Städte liegen im Kreis Aachen, im Regierungsbezirk Köln, im Bundesland Nordrhein-Westfalen, in Deutschland.</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>58.098</v>
+        <v>38.823</v>
       </c>
       <c r="G80" t="n">
         <v>1</v>
@@ -4576,17 +4574,17 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Die ACTUAL-Antwort nennt alle Städte aus der EXPECTED-Liste (Alsdorf, Simmerath, Würselen, Hürtgenwald, Roetgen, Herzogenrath, Eschweiler, Stolberg (Rhld.)) innerhalb des 5-km-Umkreises um Aachen; Zusatzinformation beeinträchtigt nicht die Vollständigkeit.</t>
+          <t>Die ACTUAL-Antwort nennt alle in der EXPECTED-Antwort aufgeführten Städte im 5-km-Umkreis um Aachen: Alsdorf, Simmerath, Würselen, Hürtgenwald, Roetgen, Herzogenrath, Eschweiler und Stolberg (Rhld.). Zusätzliche allgemeine Informationen sind korrekt und ändern nichts.</t>
         </is>
       </c>
       <c r="J80" t="n">
-        <v>0.5743</v>
+        <v>0.5137</v>
       </c>
       <c r="K80" t="n">
-        <v>0.6949</v>
+        <v>0.5826</v>
       </c>
       <c r="L80" t="n">
-        <v>0.6336000000000001</v>
+        <v>0.5483</v>
       </c>
     </row>
     <row r="81">
@@ -4612,15 +4610,14 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>In einem Umkreis von weniger als 2 km um München liegen Krailling, Hebertshausen, Putzbrunn, Gräfelfing, Pullach i.Isartal, Bergkirchen, Ottobrunn, Haar, Gröbenzell, Vaterstetten, Karlsfeld, Planegg, Puchheim, Grünwalder Forst, Neubiberg, Oberschleißheim, Germering, Perlacher Forst, Dachau, Feldkirchen, Olching, Unterföhring, Unterhaching, Garching b.München, Ismaning, Neuried, Hohenbrunn, Forstenrieder Park, Aschheim, Grünwald und Grasbrunn.
-München ist eine Stadt in einem Kreis in einem Regierungsbezirk in Bayern in Deutschland.</t>
+          <t>Ja, es gibt Städte in einem Umkreis von weniger als 2 km um München. Genannt werden Vaterstetten, Ottobrunn, Gräfelfing, Pullach i.Isartal, Hohenbrunn, Neuried, Hebertshausen, Gröbenzell, Haar, Neubiberg, Unterföhring, Ismaning, Olching, Forstenrieder Park, Karlsfeld, Aschheim, Dachau, Grünwald, Germering, Grünwalder Forst, Grasbrunn, Perlacher Forst, Oberschleißheim, Garching b.München, Feldkirchen, Bergkirchen, Putzbrunn, Krailling, Planegg, Puchheim und Unterhaching. München liegt in Bayern in Deutschland. Die genannten Orte liegen jeweils in Deutschland.</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>88.569</v>
+        <v>39.523</v>
       </c>
       <c r="G81" t="n">
-        <v>0.95</v>
+        <v>0.63</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
@@ -4629,17 +4626,17 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Die meisten erwarteten Städte sind enthalten; es fehlen jedoch Forstenrieder Park, Grünwald? (sie sind enthalten) — tatsächlich fehlen nur Aschheim? (enthalten) und weitere: Neubiberg und Putzbrunn? (Putzbrunn enthalten, Neubiberg fehlt). Außerdem ist Ottobrunn/Hebertshausen/Vaterstetten/Hohenbrunn/Grasbrunn hinzugefügt, was nicht schadet.</t>
+          <t>Die ACTUAL-Antwort enthält mehrere der EXPECTED-Städte (z.B. Forstenrieder Park, Grünwald, Feldkirchen, Aschheim, Haar, Unterhaching, Pullach i. Isartal, Bergkirchen, Neuried, Germering, Olching, Garching bei München, Planegg, Ismaning, Puchheim, Unterföhring, Gröbenzell, Neubiberg, Oberschleißheim, Putzbrunn, Perlacher Forst, Gräfelfing, Karlsfeld). Allerdings fehlen in der ACTUAL-Antwort mindestens: Puchheim ist vorhanden, aber fehlend ist u.a. Neubiberg? (ist vorhanden), es fehlen jedoch definitiv einige der EXPECTED-Einträge wie 'Gröbenzell' ist vorhanden; 'Neubiberg' ist vorhanden. Als klare Lücken fehlen 'Forstenrieder Park'? ist vorhanden. Der Hauptmangel ist: 'Gräfelfing' fehlt (stattdessen nur Gräfelfing? tatsächlich ist Gräfelfing nicht in ACTUAL genannt), 'Karlsfeld' ist vorhanden. Damit fehlen mindestens Gräfelfing; außerdem werden einige Begriffe leicht anders geschrieben, aber keine weiteren offensichtlichen fehlenden. Daher nur teilweise Übereinstimmung.</t>
         </is>
       </c>
       <c r="J81" t="n">
-        <v>0.413</v>
+        <v>0.3783</v>
       </c>
       <c r="K81" t="n">
-        <v>0.4955</v>
+        <v>0.4924</v>
       </c>
       <c r="L81" t="n">
-        <v>0.4543</v>
+        <v>0.4347</v>
       </c>
     </row>
     <row r="82">
@@ -4665,35 +4662,33 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>La ville de Münster désigne deux lieux différents :
-1. Münster se trouve dans la ville de Münster, dans le district de Münster, dans le Regierungsbezirk de Münster, dans le Bundesland de Nordrhein-Westfalen, en Allemagne.
-2. Münster se trouve dans la commune administrative de Rain, dans le district de Donau-Ries, dans le Regierungsbezirk de Schwaben, dans le Bundesland de Bayern, en Allemagne.</t>
+          <t>La ville de Münster se trouve à Münster, dans le Kreis Münster, dans le Regierungsbezirk Münster, dans le Bundesland Nordrhein-Westfalen, en Allemagne.</t>
         </is>
       </c>
       <c r="F82" t="n">
-        <v>8.83</v>
+        <v>4.818</v>
       </c>
       <c r="G82" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>L’ACTUAL mentionne bien les deux localités de Münster et donne les mêmes informations essentielles que l’EXPECTED (Rain/Donau-Ries/Souabe/Rhénanie-du-Nord-Westphalie vs Nordrhein-Westfalen), avec des termes équivalents (Land/Bundesland, circonscription/Régierungsbezirk).</t>
+          <t>L'ACTUAL réponse décrit correctement une des localités de Münster (Nordrhein-Westfalen, Münster/Kreis Münster/Regierungsbezirk Münster). En revanche, elle ne mentionne pas l'autre localité de Münster située dans la commune de Rain (Donau-Ries), en Souabe (Bavière) comme dans l'EXPECTED.</t>
         </is>
       </c>
       <c r="J82" t="n">
-        <v>0.5929</v>
+        <v>0.4274</v>
       </c>
       <c r="K82" t="n">
-        <v>0.4954</v>
+        <v>0.1766</v>
       </c>
       <c r="L82" t="n">
-        <v>0.5438</v>
+        <v>0.2952</v>
       </c>
     </row>
     <row r="83">
@@ -4719,33 +4714,33 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Cologne correspond à Köln, une ville située dans le district de Köln, dans la communauté administrative de Köln, dans le district administratif de Köln, dans le Land de Nordrhein-Westfalen, en Allemagne.</t>
+          <t>Aucune géométrie trouvée.</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>4.607</v>
+        <v>3.785</v>
       </c>
       <c r="G83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>L’ACTUAL mentionne que Cologne (Köln) se trouve dans le Land de Nordrhein-Westfalen (Rhénanie-du-Nord-Westphalie) en Allemagne. Même si le libellé de l’arrondissement est différent, l’information attendue sur la région est bien couverte.</t>
+          <t>La réponse attendue indique où se trouve Cologne (arrondissement de Cologne, Land de Rhénanie-du-Nord-Westphalie), mais la réponse réelle ne fournit aucune information.</t>
         </is>
       </c>
       <c r="J83" t="n">
-        <v>0.5061</v>
+        <v>-0.0275</v>
       </c>
       <c r="K83" t="n">
-        <v>0.4245</v>
+        <v>-0.3067</v>
       </c>
       <c r="L83" t="n">
-        <v>0.4653</v>
+        <v>-0.1779</v>
       </c>
     </row>
     <row r="84">
@@ -4771,11 +4766,11 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>La communauté de communes d’Eisenhüttenstadt se trouve à Eisenhüttenstadt, dans le district d’Oder-Spree, dans le Land de Brandebourg, en Allemagne.</t>
+          <t>La communauté de communes d’Eisenhüttenstadt se trouve à Eisenhüttenstadt, dans le district d’Oder-Spree, dans le Land de Brandebourg, en Allemagne, qui est un État souverain.</t>
         </is>
       </c>
       <c r="F84" t="n">
-        <v>4.719</v>
+        <v>5.304</v>
       </c>
       <c r="G84" t="n">
         <v>1</v>
@@ -4787,17 +4782,17 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>L’ACTUAL mentionne bien le district (arrondissement) d’Oder-Spree et le Land de Brandebourg, comme dans l’EXPECTED, et précise en plus la ville d’Eisenhüttenstadt.</t>
+          <t>L’ACTUAL indique correctement qu’elle se trouve à Eisenhüttenstadt, dans le district d’Oder-Spree, dans le Land de Brandebourg (Allemagne), ce qui correspond à l’EXPECTED. La mention que l’Allemagne est un État souverain est une information supplémentaire correcte.</t>
         </is>
       </c>
       <c r="J84" t="n">
-        <v>0.6055</v>
+        <v>0.5278</v>
       </c>
       <c r="K84" t="n">
-        <v>0.6578000000000001</v>
+        <v>0.6392</v>
       </c>
       <c r="L84" t="n">
-        <v>0.6319</v>
+        <v>0.5828</v>
       </c>
     </row>
     <row r="85">
@@ -4823,11 +4818,11 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>La communauté de communes d’Esens se trouve à Esens, dans le district de Wittmund, dans le Land de Basse-Saxe, en Allemagne.</t>
+          <t>La communauté de communes d’Esens se trouve à Esens, dans le Kreis de Wittmund, dans le Bundesland de Niedersachsen, en Allemagne.</t>
         </is>
       </c>
       <c r="F85" t="n">
-        <v>5.174</v>
+        <v>3.787</v>
       </c>
       <c r="G85" t="n">
         <v>1</v>
@@ -4839,17 +4834,17 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Les deux réponses indiquent que la communauté se situe dans le district/arrondissement de Wittmund, en Basse-Saxe (Allemagne). L’ACTUAL ajoute le fait qu’elle est à Esens, ce qui est cohérent.</t>
+          <t>L’ACTUAL précise correctement le lieu : Esens, dans le Kreis/arrondissement de Wittmund (Basse-Saxe/Niedersachsen en Allemagne), ce qui correspond à l’attendu.</t>
         </is>
       </c>
       <c r="J85" t="n">
-        <v>0.538</v>
+        <v>0.5012</v>
       </c>
       <c r="K85" t="n">
-        <v>0.6087</v>
+        <v>0.5266999999999999</v>
       </c>
       <c r="L85" t="n">
-        <v>0.5735</v>
+        <v>0.5145999999999999</v>
       </c>
     </row>
     <row r="86">
@@ -4875,11 +4870,11 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Giessen se trouve dans la ville de Gießen, dans le Land de Hessen, en Allemagne, qui est un État.</t>
+          <t>L’arrondissement de Giessen se trouve dans le district de Gießen, dans le district administratif de Gießen, dans le Land de Hessen, en Allemagne.</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>5.151</v>
+        <v>3.74</v>
       </c>
       <c r="G86" t="n">
         <v>1</v>
@@ -4891,17 +4886,17 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>L’information attendue indique que l’arrondissement de Giessen se situe dans le Land de Hesse. L’actual mentionne clairement le Land de Hessen (Hesse) en Allemagne, ce qui correspond à l’attendu.</t>
+          <t>L’ACTUAL mentionne bien que l’arrondissement de Giessen se trouve dans le Land de Hessen, comme attendu (avec des précisions supplémentaires).</t>
         </is>
       </c>
       <c r="J86" t="n">
-        <v>0.3936</v>
+        <v>0.5188</v>
       </c>
       <c r="K86" t="n">
-        <v>0.5296999999999999</v>
+        <v>0.7159</v>
       </c>
       <c r="L86" t="n">
-        <v>0.4603</v>
+        <v>0.6138</v>
       </c>
     </row>
     <row r="87">
@@ -4927,11 +4922,11 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Aucune géométrie n’a été trouvée pour l’arrondissement de Saxe du Nord.</t>
+          <t>Aucune géométrie n’a été trouvée.</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>5.09</v>
+        <v>3.796</v>
       </c>
       <c r="G87" t="n">
         <v>0</v>
@@ -4943,17 +4938,17 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>L'ACTUAL ne répond pas à la question et ne fournit aucune information sur la localisation (Land de Saxe) de l'arrondissement demandé.</t>
+          <t>L’ACTUAL ne fournit aucune information répondant à la question (indique qu’aucune géométrie n’a été trouvée).</t>
         </is>
       </c>
       <c r="J87" t="n">
-        <v>0.1121</v>
+        <v>-0.0641</v>
       </c>
       <c r="K87" t="n">
-        <v>0.2914</v>
+        <v>-0.1011</v>
       </c>
       <c r="L87" t="n">
-        <v>0.1988</v>
+        <v>-0.08119999999999999</v>
       </c>
     </row>
     <row r="88">
@@ -4983,7 +4978,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>5.347</v>
+        <v>3.687</v>
       </c>
       <c r="G88" t="n">
         <v>0</v>
@@ -4995,7 +4990,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>L’ACTUAL ne donne aucune information sur l’emplacement de la circonscription administrative de Fribourg, alors que l’attendu indique qu’il s’agit de l’arrondissement de Fribourg dans le Land de Bade-Wurtemberg.</t>
+          <t>L’ACTUAL ne fournit aucune information géographique et ne confirme pas que l’arrondissement de Fribourg se situe dans le Land de Bade-Wurtemberg.</t>
         </is>
       </c>
       <c r="J88" t="n">
@@ -5031,11 +5026,11 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Aucune géométrie trouvée.</t>
+          <t>Aucune géométrie n’a été trouvée.</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>4.74</v>
+        <v>4.699</v>
       </c>
       <c r="G89" t="n">
         <v>0</v>
@@ -5047,17 +5042,17 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>La réponse attendue indique la localisation dans le Land de Bavière, mais la réponse réelle ne fournit aucune information (aucune géométrie trouvée).</t>
+          <t>La réponse attendue précise que Haute-Franconie se situe en Bavière, mais la réponse actuelle ne fournit aucune information pertinente ("Aucune géométrie n’a été trouvée").</t>
         </is>
       </c>
       <c r="J89" t="n">
-        <v>-0.0341</v>
+        <v>-0.0607</v>
       </c>
       <c r="K89" t="n">
-        <v>-0.1249</v>
+        <v>-0.1105</v>
       </c>
       <c r="L89" t="n">
-        <v>-0.0791</v>
+        <v>-0.0843</v>
       </c>
     </row>
     <row r="90">
@@ -5083,14 +5078,14 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Le Land de Saxe se trouve en Allemagne.</t>
+          <t>Aucune géométrie n’a été trouvée.</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>6.231</v>
+        <v>4.109</v>
       </c>
       <c r="G90" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -5099,17 +5094,17 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>L’ACTUEL indique correctement que le Land de Saxe se trouve en Allemagne, mais ne donne ni la localisation “au niveau fédéral” ni les coordonnées du centre de gravité attendues.</t>
+          <t>L’ACTUAL ne fournit aucune information (pas de localisation ni de coordonnées), alors que l’EXPECTED donne le Land au niveau fédéral et des coordonnées précises du centre de gravité.</t>
         </is>
       </c>
       <c r="J90" t="n">
-        <v>0.5336</v>
+        <v>-0.0562</v>
       </c>
       <c r="K90" t="n">
-        <v>-0.1924</v>
+        <v>-0.3112</v>
       </c>
       <c r="L90" t="n">
-        <v>0.1021</v>
+        <v>-0.1925</v>
       </c>
     </row>
     <row r="91">
@@ -5139,7 +5134,7 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>4.968</v>
+        <v>3.757</v>
       </c>
       <c r="G91" t="n">
         <v>0</v>
@@ -5151,7 +5146,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>L’ACTUAL ne fournit aucune information (pas de géométrie ni de coordonnées), contrairement à l’EXPECTED qui donne les coordonnées du centre de gravité.</t>
+          <t>L’ACTUAL ne fournit ni la localisation (Land au niveau fédéral) ni les coordonnées attendues du centre de gravité.</t>
         </is>
       </c>
       <c r="J91" t="n">
@@ -5187,11 +5182,11 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>L’arrondissement de Coesfeld comprend les villes et communes de Rosendahl, Havixbeck, Senden, Billerbeck, Ascheberg, Dülmen, Nottuln, Coesfeld, Nordkirchen, Lüdinghausen et Olfen. Coesfeld est un district du Land de Rhénanie du Nord-Westphalie, en Allemagne.</t>
+          <t>Les villes de l’arrondissement de Coesfeld sont Rosendahl, Havixbeck, Senden, Billerbeck, Ascheberg, Dülmen, Nottuln, Coesfeld, Nordkirchen, Lüdinghausen et Olfen. Coesfeld est un district dans le district administratif de Münster, dans le Bundesland Nordrhein-Westfalen, en Allemagne.</t>
         </is>
       </c>
       <c r="F92" t="n">
-        <v>5.229</v>
+        <v>4.017</v>
       </c>
       <c r="G92" t="n">
         <v>1</v>
@@ -5203,17 +5198,17 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Toutes les villes listées dans l’attendu (Coesfeld, Olfen, Senden, Nottuln, Havixbeck, Nordkirchen, Billerbeck, Lüdinghausen, Rosendahl, Dülmen, Ascheberg) figurent dans la réponse, avec en plus une information contextuelle correcte.</t>
+          <t>Les villes listées dans l’ACTUAL correspondent exactement à celles de l’EXPECTED (Coesfeld, Olfen, Senden, Nottuln, Havixbeck, Nordkirchen, Billerbeck, Lüdinghausen, Rosendahl, Dülmen, Ascheberg). L’ACTUAL ajoute une information supplémentaire sur le district administratif, qui est correcte.</t>
         </is>
       </c>
       <c r="J92" t="n">
-        <v>0.543</v>
+        <v>0.5011</v>
       </c>
       <c r="K92" t="n">
-        <v>0.7684</v>
+        <v>0.6877</v>
       </c>
       <c r="L92" t="n">
-        <v>0.6509</v>
+        <v>0.5913</v>
       </c>
     </row>
     <row r="93">
@@ -5239,11 +5234,11 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Aucune géométrie n’a été trouvée pour cette recherche.</t>
+          <t>Aucune géométrie n’a été trouvée.</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>7.934</v>
+        <v>4.389</v>
       </c>
       <c r="G93" t="n">
         <v>0</v>
@@ -5255,17 +5250,17 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>La réponse réelle ne fournit aucune liste d’arrondissements ni aucune information sur la circonscription de Haute-Bavière.</t>
+          <t>L’ACTUAL ne fournit aucune liste d’arrondissements correspondant à l’EXPECTED.</t>
         </is>
       </c>
       <c r="J93" t="n">
-        <v>-0.0983</v>
+        <v>-0.1459</v>
       </c>
       <c r="K93" t="n">
-        <v>-0.4789</v>
+        <v>-0.5196</v>
       </c>
       <c r="L93" t="n">
-        <v>-0.3119</v>
+        <v>-0.356</v>
       </c>
     </row>
     <row r="94">
@@ -5291,33 +5286,33 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Le Land de Hesse se compose des arrondissements et villes suivantes : Limburg-Weilburg, Vogelsbergkreis, Lahn-Dill-Kreis, Marburg-Biedenkopf, Gießen, Hersfeld-Rotenburg, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis, Kassel, Schwalm-Eder-Kreis, Main-Kinzig-Kreis, Darmstadt, Wiesbaden, Rheingau-Taunus-Kreis, Bergstraße, Darmstadt-Dieburg, Frankfurt am Main, Offenbach, Main-Taunus-Kreis, Odenwaldkreis, Offenbach am Main, Hochtaunuskreis, Groß-Gerau et Wetteraukreis. Hesse est un Bundesland en Allemagne.</t>
+          <t>Le Land de Hesse se situe en Allemagne et comprend les arrondissements et villes-arrondissements suivants : Limburg-Weilburg, Vogelsbergkreis, Lahn-Dill-Kreis, Marburg-Biedenkopf, Gießen, Hersfeld-Rotenburg, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis, Kassel, Schwalm-Eder-Kreis, Main-Kinzig-Kreis, Darmstadt, Wiesbaden, Rheingau-Taunus-Kreis, Bergstraße, Darmstadt-Dieburg, Frankfurt am Main, Offenbach, Main-Taunus-Kreis, Odenwaldkreis, Offenbach am Main, Hochtaunuskreis, Groß-Gerau et Wetteraukreis.</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>5.567</v>
+        <v>4.987</v>
       </c>
       <c r="G94" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.82</v>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Tous les districts listés dans l’EXPECTED sont présents dans l’ACTUAL (au moins une fois), sauf Francfort-sur-le-Main qui est mentionné comme « Frankfurt am Main », et Offenbach-sur-le-Main est mentionné comme « Offenbach am Main ». Le contenu couvre donc l’information attendue avec un léger écart de formulation. L’ACTUAL inclut aussi des informations supplémentaires correctes (« Hesse est un Bundesland en Allemagne »).</t>
+          <t>L’ACTUAL liste presque tous les arrondissements attendus, mais il manque Francfort-sur-le-Main, ainsi que Odenwaldkreis/Offenbach-sur-le-Main en version attendue (présents sous d’autres libellés) et il y a des doublons (Kassel).</t>
         </is>
       </c>
       <c r="J94" t="n">
-        <v>0.6876</v>
+        <v>0.7245</v>
       </c>
       <c r="K94" t="n">
-        <v>0.6832</v>
+        <v>0.7236</v>
       </c>
       <c r="L94" t="n">
-        <v>0.6859</v>
+        <v>0.7245</v>
       </c>
     </row>
     <row r="95">
@@ -5343,11 +5338,11 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>L’arrondissement de Steinburg comprend les communes suivantes : Itzehoe-Land, Schenefeld, Wilstermarsch, Itzehoe, Horst-Herzhorn, Krempermarsch, Breitenburg, Glückstadt, Wilster et Kellinghusen. Steinburg est un arrondissement situé dans le land de Schleswig-Holstein, en Allemagne.</t>
+          <t>L’arrondissement de Steinburg comprend les communes administratives d’Itzehoe-Land, Schenefeld, Wilstermarsch, Itzehoe, Horst-Herzhorn, Krempermarsch, Breitenburg, Glückstadt, Wilster et Kellinghusen. Steinburg est un district, situé dans le Land du Schleswig-Holstein, en Allemagne.</t>
         </is>
       </c>
       <c r="F95" t="n">
-        <v>7.76</v>
+        <v>4.77</v>
       </c>
       <c r="G95" t="n">
         <v>1</v>
@@ -5359,17 +5354,17 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Les communes listées dans l’ACTUAL correspondent exactement à celles de l’EXPECTED (Wilster, Krempermarsch, Itzehoe-Land, Horst-Herzhorn, Breitenburg, Schenefeld, Wilstermarsch, Glückstadt, Kellinghusen, Itzehoe). L’ACTUAL ajoute seulement une phrase contextuelle.</t>
+          <t>Les 10 communes listées dans l’attendu (Wilster, Krempermarsch, Itzehoe-Land, Horst-Herzhorn, Breitenburg, Schenefeld, Wilstermarsch, Glückstadt, Kellinghusen, Itzehoe) sont toutes présentes dans la réponse réelle, sans omission. L’ajout “Steinburg est un district…” est correct et n’affecte pas le critère.</t>
         </is>
       </c>
       <c r="J95" t="n">
-        <v>0.6024</v>
+        <v>0.6017</v>
       </c>
       <c r="K95" t="n">
-        <v>0.7431</v>
+        <v>0.7833</v>
       </c>
       <c r="L95" t="n">
-        <v>0.6712</v>
+        <v>0.6896</v>
       </c>
     </row>
     <row r="96">
@@ -5395,11 +5390,11 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>L’arrondissement de Paderborn comprend 10 villes : Altenbeken, Hövelhof, Borchen, Delbrück, Paderborn, Büren, Bad Wünnenberg, Lichtenau, Salzkotten et Bad Lippspringe. Il s’agit d’un district situé dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne, qui est un État souverain.</t>
+          <t>L’arrondissement de Paderborn comprend 10 villes : Altenbeken, Hövelhof, Borchen, Delbrück, Paderborn, Büren, Bad Wünnenberg, Lichtenau, Salzkotten et Bad Lippspringe. Cet arrondissement appartient au district administratif de Detmold, dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne.</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>5.27</v>
+        <v>4.561</v>
       </c>
       <c r="G96" t="n">
         <v>1</v>
@@ -5411,17 +5406,17 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Les 10 villes listées dans l’ACTUAL correspondent exactement à celles attendues (mêmes noms, même nombre). L’information supplémentaire sur le Land est correcte et n’affecte pas la comparaison.</t>
+          <t>Les 10 villes listées dans l’ACTUAL correspondent exactement à celles de l’EXPECTED, avec des informations supplémentaires correctes sur le district administratif.</t>
         </is>
       </c>
       <c r="J96" t="n">
-        <v>0.3887</v>
+        <v>0.4422</v>
       </c>
       <c r="K96" t="n">
-        <v>0.7456</v>
+        <v>0.755</v>
       </c>
       <c r="L96" t="n">
-        <v>0.5538999999999999</v>
+        <v>0.5887</v>
       </c>
     </row>
     <row r="97">
@@ -5447,11 +5442,11 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Oui. Dülmen est une ville située dans l’arrondissement de Coesfeld, et l’arrondissement de Coesfeld se trouve en Allemagne.</t>
+          <t>Oui, Dülmen se trouve dans le Kreis de Coesfeld, en Allemagne. La hiérarchie indiquée est : ville Dülmen, Kreis Coesfeld, puis Allemagne comme Bundesstaat.</t>
         </is>
       </c>
       <c r="F97" t="n">
-        <v>5.671</v>
+        <v>3.986</v>
       </c>
       <c r="G97" t="n">
         <v>1</v>
@@ -5463,17 +5458,17 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>L’ACTUAL confirme que Dülmen est une ville située dans l’arrondissement (Landkreis) de Coesfeld, comme dans l’EXPECTED. La mention supplémentaire de l’Allemagne est correcte et n’affecte pas la réponse.</t>
+          <t>L’affirmation attendue est présente : Dülmen se trouve bien dans le Kreis (arrondissement) de Coesfeld. L’ACTUAL fournit en plus la hiérarchie et le pays, sans contredire l’information attendue.</t>
         </is>
       </c>
       <c r="J97" t="n">
-        <v>0.5237000000000001</v>
+        <v>0.3329</v>
       </c>
       <c r="K97" t="n">
-        <v>0.6372</v>
+        <v>0.536</v>
       </c>
       <c r="L97" t="n">
-        <v>0.5797</v>
+        <v>0.4305</v>
       </c>
     </row>
     <row r="98">
@@ -5499,11 +5494,11 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Non, aucune géométrie n’a été trouvée pour l’arrondissement de Coesfeld. Il n’y a donc aucune information disponible indiquant sa présence dans une région administrative, un Land fédéral ou en Allemagne.</t>
+          <t>Non, rien n’a été trouvé dans les données fournies. Il n’y a donc aucune information permettant d’affirmer que l’arrondissement de Coesfeld se trouve dans la région administrative de Münster.</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>5.046</v>
+        <v>4.104</v>
       </c>
       <c r="G98" t="n">
         <v>0</v>
@@ -5515,17 +5510,17 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>L’actual ne confirme pas que l’arrondissement de Coesfeld est dans la circonscription administrative de Münster ; au contraire, il indique qu’aucune information géographique n’a été trouvée.</t>
+          <t>L’ACTUAL répond « Non » et ne fournit aucune information confirmant que l’arrondissement de Coesfeld est situé dans la circonscription administrative de Münster, contrairement à l’attendu.</t>
         </is>
       </c>
       <c r="J98" t="n">
-        <v>0.0924</v>
+        <v>0.1923</v>
       </c>
       <c r="K98" t="n">
-        <v>0.4569</v>
+        <v>0.6512</v>
       </c>
       <c r="L98" t="n">
-        <v>0.2591</v>
+        <v>0.3981</v>
       </c>
     </row>
     <row r="99">
@@ -5555,7 +5550,7 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>7.014</v>
+        <v>4.129</v>
       </c>
       <c r="G99" t="n">
         <v>0</v>
@@ -5567,7 +5562,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>L’ACTUAL ne répond pas à la question et indique qu’aucune géométrie n’a été trouvée, ce qui ne correspond pas à l’attendu (Haute-Franconie fait partie de la Bavière).</t>
+          <t>L’ACTUAL n’apporte pas l’information demandée (il indique seulement qu’aucune géométrie n’a été trouvée) et contredit l’affirmation attendue.</t>
         </is>
       </c>
       <c r="J99" t="n">
@@ -5603,33 +5598,33 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Non, rien n’a été trouvé dans les données fournies : aucune géométrie n’est disponible pour l’arrondissement de Steinfurt, donc il n’est pas possible d’indiquer qu’il se trouve dans le Land de Rhénanie-du-Nord-Westphalie à partir de ce résultat.</t>
+          <t>Oui. L’arrondissement de Steinfurt se trouve dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne.</t>
         </is>
       </c>
       <c r="F100" t="n">
-        <v>5.273</v>
+        <v>4.246</v>
       </c>
       <c r="G100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>L’ACTUAL répond que l’information n’est pas disponible et n’affirme pas que l’arrondissement de Steinfurt se trouve dans le Land de Rhénanie-du-Nord-Westphalie, contrairement à l’EXPECTED.</t>
+          <t>L’ACTUAL confirme clairement que l’arrondissement de Steinfurt est situé dans le Land de Rhénanie-du-Nord-Westphalie; la mention supplémentaire que c’est en Allemagne ne contredit rien.</t>
         </is>
       </c>
       <c r="J100" t="n">
-        <v>0.1731</v>
+        <v>0.7158</v>
       </c>
       <c r="K100" t="n">
-        <v>0.6355</v>
+        <v>0.7816</v>
       </c>
       <c r="L100" t="n">
-        <v>0.3801</v>
+        <v>0.7486</v>
       </c>
     </row>
     <row r="101">
@@ -5655,33 +5650,33 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Non. Le résultat indique seulement Bocholt et un seul appariement avec Bocholt, sans montrer qu’elle se trouve dans l’arrondissement de Cloppenburg. Aucune autre hiérarchie n’est fournie, donc on ne peut pas confirmer une appartenance à un district, à un district administratif, à un Land fédéral ou à l’Allemagne à partir de ce résultat seul.</t>
+          <t>Non, aucune géométrie n’a été trouvée pour cette recherche.</t>
         </is>
       </c>
       <c r="F101" t="n">
-        <v>5.612</v>
+        <v>4.052</v>
       </c>
       <c r="G101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>L’ACTUAL répond également que Bocholt ne peut pas être confirmé comme se trouvant dans l’arrondissement de Cloppenburg et ne fournit pas d’élément indiquant qu’elle y appartient ; cela correspond à l’attendu « Non ».</t>
+          <t>La réponse attendue indique que Bocholt n'est pas dans l'arrondissement de Cloppenburg, mais la réponse réelle ne fournit aucune information pertinente et signale seulement un problème de géométrie.</t>
         </is>
       </c>
       <c r="J101" t="n">
-        <v>0.0766</v>
+        <v>0.1617</v>
       </c>
       <c r="K101" t="n">
-        <v>0.5678</v>
+        <v>0.1315</v>
       </c>
       <c r="L101" t="n">
-        <v>0.2938</v>
+        <v>0.1478</v>
       </c>
     </row>
     <row r="102">
@@ -5707,11 +5702,11 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Oui, les arrondissements de Coesfeld et de Borken sont limitrophes. Coesfeld est un district, situé dans un district administratif, dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne. Borken est également un district, situé dans un district administratif, dans le même Land de Rhénanie-du-Nord-Westphalie, en Allemagne.</t>
+          <t>Oui, les arrondissements de Coesfeld et de Borken sont limitrophes. Coesfeld est un district situé dans le district administratif de Münster, dans le Bundesland Nordrhein-Westfalen, en Allemagne. Borken est un district situé dans le district administratif de Münster, dans le Bundesland Nordrhein-Westfalen, en Allemagne.</t>
         </is>
       </c>
       <c r="F102" t="n">
-        <v>5.44</v>
+        <v>4.605</v>
       </c>
       <c r="G102" t="n">
         <v>1</v>
@@ -5723,17 +5718,17 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>L’ACTUAL confirme bien que les arrondissements de Coesfeld et de Borken sont limitrophes; les informations supplémentaires sont correctes et ne contredisent pas l’attendu.</t>
+          <t>L’ACTUAL confirme que les arrondissements de Coesfeld et de Borken sont limitrophes, comme dans l’EXPECTED. Les détails supplémentaires sur les districts administratifs et le Land sont corrects et n’empêchent pas la correspondance.</t>
         </is>
       </c>
       <c r="J102" t="n">
-        <v>0.0668</v>
+        <v>0.2047</v>
       </c>
       <c r="K102" t="n">
-        <v>0.6084000000000001</v>
+        <v>0.5983000000000001</v>
       </c>
       <c r="L102" t="n">
-        <v>0.303</v>
+        <v>0.3842</v>
       </c>
     </row>
     <row r="103">
@@ -5759,14 +5754,14 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Bonjour. Ce chatbot répond uniquement aux questions sur la géographie de l’Allemagne. Veuillez réessayer avec une autre question.</t>
+          <t>Non. D’après l’information fournie, Senden a été trouvée comme ville, et aucune géométrie cible n’a été trouvée pour Münster. La ville de Senden appartient à aucun niveau administratif supplémentaire indiqué ici au-delà de la ville, puis l’ensemble se termine par l’Allemagne comme État.</t>
         </is>
       </c>
       <c r="F103" t="n">
-        <v>4.918</v>
+        <v>5.95</v>
       </c>
       <c r="G103" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -5775,17 +5770,17 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>La réponse réelle ne répond pas à la question sur la séparation géographique entre Senden et Münster.</t>
+          <t>L’ACTUAL répond par 'Non', mais ne confirme pas que Senden et Münster sont voisins; il mentionne surtout l’absence de géométrie pour Münster.</t>
         </is>
       </c>
       <c r="J103" t="n">
-        <v>-0.0939</v>
+        <v>-0.1079</v>
       </c>
       <c r="K103" t="n">
-        <v>0.075</v>
+        <v>0.3738</v>
       </c>
       <c r="L103" t="n">
-        <v>-0.0121</v>
+        <v>0.103</v>
       </c>
     </row>
     <row r="104">
@@ -5811,11 +5806,11 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Non, aucune géométrie n’a été trouvée dans les informations fournies. Aucun lieu n’est indiqué comme appartenant à une hiérarchie allant jusqu’au Land de Basse-Saxe, au Land de Rhénanie-du-Nord-Westphalie, ni à l’Allemagne.</t>
+          <t>Non, rien n’indique une géométrie trouvée. Le résultat est vide, donc aucun rattachement hiérarchique ne peut être décrit, et il n’y a pas d’information permettant de dire que la Basse-Saxe est limitrophe de la Rhénanie-du-Nord-Westphalie.</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>5.72</v>
+        <v>4.596</v>
       </c>
       <c r="G104" t="n">
         <v>0</v>
@@ -5827,17 +5822,17 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>L’ACTUAL répond que ce n’est pas le cas (ou qu’aucune information pertinente n’est disponible), alors que l’EXPECTED affirme que la Basse-Saxe est limitrophe de la Rhénanie-du-Nord-Westphalie.</t>
+          <t>L’ACTUAL répond “Non” et ne fournit aucune correspondance avec l’assertion attendue “Oui”.</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>0.1862</v>
+        <v>0.1455</v>
       </c>
       <c r="K104" t="n">
-        <v>0.6281</v>
+        <v>0.6146</v>
       </c>
       <c r="L104" t="n">
-        <v>0.3852</v>
+        <v>0.3548</v>
       </c>
     </row>
     <row r="105">
@@ -5863,14 +5858,14 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Oui. Berlin est reliée à Schöneiche bei Berlin et à Neuenhagen bei Berlin. Ces localités sont des villes, situées en Allemagne, ce qui indique que Berlin n’est pas entièrement entourée par le Brandebourg d’après le résultat fourni.</t>
+          <t>Oui. Berlin est reliée à Schöneiche bei Berlin et à Neuenhagen bei Berlin, qui sont des villes situées en Allemagne.</t>
         </is>
       </c>
       <c r="F105" t="n">
-        <v>9.042</v>
+        <v>4.816</v>
       </c>
       <c r="G105" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
@@ -5879,17 +5874,17 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>The expected answer states that Berlin is entirely surrounded by Brandenburg, but the actual answer claims that Berlin is not entirely surrounded (contradicting the expected information).</t>
+          <t>L’ACTUEL n’indique pas clairement que Berlin est entièrement entourée par le Brandebourg; il mentionne seulement des localités reliées à Berlin.</t>
         </is>
       </c>
       <c r="J105" t="n">
-        <v>0.1965</v>
+        <v>0.2206</v>
       </c>
       <c r="K105" t="n">
-        <v>0.6806</v>
+        <v>0.4205</v>
       </c>
       <c r="L105" t="n">
-        <v>0.4123</v>
+        <v>0.3167</v>
       </c>
     </row>
     <row r="106">
@@ -5915,11 +5910,11 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Oui, Münster se trouve au nord de Dortmund. Dortmund est en Allemagne, et Münster est également en Allemagne.</t>
+          <t>Oui, Münster se trouve au nord de Dortmund. Les deux villes se situent en Allemagne, et l’une est au nord de l’autre.</t>
         </is>
       </c>
       <c r="F106" t="n">
-        <v>8.898999999999999</v>
+        <v>5.049</v>
       </c>
       <c r="G106" t="n">
         <v>1</v>
@@ -5931,17 +5926,17 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>L’information attendue est présente : Münster se trouve au nord de Dortmund. L’ACTUEL ajoute seulement des précisions correctes sur le pays.</t>
+          <t>L’ACTUEL confirme bien que Münster se trouve au nord de Dortmund. L’ajout d’informations générales ne contredit pas l’EXPECTED.</t>
         </is>
       </c>
       <c r="J106" t="n">
-        <v>0.5633</v>
+        <v>0.3643</v>
       </c>
       <c r="K106" t="n">
-        <v>0.8458</v>
+        <v>0.8687</v>
       </c>
       <c r="L106" t="n">
-        <v>0.6968</v>
+        <v>0.5899</v>
       </c>
     </row>
     <row r="107">
@@ -5967,11 +5962,11 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Greven se trouve juste au nord de Münster. Greven est une ville, située dans le Bundesland Nordrhein-Westfalen en Allemagne.</t>
+          <t>Greven se trouve juste au nord de Münster. Greven est une ville dans le district, le district administratif, le Land de l’État de l’Allemagne.</t>
         </is>
       </c>
       <c r="F107" t="n">
-        <v>6.809</v>
+        <v>4.749</v>
       </c>
       <c r="G107" t="n">
         <v>1</v>
@@ -5983,17 +5978,17 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>L’ACTUAL indique correctement que Greven se trouve juste au nord de Münster. La mention supplémentaire du Bundesland est exacte et n’affecte pas la réponse.</t>
+          <t>L’ACTUAL indique clairement que Greven se trouve juste au nord de Münster, ce qui correspond à l’EXPECTED. L’information supplémentaire sur le district est en plus et ne contredit pas.</t>
         </is>
       </c>
       <c r="J107" t="n">
-        <v>0.3443</v>
+        <v>0.1482</v>
       </c>
       <c r="K107" t="n">
-        <v>0.584</v>
+        <v>0.5668</v>
       </c>
       <c r="L107" t="n">
-        <v>0.4584</v>
+        <v>0.3375</v>
       </c>
     </row>
     <row r="108">
@@ -6019,11 +6014,11 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Oui. Leipzig se trouve au nord-est d’Erfurt, en Allemagne.</t>
+          <t>Oui, Leipzig se trouve au nord-est d’Erfurt. Les deux villes sont situées en Allemagne.</t>
         </is>
       </c>
       <c r="F108" t="n">
-        <v>15.959</v>
+        <v>5.559</v>
       </c>
       <c r="G108" t="n">
         <v>1</v>
@@ -6035,17 +6030,17 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>L'ACTUAL confirme que Leipzig est située au nord-est d’Erfurt, ce qui implique qu’elle est à l’est. Contenu attendu entièrement inclus.</t>
+          <t>L’ACTUAL indique correctement que Leipzig est au nord-est d’Erfurt (ce qui répond à la question). La mention que les deux villes sont en Allemagne est en plus et correcte.</t>
         </is>
       </c>
       <c r="J108" t="n">
-        <v>0.6254999999999999</v>
+        <v>0.6163</v>
       </c>
       <c r="K108" t="n">
-        <v>0.7351</v>
+        <v>0.8316</v>
       </c>
       <c r="L108" t="n">
-        <v>0.6796</v>
+        <v>0.7197</v>
       </c>
     </row>
     <row r="109">
@@ -6071,11 +6066,11 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>La distance entre Cologne et Bonn est de 6,63 km. Cologne est une ville en Allemagne. Bonn est une ville en Allemagne.</t>
+          <t>Köln est une ville située dans le district administratif de Cologne, dans le district de Cologne, dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne. Bonn est une ville située dans le district administratif de Cologne, dans le district de Bonn, dans le Land de Rhénanie-du-Nord-Westphalie, en Allemagne. La distance entre Cologne et Bonn est de 6,63 km.</t>
         </is>
       </c>
       <c r="F109" t="n">
-        <v>26.363</v>
+        <v>10.779</v>
       </c>
       <c r="G109" t="n">
         <v>1</v>
@@ -6087,17 +6082,17 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>L’ACTUEL fournit exactement la même distance (6,63 km) entre Cologne et Bonn. Les informations supplémentaires sur le pays des villes sont correctes et ne manquent pas à l’élément attendu.</t>
+          <t>L’actuel mentionne explicitement que la distance entre Cologne et Bonn est de 6,63 km, ce qui correspond à l’attendu.</t>
         </is>
       </c>
       <c r="J109" t="n">
-        <v>0.4208</v>
+        <v>0.023</v>
       </c>
       <c r="K109" t="n">
-        <v>0.5738</v>
+        <v>0.6568000000000001</v>
       </c>
       <c r="L109" t="n">
-        <v>0.4954</v>
+        <v>0.2922</v>
       </c>
     </row>
     <row r="110">
@@ -6123,11 +6118,11 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Aucune géométrie n’a été trouvée. Il n’y a donc pas d’information disponible sur la distance entre Hanovre et Brunswick.</t>
+          <t>Aucune géométrie n’a été trouvée pour cette requête.</t>
         </is>
       </c>
       <c r="F110" t="n">
-        <v>5.178</v>
+        <v>4.024</v>
       </c>
       <c r="G110" t="n">
         <v>0</v>
@@ -6139,17 +6134,17 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>La réponse réelle ne fournit aucune distance et indique qu’aucune donnée n’est disponible, donc l’information attendue (34,92 km) manque.</t>
+          <t>La réponse attendue indique une distance de 34,92 km, mais la réponse actuelle ne fournit aucune information de distance.</t>
         </is>
       </c>
       <c r="J110" t="n">
-        <v>0.0573</v>
+        <v>-0.0461</v>
       </c>
       <c r="K110" t="n">
-        <v>0.2866</v>
+        <v>-0.0803</v>
       </c>
       <c r="L110" t="n">
-        <v>0.1663</v>
+        <v>-0.0618</v>
       </c>
     </row>
     <row r="111">
@@ -6175,11 +6170,11 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>La Hesse et la Thuringe se trouvent à une distance de 0,0 km l’une de l’autre. La Hesse est un Bundesland en Allemagne, et la Thuringe est aussi un Bundesland en Allemagne. L’Allemagne est un État.</t>
+          <t>La Hesse et la Thuringe se trouvent à une distance de 0,0 km l’une de l’autre. La Hesse est un Bundesland en Allemagne, et la Thuringe est aussi un Bundesland en Allemagne. Les deux appartiennent au Bundesstaat Allemagne.</t>
         </is>
       </c>
       <c r="F111" t="n">
-        <v>28.853</v>
+        <v>11.641</v>
       </c>
       <c r="G111" t="n">
         <v>1</v>
@@ -6191,17 +6186,17 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>L’ACTUAL indique que la distance entre la Hesse et la Thuringe est de 0,0 km, ce qui correspond à l’EXPECTED. Les informations supplémentaires sont correctes et n’affectent pas la réponse.</t>
+          <t>L’ACTUAL indique bien que la distance entre la Hesse et la Thuringe est de 0,0 km, comme dans l’EXPECTED. Les informations supplémentaires sont pertinentes.</t>
         </is>
       </c>
       <c r="J111" t="n">
-        <v>0.4368</v>
+        <v>0.3978</v>
       </c>
       <c r="K111" t="n">
-        <v>0.5968</v>
+        <v>0.5908</v>
       </c>
       <c r="L111" t="n">
-        <v>0.5147</v>
+        <v>0.4909</v>
       </c>
     </row>
     <row r="112">
@@ -6227,11 +6222,11 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Les trois districts les plus proches de Miesbach sont München, Bad Tölz-Wolfratshausen et Rosenheim. Miesbach est un district dans le district administratif de Haute-Bavière, dans le Land de Bavière, en Allemagne.</t>
+          <t>Les trois districts les plus proches de Miesbach sont München, Bad Tölz-Wolfratshausen et Rosenheim. Miesbach est un district en Bavière, en Allemagne, et ces trois districts sont également des districts situés en Bavière, en Allemagne.</t>
         </is>
       </c>
       <c r="F112" t="n">
-        <v>5.78</v>
+        <v>3.95</v>
       </c>
       <c r="G112" t="n">
         <v>1</v>
@@ -6243,17 +6238,17 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Les trois districts les plus proches mentionnés correspondent : Bad Tölz-Wolfratshausen, Munich (écrit München) et Rosenheim. L’ACTUAL ajoute des informations contextuelles supplémentaires sans contredire la réponse attendue.</t>
+          <t>Les trois districts les plus proches cités sont les mêmes que dans l'attendu (Bad Tölz-Wolfratshausen, Munich/München, Rosenheim). L'ajout de précisions sur la localisation en Bavière est correct.</t>
         </is>
       </c>
       <c r="J112" t="n">
-        <v>0.4915</v>
+        <v>0.5044999999999999</v>
       </c>
       <c r="K112" t="n">
-        <v>0.7723</v>
+        <v>0.7899</v>
       </c>
       <c r="L112" t="n">
-        <v>0.6241</v>
+        <v>0.6392</v>
       </c>
     </row>
     <row r="113">
@@ -6279,11 +6274,11 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Le district de Warendorf a pour districts limitrophes Gütersloh, Steinfurt, Soest, Coesfeld, Osnabrück, Münster et Hamm. Warendorf est un district en Allemagne.</t>
+          <t>Les districts limitrophes du district de Warendorf sont Gütersloh, Steinfurt, Soest, Coesfeld, Osnabrück, Münster et Hamm. Warendorf est un district en Allemagne.</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>5.913</v>
+        <v>3.881</v>
       </c>
       <c r="G113" t="n">
         <v>1</v>
@@ -6295,17 +6290,17 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Les districts limitrophes mentionnés dans l’ACTUAL (Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld, Soest) correspondent exactement aux districts attendus.</t>
+          <t>Les districts limitrophes mentionnés sont exactement les mêmes que dans l'attendu (Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld, Soest). L'info supplémentaire « Warendorf est un district en Allemagne » est correcte.</t>
         </is>
       </c>
       <c r="J113" t="n">
-        <v>0.6238</v>
+        <v>0.624</v>
       </c>
       <c r="K113" t="n">
-        <v>0.7024</v>
+        <v>0.6978</v>
       </c>
       <c r="L113" t="n">
-        <v>0.6629</v>
+        <v>0.6609</v>
       </c>
     </row>
     <row r="114">
@@ -6331,11 +6326,11 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Les communes administratives limitrophes de Leezen sont Bad Oldesloe-Land, Trave-Land, Boostedt-Rickling, Auenland Südholstein, Wahlstedt, Kisdorf, Bad Segeberg, Itzstedt et Buchholz (Forstgutsbez.). Leezen est une commune administrative en Allemagne.</t>
+          <t>Les communes administratives limitrophes de la commune administrative de Leezen sont Bad Oldesloe-Land, Trave-Land, Boostedt-Rickling, Auenland Südholstein, Wahlstedt, Kisdorf, Bad Segeberg, Itzstedt et Buchholz (Forstgutsbez.). Leezen est une commune administrative du district de Segeberg, dans le Land de Schleswig-Holstein, en Allemagne.</t>
         </is>
       </c>
       <c r="F114" t="n">
-        <v>5.283</v>
+        <v>3.979</v>
       </c>
       <c r="G114" t="n">
         <v>1</v>
@@ -6347,17 +6342,17 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>L’ACTUAL liste exactement les 9 communes limitrophes attendues (Auenland Südholstein, Kisdorf, Bad Oldesloe-Land, Trave-Land, Wahlstedt, Itzstedt, Bad Segeberg, Boostedt-Rickling, Buchholz (Forstgutsbez.)).</t>
+          <t>L’ACTUAL liste exactement toutes les communes limitrophes attendues (Auenland Südholstein, Kisdorf, Bad Oldesloe-Land, Trave-Land, Wahlstedt, Itzstedt, Bad Segeberg, Boostedt-Rickling, Buchholz (Forstgutsbez.)). L’ACTUAL ajoute seulement une phrase contextuelle sans manquer d’info attendue.</t>
         </is>
       </c>
       <c r="J114" t="n">
-        <v>0.6833</v>
+        <v>0.5406</v>
       </c>
       <c r="K114" t="n">
-        <v>0.7364000000000001</v>
+        <v>0.7089</v>
       </c>
       <c r="L114" t="n">
-        <v>0.71</v>
+        <v>0.6223</v>
       </c>
     </row>
     <row r="115">
@@ -6383,11 +6378,11 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Aucune géométrie n’a été trouvée ; il n’y a donc aucune information disponible sur les districts administratifs entourant la Moyenne-Franconie.</t>
+          <t>Aucune géométrie n’a été trouvée pour cette question.</t>
         </is>
       </c>
       <c r="F115" t="n">
-        <v>4.535</v>
+        <v>4.199</v>
       </c>
       <c r="G115" t="n">
         <v>0</v>
@@ -6399,17 +6394,17 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>La réponse attendue mentionne l’entourage (la Moyenne-Franconie est entourée par la Bavière), mais la réponse réelle indique qu’aucune information n’est disponible.</t>
+          <t>La réponse attendue doit indiquer que la Moyenne-Franconie est entourée par la Bavière, mais la réponse réelle ne fournit aucune information.</t>
         </is>
       </c>
       <c r="J115" t="n">
-        <v>0.1471</v>
+        <v>0.0406</v>
       </c>
       <c r="K115" t="n">
-        <v>0.3851</v>
+        <v>-0.0154</v>
       </c>
       <c r="L115" t="n">
-        <v>0.2601</v>
+        <v>0.0136</v>
       </c>
     </row>
     <row r="116">
@@ -6435,11 +6430,11 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Les Länder situés au nord de la Thuringe sont le Mecklembourg-Poméranie-Occidentale, la Saxe-Anhalt, le Schleswig-Holstein et Hambourg. La Thuringe est un Land de l’Allemagne, un État fédéral d’Allemagne.</t>
+          <t>Au nord de la Thuringe, on trouve le Land de la Thuringe elle-même, ainsi que le Schleswig-Holstein, la Saxe-Anhalt, le Mecklembourg-Poméranie-Occidentale et Hambourg, tous situés en Allemagne.</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>68.774</v>
+        <v>30.525</v>
       </c>
       <c r="G116" t="n">
         <v>1</v>
@@ -6451,17 +6446,17 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Les quatre Länder cités correspondent exactement à l’attendu : Hambourg, Schleswig-Holstein, Mecklembourg-Poméranie occidentale et Saxe-Anhalt. La mention supplémentaire sur la Thuringe est exacte mais non nécessaire.</t>
+          <t>L’ACTUAL mentionne les mêmes Länder attendus au nord de la Thuringe : Hambourg, le Schleswig-Holstein, le Mecklembourg-Poméranie occidentale et la Saxe-Anhalt (avec une précision lexicale différente). Le fait qu’elle ajoute la Thuringe n’enlève rien aux éléments attendus, et ne contredit pas la liste demandée.</t>
         </is>
       </c>
       <c r="J116" t="n">
-        <v>0.5973000000000001</v>
+        <v>0.5792</v>
       </c>
       <c r="K116" t="n">
-        <v>0.7892</v>
+        <v>0.7577</v>
       </c>
       <c r="L116" t="n">
-        <v>0.6899</v>
+        <v>0.6657</v>
       </c>
     </row>
     <row r="117">
@@ -6487,11 +6482,11 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Les districts situés à l’ouest du district de Münster sont Kleve et Borken. Münster est un district situé dans le Regierungsbezirk Münster, dans le Bundesland Nordrhein-Westfalen, en Allemagne.</t>
+          <t>Les districts situés à l’ouest de Münster sont Kleve et Borken. Münster est un district situé dans le Regierungsbezirk de Münster, dans le Bundesland de Rhénanie-du-Nord-Westphalie, en Allemagne. Kleve et Borken sont également des districts situés dans le Regierungsbezirk de Münster, dans le Bundesland de Rhénanie-du-Nord-Westphalie, en Allemagne.</t>
         </is>
       </c>
       <c r="F117" t="n">
-        <v>75.13800000000001</v>
+        <v>32.456</v>
       </c>
       <c r="G117" t="n">
         <v>1</v>
@@ -6503,17 +6498,17 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>L’ACTUAL mentionne correctement que Kleve et Borken sont à l’ouest de Münster. L’information supplémentaire sur la localisation de Münster est pertinente.</t>
+          <t>L’ACTUAL mentionne bien que les districts à l’ouest de Münster sont Clèves (Kleve) et Borken, ce qui correspond à l’EXPECTED. Le reste est une information supplémentaire correcte.</t>
         </is>
       </c>
       <c r="J117" t="n">
-        <v>0.2479</v>
+        <v>0.0211</v>
       </c>
       <c r="K117" t="n">
-        <v>0.4321</v>
+        <v>0.381</v>
       </c>
       <c r="L117" t="n">
-        <v>0.3369</v>
+        <v>0.1854</v>
       </c>
     </row>
     <row r="118">
@@ -6539,33 +6534,33 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Au nord de la communauté administrative de Kiel, on trouve les communautés administratives de Geltinger Bucht, Dänischenhagen, Altenholz et Kappeln. Kiel et ces communautés administratives se situent dans un district, dans un district administratif, dans le land du Schleswig-Holstein, en Allemagne.</t>
+          <t>Les communautés administratives situées au nord de Kiel sont Geltinger Bucht, Kiel, Altenholz, Dänischenhagen et Kappeln. Kiel est une communauté administrative située dans le district, puis dans le district administratif, dans le Land de Schleswig-Holstein, en Allemagne.</t>
         </is>
       </c>
       <c r="F118" t="n">
-        <v>68.554</v>
+        <v>31.136</v>
       </c>
       <c r="G118" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>L’ACTUAL liste exactement les mêmes communes au nord (Altenholz, Dänischenhagen, Kappeln, Geltinger Bucht). Le reste des informations supplémentaires est correct et ne manque pas à l’attendu.</t>
+          <t>L’ACTUAL liste bien Altenholz, Dänischenhagen, Kappeln et Geltinger Bucht, mais ajoute aussi Kiel (alors que l’EXPECTED ne l’inclut pas puisqu’il s’agit de la référence).</t>
         </is>
       </c>
       <c r="J118" t="n">
-        <v>0.3574</v>
+        <v>0.424</v>
       </c>
       <c r="K118" t="n">
-        <v>0.6409</v>
+        <v>0.6874</v>
       </c>
       <c r="L118" t="n">
-        <v>0.4909</v>
+        <v>0.5488</v>
       </c>
     </row>
     <row r="119">
@@ -6591,11 +6586,11 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Autour du district de Göttingen, les districts suivants sont indiqués comme situés dans un rayon de 10 km : Northeim, Kassel, Goslar, Nordhausen, Werra-Meißner-Kreis, Eichsfeld et Harz. Göttingen est un district en Allemagne.</t>
+          <t>Autour de Göttingen, les districts mentionnés sont Harz, Eichsfeld, Kassel, Werra-Meißner-Kreis, Kassel, Northeim, Nordhausen et Goslar. Göttingen est un district situé dans le Land de Basse-Saxe en Allemagne, et les districts indiqués se trouvent dans le même niveau hiérarchique de district en Allemagne.</t>
         </is>
       </c>
       <c r="F119" t="n">
-        <v>90.797</v>
+        <v>43.484</v>
       </c>
       <c r="G119" t="n">
         <v>1</v>
@@ -6607,17 +6602,17 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>L’ACTUAL liste exactement les mêmes districts que l’EXPECTED (Harz, Northeim, Goslar, Kassel, Eichsfeld, Werra‑Meißner‑Kreis, Nordhausen) ; l’information supplémentaire sur l’Allemagne est correcte.</t>
+          <t>L’ACTUAL liste exactement les mêmes districts que l’EXPECTED (Harz, Northeim, Goslar, Kassel, Eichsfeld, Werra‑Meißner‑Kreis, Nordhausen). La seule différence est une répétition de Kassel et des informations contextuelles supplémentaires, qui ne manquent pas à l’essentiel attendu.</t>
         </is>
       </c>
       <c r="J119" t="n">
-        <v>0.6169</v>
+        <v>0.3979</v>
       </c>
       <c r="K119" t="n">
-        <v>0.7705</v>
+        <v>0.5998</v>
       </c>
       <c r="L119" t="n">
-        <v>0.6917</v>
+        <v>0.495</v>
       </c>
     </row>
     <row r="120">
@@ -6643,11 +6638,11 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Autour d’Aix-la-Chapelle, les villes indiquées sont Würselen, Alsdorf, Roetgen, Herzogenrath, Eschweiler, Hürtgenwald, Stolberg (Rhld.) et Simmerath. Elles sont toutes situées en Allemagne.</t>
+          <t>Les villes situées dans un rayon de 5 km autour d’Aix-la-Chapelle sont Stolberg (Rhld.), Würselen, Alsdorf, Simmerath, Hürtgenwald, Eschweiler, Roetgen et Herzogenrath. Aachen est une ville en Allemagne.</t>
         </is>
       </c>
       <c r="F120" t="n">
-        <v>84.54300000000001</v>
+        <v>37.483</v>
       </c>
       <c r="G120" t="n">
         <v>1</v>
@@ -6659,17 +6654,17 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>L’ACTUAL liste exactement toutes les villes attendues dans le rayon de 5 km (Alsdorf, Simmerath, Würselen, Hürtgenwald, Roetgen, Herzogenrath, Eschweiler, Stolberg) ; seules des informations supplémentaires générales sont ajoutées.</t>
+          <t>Toutes les villes de la liste attendue (Alsdorf, Simmerath, Würselen, Hürtgenwald, Roetgen, Herzogenrath, Eschweiler, Stolberg) sont présentes dans la réponse réelle. L’info supplémentaire sur Aachen ne contredit rien.</t>
         </is>
       </c>
       <c r="J120" t="n">
-        <v>0.6536999999999999</v>
+        <v>0.6942</v>
       </c>
       <c r="K120" t="n">
-        <v>0.6723</v>
+        <v>0.738</v>
       </c>
       <c r="L120" t="n">
-        <v>0.6635</v>
+        <v>0.7163</v>
       </c>
     </row>
     <row r="121">
@@ -6695,34 +6690,33 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Les villes situées dans un rayon de moins de 2 km autour de Munich sont Krailling, Hebertshausen, Putzbrunn, Gräfelfing, Pullach i.Isartal, Bergkirchen, Ottobrunn, Haar, Gröbenzell, Vaterstetten, Karlsfeld, Planegg, Puchheim, Grünwalder Forst, Neubiberg, Oberschleißheim, Germering, Perlacher Forst, Dachau, Feldkirchen, Olching, Unterföhring, Unterhaching, Garching b.München, Ismaning, Neuried, Hohenbrunn, Forstenrieder Park, Aschheim, Grünwald et Grasbrunn.
-München est une ville située en Allemagne, et les lieux listés sont des villes ou des zones situées autour d’elle, en Allemagne.</t>
+          <t>Les villes situées dans un rayon de moins de 2 km autour de Munich sont Vaterstetten, Ottobrunn, Gräfelfing, Pullach i.Isartal, Hohenbrunn, Neuried, Hebertshausen, Gröbenzell, Haar, Neubiberg, Unterföhring, Ismaning, Olching, Forstenrieder Park, Karlsfeld, Aschheim, Dachau, Grünwald, Germering, Grünwalder Forst, Grasbrunn, Perlacher Forst, Oberschleißheim, Garching b.München, Feldkirchen, Bergkirchen, Putzbrunn, Krailling, Planegg, Puchheim et Unterhaching. Munich est une ville située dans le district de Munich, dans le district administratif de Haute-Bavière, dans le Bundesland de Bavière, en Allemagne.</t>
         </is>
       </c>
       <c r="F121" t="n">
-        <v>86.595</v>
+        <v>39.032</v>
       </c>
       <c r="G121" t="n">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>L’ACTUEL contient la majorité des villes attendues (25/24 environ) mais inclut aussi des villes non attendues (ex. Krailling, Hebertshausen, Ottobrunn, Vaterstetten, Hohenbrunn, Grasbrunn, Dachau) et ne liste pas explicitement Feldkirchen? (elle est présente) ; au final, l’écart principal est l’ajout d’éléments non attendus, et certains noms/mailles attendues semblent manquer ou être remplacés par des zones proches. La couverture exacte des 22 noms attendus n’est pas totale.</t>
+          <t>Tous les éléments attendus ne sont pas présents : il manque notamment Unterföhring n'est présent? (oui), mais il manque Feldkirchen? (présent), Pullach i.Isartal (présent), cependant il manque Puchheim? (présent), Gräfelfing (présent), Forstenrieder Park (présent), Perlacher Forst (présent), Gründwald? (présent via Grünwald), en revanche l'item "Haar" (présent) et "Neubiberg" (présent). La principale omission est la ville "Neubiberg" est présente; il manque tout de même "Haar"? présent. En réalité, seules deux villes de l'attendu semblent absentes : "Putzbrunn" est présent, "Bergkirchen" présent, "Germering" présent. Les absences notables sont "Grünwald" présent, "Unterhaching" présent, "Ismaning" présent, "Feldkirchen" présent. Il manque toutefois "Dachau" n'est pas dans l'attendu (ajout ok) mais il faut les manques : l'attendu contient "Neubiberg" (présent) et "Oberschleißheim" (présent). L'attendu contient "Vaterstetten" non. Au final, toutes les villes attendues semblent incluses ; si c'est le cas, score devrait être 1. Mais l'attendu inclut "Karlsfeld" (présent) et "Garching b.München" (présent). Conclusion : l'ensemble attendu est bien présent, avec des ajouts corrects, donc PASSED.</t>
         </is>
       </c>
       <c r="J121" t="n">
-        <v>0.5757</v>
+        <v>0.5463</v>
       </c>
       <c r="K121" t="n">
-        <v>0.7318</v>
+        <v>0.7319</v>
       </c>
       <c r="L121" t="n">
-        <v>0.6518</v>
+        <v>0.636</v>
       </c>
     </row>
     <row r="122">
@@ -6736,21 +6730,21 @@
       <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="n">
-        <v>16.401</v>
+        <v>9.733000000000001</v>
       </c>
       <c r="G122" t="n">
-        <v>0.7733</v>
+        <v>0.7318</v>
       </c>
       <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr"/>
       <c r="J122" t="n">
-        <v>0.4308</v>
+        <v>0.4043</v>
       </c>
       <c r="K122" t="n">
-        <v>0.5494</v>
+        <v>0.5327</v>
       </c>
       <c r="L122" t="n">
-        <v>0.4826</v>
+        <v>0.4605</v>
       </c>
     </row>
   </sheetData>

</xml_diff>